<commit_message>
Add CI workflow, documentation and dev dependencies
- GitHub Actions workflow (lint, format, type check, imports)
- Ruff and mypy configuration
- README and AGENTS.md documentation
- .env.example template for ZapSign credentials
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL7"/>
+  <dimension ref="A1:EL9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3503,47 +3503,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C7" t="n">
+        <v>84</v>
+      </c>
+      <c r="D7" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F7" t="n">
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
+        <v>22133</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L7" t="n">
+        <v>408</v>
       </c>
       <c r="M7" t="inlineStr">
         <is>
@@ -3555,25 +3541,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O7" t="n">
+        <v>408</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q7" t="inlineStr">
-        <is>
-          <t>1780628400</t>
-        </is>
-      </c>
-      <c r="R7" t="inlineStr">
-        <is>
-          <t>1780666934</t>
-        </is>
+      <c r="Q7" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R7" t="n">
+        <v>1780666934</v>
       </c>
       <c r="S7" t="inlineStr">
         <is>
@@ -3595,10 +3575,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W7" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W7" t="n">
+        <v>22133</v>
       </c>
       <c r="X7" t="inlineStr">
         <is>
@@ -3610,35 +3588,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z7" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z7" t="n">
+        <v>127857</v>
       </c>
       <c r="AA7" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB7" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC7" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB7" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC7" t="n">
+        <v>487</v>
       </c>
       <c r="AD7" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE7" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE7" t="n">
+        <v>121</v>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
@@ -3655,10 +3625,8 @@
       <c r="AJ7" t="inlineStr"/>
       <c r="AK7" t="inlineStr"/>
       <c r="AL7" t="inlineStr"/>
-      <c r="AM7" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM7" t="n">
+        <v>127857</v>
       </c>
       <c r="AN7" t="inlineStr">
         <is>
@@ -3690,10 +3658,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT7" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT7" t="n">
+        <v>3500</v>
       </c>
       <c r="AU7" t="inlineStr"/>
       <c r="AV7" t="inlineStr">
@@ -3821,10 +3787,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE7" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE7" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF7" t="inlineStr">
         <is>
@@ -3841,15 +3805,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI7" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ7" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI7" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ7" t="n">
+        <v>12344</v>
       </c>
       <c r="DK7" t="inlineStr">
         <is>
@@ -3861,10 +3821,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM7" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM7" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN7" t="inlineStr"/>
       <c r="DO7" t="inlineStr">
@@ -3882,15 +3840,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR7" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS7" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR7" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS7" t="n">
+        <v>3144</v>
       </c>
       <c r="DT7" t="inlineStr">
         <is>
@@ -3907,10 +3861,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW7" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW7" t="n">
+        <v>124</v>
       </c>
       <c r="DX7" t="inlineStr">
         <is>
@@ -3975,6 +3927,926 @@
         </is>
       </c>
       <c r="EL7" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>05/06/2026, 10:56:41</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>84</v>
+      </c>
+      <c r="D8" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L8" t="n">
+        <v>408</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O8" t="n">
+        <v>408</v>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q8" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R8" t="n">
+        <v>1780667320</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>10:48</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>05/06/2026 10:48</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W8" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z8" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB8" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC8" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE8" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr"/>
+      <c r="AI8" t="inlineStr"/>
+      <c r="AJ8" t="inlineStr"/>
+      <c r="AK8" t="inlineStr"/>
+      <c r="AL8" t="inlineStr"/>
+      <c r="AM8" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT8" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU8" t="inlineStr"/>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr"/>
+      <c r="BD8" t="inlineStr"/>
+      <c r="BE8" t="inlineStr"/>
+      <c r="BF8" t="inlineStr"/>
+      <c r="BG8" t="inlineStr"/>
+      <c r="BH8" t="inlineStr"/>
+      <c r="BI8" t="inlineStr"/>
+      <c r="BJ8" t="inlineStr"/>
+      <c r="BK8" t="inlineStr"/>
+      <c r="BL8" t="inlineStr"/>
+      <c r="BM8" t="inlineStr"/>
+      <c r="BN8" t="inlineStr"/>
+      <c r="BO8" t="inlineStr"/>
+      <c r="BP8" t="inlineStr"/>
+      <c r="BQ8" t="inlineStr"/>
+      <c r="BR8" t="inlineStr"/>
+      <c r="BS8" t="inlineStr"/>
+      <c r="BT8" t="inlineStr"/>
+      <c r="BU8" t="inlineStr"/>
+      <c r="BV8" t="inlineStr"/>
+      <c r="BW8" t="inlineStr"/>
+      <c r="BX8" t="inlineStr"/>
+      <c r="BY8" t="inlineStr"/>
+      <c r="BZ8" t="inlineStr"/>
+      <c r="CA8" t="inlineStr"/>
+      <c r="CB8" t="inlineStr"/>
+      <c r="CC8" t="inlineStr"/>
+      <c r="CD8" t="inlineStr"/>
+      <c r="CE8" t="inlineStr"/>
+      <c r="CF8" t="inlineStr"/>
+      <c r="CG8" t="inlineStr"/>
+      <c r="CH8" t="inlineStr"/>
+      <c r="CI8" t="inlineStr"/>
+      <c r="CJ8" t="inlineStr"/>
+      <c r="CK8" t="inlineStr"/>
+      <c r="CL8" t="inlineStr"/>
+      <c r="CM8" t="inlineStr"/>
+      <c r="CN8" t="inlineStr"/>
+      <c r="CO8" t="inlineStr"/>
+      <c r="CP8" t="inlineStr"/>
+      <c r="CQ8" t="inlineStr"/>
+      <c r="CR8" t="inlineStr"/>
+      <c r="CS8" t="inlineStr"/>
+      <c r="CT8" t="inlineStr"/>
+      <c r="CU8" t="inlineStr"/>
+      <c r="CV8" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW8" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX8" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY8" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ8" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA8" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB8" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC8" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD8" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE8" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF8" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG8" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH8" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI8" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ8" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK8" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL8" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM8" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN8" t="inlineStr"/>
+      <c r="DO8" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP8" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ8" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR8" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS8" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT8" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU8" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV8" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW8" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX8" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY8" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ8" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA8" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB8" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC8" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED8" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE8" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF8" t="inlineStr"/>
+      <c r="EG8" t="inlineStr"/>
+      <c r="EH8" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI8" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ8" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK8" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>05/06/2026, 10:58:51</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>1780628400</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>1780667450</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>10:50</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>05/06/2026 10:50</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr"/>
+      <c r="AI9" t="inlineStr"/>
+      <c r="AJ9" t="inlineStr"/>
+      <c r="AK9" t="inlineStr"/>
+      <c r="AL9" t="inlineStr"/>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr"/>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr"/>
+      <c r="BD9" t="inlineStr"/>
+      <c r="BE9" t="inlineStr"/>
+      <c r="BF9" t="inlineStr"/>
+      <c r="BG9" t="inlineStr"/>
+      <c r="BH9" t="inlineStr"/>
+      <c r="BI9" t="inlineStr"/>
+      <c r="BJ9" t="inlineStr"/>
+      <c r="BK9" t="inlineStr"/>
+      <c r="BL9" t="inlineStr"/>
+      <c r="BM9" t="inlineStr"/>
+      <c r="BN9" t="inlineStr"/>
+      <c r="BO9" t="inlineStr"/>
+      <c r="BP9" t="inlineStr"/>
+      <c r="BQ9" t="inlineStr"/>
+      <c r="BR9" t="inlineStr"/>
+      <c r="BS9" t="inlineStr"/>
+      <c r="BT9" t="inlineStr"/>
+      <c r="BU9" t="inlineStr"/>
+      <c r="BV9" t="inlineStr"/>
+      <c r="BW9" t="inlineStr"/>
+      <c r="BX9" t="inlineStr"/>
+      <c r="BY9" t="inlineStr"/>
+      <c r="BZ9" t="inlineStr"/>
+      <c r="CA9" t="inlineStr"/>
+      <c r="CB9" t="inlineStr"/>
+      <c r="CC9" t="inlineStr"/>
+      <c r="CD9" t="inlineStr"/>
+      <c r="CE9" t="inlineStr"/>
+      <c r="CF9" t="inlineStr"/>
+      <c r="CG9" t="inlineStr"/>
+      <c r="CH9" t="inlineStr"/>
+      <c r="CI9" t="inlineStr"/>
+      <c r="CJ9" t="inlineStr"/>
+      <c r="CK9" t="inlineStr"/>
+      <c r="CL9" t="inlineStr"/>
+      <c r="CM9" t="inlineStr"/>
+      <c r="CN9" t="inlineStr"/>
+      <c r="CO9" t="inlineStr"/>
+      <c r="CP9" t="inlineStr"/>
+      <c r="CQ9" t="inlineStr"/>
+      <c r="CR9" t="inlineStr"/>
+      <c r="CS9" t="inlineStr"/>
+      <c r="CT9" t="inlineStr"/>
+      <c r="CU9" t="inlineStr"/>
+      <c r="CV9" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW9" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX9" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY9" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ9" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA9" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB9" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC9" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD9" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE9" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF9" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG9" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH9" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI9" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ9" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK9" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL9" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM9" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN9" t="inlineStr"/>
+      <c r="DO9" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP9" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ9" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR9" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS9" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT9" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU9" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV9" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW9" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX9" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY9" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ9" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA9" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB9" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC9" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED9" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE9" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF9" t="inlineStr"/>
+      <c r="EG9" t="inlineStr"/>
+      <c r="EH9" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI9" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ9" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK9" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4209,13 +5081,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{974F33F7-5E24-44D5-91E3-C646EF4340AF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08CAB4CC-F01A-4A7D-9B08-31B78D4FE740}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{13C876D4-FB18-4A23-9087-8C0E0D8E7E2A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D565463-EA89-4DEE-A91D-49D4A0C39119}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{50CE03C6-A416-498C-B797-9A86597A19C1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1099D124-125E-45CF-9E63-66376AF57B53}"/>
 </file>
</xml_diff>

<commit_message>
Activate test mode in Triata workflow
Clicks the Modo Teste button after login, with JavaScript fallback
to call ModoTeste('I'). Increases browser slow_mo to 500ms.
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL9"/>
+  <dimension ref="A1:EL12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4375,47 +4375,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C9" t="n">
+        <v>84</v>
+      </c>
+      <c r="D9" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>22133</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L9" t="n">
+        <v>408</v>
       </c>
       <c r="M9" t="inlineStr">
         <is>
@@ -4427,25 +4413,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O9" t="n">
+        <v>408</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
-        <is>
-          <t>1780628400</t>
-        </is>
-      </c>
-      <c r="R9" t="inlineStr">
-        <is>
-          <t>1780667450</t>
-        </is>
+      <c r="Q9" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R9" t="n">
+        <v>1780667450</v>
       </c>
       <c r="S9" t="inlineStr">
         <is>
@@ -4467,10 +4447,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W9" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W9" t="n">
+        <v>22133</v>
       </c>
       <c r="X9" t="inlineStr">
         <is>
@@ -4482,35 +4460,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z9" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z9" t="n">
+        <v>127857</v>
       </c>
       <c r="AA9" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB9" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC9" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB9" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC9" t="n">
+        <v>487</v>
       </c>
       <c r="AD9" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE9" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE9" t="n">
+        <v>121</v>
       </c>
       <c r="AF9" t="inlineStr">
         <is>
@@ -4527,10 +4497,8 @@
       <c r="AJ9" t="inlineStr"/>
       <c r="AK9" t="inlineStr"/>
       <c r="AL9" t="inlineStr"/>
-      <c r="AM9" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM9" t="n">
+        <v>127857</v>
       </c>
       <c r="AN9" t="inlineStr">
         <is>
@@ -4562,10 +4530,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT9" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT9" t="n">
+        <v>3500</v>
       </c>
       <c r="AU9" t="inlineStr"/>
       <c r="AV9" t="inlineStr">
@@ -4693,10 +4659,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE9" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE9" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF9" t="inlineStr">
         <is>
@@ -4713,15 +4677,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI9" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ9" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI9" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ9" t="n">
+        <v>12344</v>
       </c>
       <c r="DK9" t="inlineStr">
         <is>
@@ -4733,10 +4693,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM9" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM9" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN9" t="inlineStr"/>
       <c r="DO9" t="inlineStr">
@@ -4754,15 +4712,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR9" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS9" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR9" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS9" t="n">
+        <v>3144</v>
       </c>
       <c r="DT9" t="inlineStr">
         <is>
@@ -4779,10 +4733,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW9" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW9" t="n">
+        <v>124</v>
       </c>
       <c r="DX9" t="inlineStr">
         <is>
@@ -4847,247 +4799,1364 @@
         </is>
       </c>
       <c r="EL9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>05/06/2026, 13:45:43</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>84</v>
+      </c>
+      <c r="D10" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E10" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F10" t="n">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L10" t="n">
+        <v>408</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O10" t="n">
+        <v>408</v>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q10" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R10" t="n">
+        <v>1780677461</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>13:37</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>05/06/2026 13:37</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W10" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z10" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB10" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC10" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE10" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr"/>
+      <c r="AI10" t="inlineStr"/>
+      <c r="AJ10" t="inlineStr"/>
+      <c r="AK10" t="inlineStr"/>
+      <c r="AL10" t="inlineStr"/>
+      <c r="AM10" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT10" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU10" t="inlineStr"/>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr"/>
+      <c r="BD10" t="inlineStr"/>
+      <c r="BE10" t="inlineStr"/>
+      <c r="BF10" t="inlineStr"/>
+      <c r="BG10" t="inlineStr"/>
+      <c r="BH10" t="inlineStr"/>
+      <c r="BI10" t="inlineStr"/>
+      <c r="BJ10" t="inlineStr"/>
+      <c r="BK10" t="inlineStr"/>
+      <c r="BL10" t="inlineStr"/>
+      <c r="BM10" t="inlineStr"/>
+      <c r="BN10" t="inlineStr"/>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr"/>
+      <c r="BU10" t="inlineStr"/>
+      <c r="BV10" t="inlineStr"/>
+      <c r="BW10" t="inlineStr"/>
+      <c r="BX10" t="inlineStr"/>
+      <c r="BY10" t="inlineStr"/>
+      <c r="BZ10" t="inlineStr"/>
+      <c r="CA10" t="inlineStr"/>
+      <c r="CB10" t="inlineStr"/>
+      <c r="CC10" t="inlineStr"/>
+      <c r="CD10" t="inlineStr"/>
+      <c r="CE10" t="inlineStr"/>
+      <c r="CF10" t="inlineStr"/>
+      <c r="CG10" t="inlineStr"/>
+      <c r="CH10" t="inlineStr"/>
+      <c r="CI10" t="inlineStr"/>
+      <c r="CJ10" t="inlineStr"/>
+      <c r="CK10" t="inlineStr"/>
+      <c r="CL10" t="inlineStr"/>
+      <c r="CM10" t="inlineStr"/>
+      <c r="CN10" t="inlineStr"/>
+      <c r="CO10" t="inlineStr"/>
+      <c r="CP10" t="inlineStr"/>
+      <c r="CQ10" t="inlineStr"/>
+      <c r="CR10" t="inlineStr"/>
+      <c r="CS10" t="inlineStr"/>
+      <c r="CT10" t="inlineStr"/>
+      <c r="CU10" t="inlineStr"/>
+      <c r="CV10" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW10" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX10" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY10" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ10" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA10" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB10" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC10" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD10" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE10" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF10" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG10" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH10" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI10" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ10" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK10" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL10" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM10" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN10" t="inlineStr"/>
+      <c r="DO10" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP10" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ10" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR10" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS10" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT10" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU10" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV10" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW10" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX10" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY10" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ10" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA10" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB10" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC10" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED10" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE10" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF10" t="inlineStr"/>
+      <c r="EG10" t="inlineStr"/>
+      <c r="EH10" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI10" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ10" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK10" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL10" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>05/06/2026, 13:52:22</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>84</v>
+      </c>
+      <c r="D11" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L11" t="n">
+        <v>408</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O11" t="n">
+        <v>408</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q11" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R11" t="n">
+        <v>1780677859</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>13:44</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>05/06/2026 13:44</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W11" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z11" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB11" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC11" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE11" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr"/>
+      <c r="AI11" t="inlineStr"/>
+      <c r="AJ11" t="inlineStr"/>
+      <c r="AK11" t="inlineStr"/>
+      <c r="AL11" t="inlineStr"/>
+      <c r="AM11" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT11" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU11" t="inlineStr"/>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr"/>
+      <c r="BD11" t="inlineStr"/>
+      <c r="BE11" t="inlineStr"/>
+      <c r="BF11" t="inlineStr"/>
+      <c r="BG11" t="inlineStr"/>
+      <c r="BH11" t="inlineStr"/>
+      <c r="BI11" t="inlineStr"/>
+      <c r="BJ11" t="inlineStr"/>
+      <c r="BK11" t="inlineStr"/>
+      <c r="BL11" t="inlineStr"/>
+      <c r="BM11" t="inlineStr"/>
+      <c r="BN11" t="inlineStr"/>
+      <c r="BO11" t="inlineStr"/>
+      <c r="BP11" t="inlineStr"/>
+      <c r="BQ11" t="inlineStr"/>
+      <c r="BR11" t="inlineStr"/>
+      <c r="BS11" t="inlineStr"/>
+      <c r="BT11" t="inlineStr"/>
+      <c r="BU11" t="inlineStr"/>
+      <c r="BV11" t="inlineStr"/>
+      <c r="BW11" t="inlineStr"/>
+      <c r="BX11" t="inlineStr"/>
+      <c r="BY11" t="inlineStr"/>
+      <c r="BZ11" t="inlineStr"/>
+      <c r="CA11" t="inlineStr"/>
+      <c r="CB11" t="inlineStr"/>
+      <c r="CC11" t="inlineStr"/>
+      <c r="CD11" t="inlineStr"/>
+      <c r="CE11" t="inlineStr"/>
+      <c r="CF11" t="inlineStr"/>
+      <c r="CG11" t="inlineStr"/>
+      <c r="CH11" t="inlineStr"/>
+      <c r="CI11" t="inlineStr"/>
+      <c r="CJ11" t="inlineStr"/>
+      <c r="CK11" t="inlineStr"/>
+      <c r="CL11" t="inlineStr"/>
+      <c r="CM11" t="inlineStr"/>
+      <c r="CN11" t="inlineStr"/>
+      <c r="CO11" t="inlineStr"/>
+      <c r="CP11" t="inlineStr"/>
+      <c r="CQ11" t="inlineStr"/>
+      <c r="CR11" t="inlineStr"/>
+      <c r="CS11" t="inlineStr"/>
+      <c r="CT11" t="inlineStr"/>
+      <c r="CU11" t="inlineStr"/>
+      <c r="CV11" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW11" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX11" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY11" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ11" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA11" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB11" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC11" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD11" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE11" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF11" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG11" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH11" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI11" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ11" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK11" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL11" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM11" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN11" t="inlineStr"/>
+      <c r="DO11" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP11" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ11" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR11" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS11" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT11" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU11" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV11" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW11" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX11" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY11" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ11" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA11" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB11" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC11" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED11" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE11" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF11" t="inlineStr"/>
+      <c r="EG11" t="inlineStr"/>
+      <c r="EH11" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI11" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ11" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK11" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>05/06/2026, 13:53:11</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>1780628400</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>1780677909</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>05/06/2026 13:45</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z12" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr"/>
+      <c r="AI12" t="inlineStr"/>
+      <c r="AJ12" t="inlineStr"/>
+      <c r="AK12" t="inlineStr"/>
+      <c r="AL12" t="inlineStr"/>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr"/>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr"/>
+      <c r="BD12" t="inlineStr"/>
+      <c r="BE12" t="inlineStr"/>
+      <c r="BF12" t="inlineStr"/>
+      <c r="BG12" t="inlineStr"/>
+      <c r="BH12" t="inlineStr"/>
+      <c r="BI12" t="inlineStr"/>
+      <c r="BJ12" t="inlineStr"/>
+      <c r="BK12" t="inlineStr"/>
+      <c r="BL12" t="inlineStr"/>
+      <c r="BM12" t="inlineStr"/>
+      <c r="BN12" t="inlineStr"/>
+      <c r="BO12" t="inlineStr"/>
+      <c r="BP12" t="inlineStr"/>
+      <c r="BQ12" t="inlineStr"/>
+      <c r="BR12" t="inlineStr"/>
+      <c r="BS12" t="inlineStr"/>
+      <c r="BT12" t="inlineStr"/>
+      <c r="BU12" t="inlineStr"/>
+      <c r="BV12" t="inlineStr"/>
+      <c r="BW12" t="inlineStr"/>
+      <c r="BX12" t="inlineStr"/>
+      <c r="BY12" t="inlineStr"/>
+      <c r="BZ12" t="inlineStr"/>
+      <c r="CA12" t="inlineStr"/>
+      <c r="CB12" t="inlineStr"/>
+      <c r="CC12" t="inlineStr"/>
+      <c r="CD12" t="inlineStr"/>
+      <c r="CE12" t="inlineStr"/>
+      <c r="CF12" t="inlineStr"/>
+      <c r="CG12" t="inlineStr"/>
+      <c r="CH12" t="inlineStr"/>
+      <c r="CI12" t="inlineStr"/>
+      <c r="CJ12" t="inlineStr"/>
+      <c r="CK12" t="inlineStr"/>
+      <c r="CL12" t="inlineStr"/>
+      <c r="CM12" t="inlineStr"/>
+      <c r="CN12" t="inlineStr"/>
+      <c r="CO12" t="inlineStr"/>
+      <c r="CP12" t="inlineStr"/>
+      <c r="CQ12" t="inlineStr"/>
+      <c r="CR12" t="inlineStr"/>
+      <c r="CS12" t="inlineStr"/>
+      <c r="CT12" t="inlineStr"/>
+      <c r="CU12" t="inlineStr"/>
+      <c r="CV12" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW12" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX12" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY12" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ12" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA12" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB12" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC12" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD12" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE12" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF12" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG12" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH12" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI12" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ12" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK12" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL12" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM12" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN12" t="inlineStr"/>
+      <c r="DO12" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP12" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ12" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR12" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS12" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT12" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU12" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV12" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW12" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX12" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY12" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ12" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA12" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB12" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC12" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED12" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE12" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF12" t="inlineStr"/>
+      <c r="EG12" t="inlineStr"/>
+      <c r="EH12" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI12" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ12" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK12" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B5FCC50092DEF84396333E47DAEFEB5E" ma:contentTypeVersion="13" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3f5dff31fa7a2b799118bc7c00128ae3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" xmlns:ns3="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a22452f93ee1f3c8f432c572ea5d732" ns2:_="" ns3:_="">
-    <xsd:import namespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51"/>
-    <xsd:import namespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4410abd1-e841-4d52-8c09-cc5936d54c0f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{78d918e0-dd2a-4d55-9cd7-b9c5d47e1b97}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5df11fd7-6aff-4cc6-9d69-481ebafd3f51">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{08CAB4CC-F01A-4A7D-9B08-31B78D4FE740}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4D565463-EA89-4DEE-A91D-49D4A0C39119}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1099D124-125E-45CF-9E63-66376AF57B53}"/>
 </file>
</xml_diff>

<commit_message>
Add HTML contract template for PDF generation
- Add modelo_contrato.html with styled contract template
- Add modelo_contrato.txt text version
- Update PDF generator with necessary imports
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL12"/>
+  <dimension ref="A1:EL18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5683,47 +5683,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C12" t="n">
+        <v>84</v>
+      </c>
+      <c r="D12" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>22133</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L12" t="n">
+        <v>408</v>
       </c>
       <c r="M12" t="inlineStr">
         <is>
@@ -5735,25 +5721,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O12" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O12" t="n">
+        <v>408</v>
       </c>
       <c r="P12" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q12" t="inlineStr">
-        <is>
-          <t>1780628400</t>
-        </is>
-      </c>
-      <c r="R12" t="inlineStr">
-        <is>
-          <t>1780677909</t>
-        </is>
+      <c r="Q12" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R12" t="n">
+        <v>1780677909</v>
       </c>
       <c r="S12" t="inlineStr">
         <is>
@@ -5775,10 +5755,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W12" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W12" t="n">
+        <v>22133</v>
       </c>
       <c r="X12" t="inlineStr">
         <is>
@@ -5790,35 +5768,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z12" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z12" t="n">
+        <v>127857</v>
       </c>
       <c r="AA12" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB12" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC12" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB12" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC12" t="n">
+        <v>487</v>
       </c>
       <c r="AD12" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE12" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE12" t="n">
+        <v>121</v>
       </c>
       <c r="AF12" t="inlineStr">
         <is>
@@ -5835,10 +5805,8 @@
       <c r="AJ12" t="inlineStr"/>
       <c r="AK12" t="inlineStr"/>
       <c r="AL12" t="inlineStr"/>
-      <c r="AM12" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM12" t="n">
+        <v>127857</v>
       </c>
       <c r="AN12" t="inlineStr">
         <is>
@@ -5870,10 +5838,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT12" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT12" t="n">
+        <v>3500</v>
       </c>
       <c r="AU12" t="inlineStr"/>
       <c r="AV12" t="inlineStr">
@@ -6001,10 +5967,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE12" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE12" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF12" t="inlineStr">
         <is>
@@ -6021,15 +5985,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI12" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ12" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI12" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ12" t="n">
+        <v>12344</v>
       </c>
       <c r="DK12" t="inlineStr">
         <is>
@@ -6041,10 +6001,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM12" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM12" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN12" t="inlineStr"/>
       <c r="DO12" t="inlineStr">
@@ -6062,15 +6020,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR12" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS12" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR12" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS12" t="n">
+        <v>3144</v>
       </c>
       <c r="DT12" t="inlineStr">
         <is>
@@ -6087,10 +6041,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW12" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW12" t="n">
+        <v>124</v>
       </c>
       <c r="DX12" t="inlineStr">
         <is>
@@ -6155,8 +6107,2911 @@
         </is>
       </c>
       <c r="EL12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>05/06/2026, 15:12:41</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>84</v>
+      </c>
+      <c r="D13" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L13" t="n">
+        <v>408</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O13" t="n">
+        <v>408</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q13" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R13" t="n">
+        <v>1780682678</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>05/06/2026 15:04</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W13" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z13" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB13" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC13" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE13" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr"/>
+      <c r="AI13" t="inlineStr"/>
+      <c r="AJ13" t="inlineStr"/>
+      <c r="AK13" t="inlineStr"/>
+      <c r="AL13" t="inlineStr"/>
+      <c r="AM13" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT13" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU13" t="inlineStr"/>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr"/>
+      <c r="BD13" t="inlineStr"/>
+      <c r="BE13" t="inlineStr"/>
+      <c r="BF13" t="inlineStr"/>
+      <c r="BG13" t="inlineStr"/>
+      <c r="BH13" t="inlineStr"/>
+      <c r="BI13" t="inlineStr"/>
+      <c r="BJ13" t="inlineStr"/>
+      <c r="BK13" t="inlineStr"/>
+      <c r="BL13" t="inlineStr"/>
+      <c r="BM13" t="inlineStr"/>
+      <c r="BN13" t="inlineStr"/>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr"/>
+      <c r="BU13" t="inlineStr"/>
+      <c r="BV13" t="inlineStr"/>
+      <c r="BW13" t="inlineStr"/>
+      <c r="BX13" t="inlineStr"/>
+      <c r="BY13" t="inlineStr"/>
+      <c r="BZ13" t="inlineStr"/>
+      <c r="CA13" t="inlineStr"/>
+      <c r="CB13" t="inlineStr"/>
+      <c r="CC13" t="inlineStr"/>
+      <c r="CD13" t="inlineStr"/>
+      <c r="CE13" t="inlineStr"/>
+      <c r="CF13" t="inlineStr"/>
+      <c r="CG13" t="inlineStr"/>
+      <c r="CH13" t="inlineStr"/>
+      <c r="CI13" t="inlineStr"/>
+      <c r="CJ13" t="inlineStr"/>
+      <c r="CK13" t="inlineStr"/>
+      <c r="CL13" t="inlineStr"/>
+      <c r="CM13" t="inlineStr"/>
+      <c r="CN13" t="inlineStr"/>
+      <c r="CO13" t="inlineStr"/>
+      <c r="CP13" t="inlineStr"/>
+      <c r="CQ13" t="inlineStr"/>
+      <c r="CR13" t="inlineStr"/>
+      <c r="CS13" t="inlineStr"/>
+      <c r="CT13" t="inlineStr"/>
+      <c r="CU13" t="inlineStr"/>
+      <c r="CV13" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW13" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX13" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY13" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ13" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA13" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB13" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC13" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD13" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE13" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF13" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG13" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH13" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI13" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ13" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK13" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL13" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM13" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN13" t="inlineStr"/>
+      <c r="DO13" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP13" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ13" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR13" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS13" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT13" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU13" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV13" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW13" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX13" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY13" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ13" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA13" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB13" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC13" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED13" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE13" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF13" t="inlineStr"/>
+      <c r="EG13" t="inlineStr"/>
+      <c r="EH13" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI13" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ13" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK13" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL13" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05/06/2026, 16:03:47</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>84</v>
+      </c>
+      <c r="D14" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F14" t="n">
+        <v>1</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L14" t="n">
+        <v>408</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O14" t="n">
+        <v>408</v>
+      </c>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q14" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R14" t="n">
+        <v>1780685744</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>15:55</t>
+        </is>
+      </c>
+      <c r="U14" t="inlineStr">
+        <is>
+          <t>05/06/2026 15:55</t>
+        </is>
+      </c>
+      <c r="V14" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W14" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X14" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y14" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z14" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA14" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB14" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC14" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD14" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE14" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF14" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG14" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH14" t="inlineStr"/>
+      <c r="AI14" t="inlineStr"/>
+      <c r="AJ14" t="inlineStr"/>
+      <c r="AK14" t="inlineStr"/>
+      <c r="AL14" t="inlineStr"/>
+      <c r="AM14" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN14" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO14" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP14" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ14" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR14" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS14" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT14" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU14" t="inlineStr"/>
+      <c r="AV14" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW14" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX14" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY14" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ14" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA14" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB14" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC14" t="inlineStr"/>
+      <c r="BD14" t="inlineStr"/>
+      <c r="BE14" t="inlineStr"/>
+      <c r="BF14" t="inlineStr"/>
+      <c r="BG14" t="inlineStr"/>
+      <c r="BH14" t="inlineStr"/>
+      <c r="BI14" t="inlineStr"/>
+      <c r="BJ14" t="inlineStr"/>
+      <c r="BK14" t="inlineStr"/>
+      <c r="BL14" t="inlineStr"/>
+      <c r="BM14" t="inlineStr"/>
+      <c r="BN14" t="inlineStr"/>
+      <c r="BO14" t="inlineStr"/>
+      <c r="BP14" t="inlineStr"/>
+      <c r="BQ14" t="inlineStr"/>
+      <c r="BR14" t="inlineStr"/>
+      <c r="BS14" t="inlineStr"/>
+      <c r="BT14" t="inlineStr"/>
+      <c r="BU14" t="inlineStr"/>
+      <c r="BV14" t="inlineStr"/>
+      <c r="BW14" t="inlineStr"/>
+      <c r="BX14" t="inlineStr"/>
+      <c r="BY14" t="inlineStr"/>
+      <c r="BZ14" t="inlineStr"/>
+      <c r="CA14" t="inlineStr"/>
+      <c r="CB14" t="inlineStr"/>
+      <c r="CC14" t="inlineStr"/>
+      <c r="CD14" t="inlineStr"/>
+      <c r="CE14" t="inlineStr"/>
+      <c r="CF14" t="inlineStr"/>
+      <c r="CG14" t="inlineStr"/>
+      <c r="CH14" t="inlineStr"/>
+      <c r="CI14" t="inlineStr"/>
+      <c r="CJ14" t="inlineStr"/>
+      <c r="CK14" t="inlineStr"/>
+      <c r="CL14" t="inlineStr"/>
+      <c r="CM14" t="inlineStr"/>
+      <c r="CN14" t="inlineStr"/>
+      <c r="CO14" t="inlineStr"/>
+      <c r="CP14" t="inlineStr"/>
+      <c r="CQ14" t="inlineStr"/>
+      <c r="CR14" t="inlineStr"/>
+      <c r="CS14" t="inlineStr"/>
+      <c r="CT14" t="inlineStr"/>
+      <c r="CU14" t="inlineStr"/>
+      <c r="CV14" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW14" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX14" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY14" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ14" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA14" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB14" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC14" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD14" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE14" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF14" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG14" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH14" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI14" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ14" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK14" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL14" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM14" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN14" t="inlineStr"/>
+      <c r="DO14" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP14" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ14" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR14" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS14" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT14" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU14" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV14" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW14" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX14" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY14" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ14" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA14" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB14" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC14" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED14" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE14" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF14" t="inlineStr"/>
+      <c r="EG14" t="inlineStr"/>
+      <c r="EH14" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI14" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ14" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK14" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05/06/2026, 16:10:26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>84</v>
+      </c>
+      <c r="D15" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F15" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L15" t="n">
+        <v>408</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O15" t="n">
+        <v>408</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q15" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R15" t="n">
+        <v>1780686143</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>16:02</t>
+        </is>
+      </c>
+      <c r="U15" t="inlineStr">
+        <is>
+          <t>05/06/2026 16:02</t>
+        </is>
+      </c>
+      <c r="V15" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W15" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X15" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y15" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z15" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA15" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC15" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD15" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE15" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF15" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG15" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH15" t="inlineStr"/>
+      <c r="AI15" t="inlineStr"/>
+      <c r="AJ15" t="inlineStr"/>
+      <c r="AK15" t="inlineStr"/>
+      <c r="AL15" t="inlineStr"/>
+      <c r="AM15" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN15" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO15" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP15" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR15" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS15" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT15" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU15" t="inlineStr"/>
+      <c r="AV15" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW15" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX15" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY15" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ15" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA15" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB15" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC15" t="inlineStr"/>
+      <c r="BD15" t="inlineStr"/>
+      <c r="BE15" t="inlineStr"/>
+      <c r="BF15" t="inlineStr"/>
+      <c r="BG15" t="inlineStr"/>
+      <c r="BH15" t="inlineStr"/>
+      <c r="BI15" t="inlineStr"/>
+      <c r="BJ15" t="inlineStr"/>
+      <c r="BK15" t="inlineStr"/>
+      <c r="BL15" t="inlineStr"/>
+      <c r="BM15" t="inlineStr"/>
+      <c r="BN15" t="inlineStr"/>
+      <c r="BO15" t="inlineStr"/>
+      <c r="BP15" t="inlineStr"/>
+      <c r="BQ15" t="inlineStr"/>
+      <c r="BR15" t="inlineStr"/>
+      <c r="BS15" t="inlineStr"/>
+      <c r="BT15" t="inlineStr"/>
+      <c r="BU15" t="inlineStr"/>
+      <c r="BV15" t="inlineStr"/>
+      <c r="BW15" t="inlineStr"/>
+      <c r="BX15" t="inlineStr"/>
+      <c r="BY15" t="inlineStr"/>
+      <c r="BZ15" t="inlineStr"/>
+      <c r="CA15" t="inlineStr"/>
+      <c r="CB15" t="inlineStr"/>
+      <c r="CC15" t="inlineStr"/>
+      <c r="CD15" t="inlineStr"/>
+      <c r="CE15" t="inlineStr"/>
+      <c r="CF15" t="inlineStr"/>
+      <c r="CG15" t="inlineStr"/>
+      <c r="CH15" t="inlineStr"/>
+      <c r="CI15" t="inlineStr"/>
+      <c r="CJ15" t="inlineStr"/>
+      <c r="CK15" t="inlineStr"/>
+      <c r="CL15" t="inlineStr"/>
+      <c r="CM15" t="inlineStr"/>
+      <c r="CN15" t="inlineStr"/>
+      <c r="CO15" t="inlineStr"/>
+      <c r="CP15" t="inlineStr"/>
+      <c r="CQ15" t="inlineStr"/>
+      <c r="CR15" t="inlineStr"/>
+      <c r="CS15" t="inlineStr"/>
+      <c r="CT15" t="inlineStr"/>
+      <c r="CU15" t="inlineStr"/>
+      <c r="CV15" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW15" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX15" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY15" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ15" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA15" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB15" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC15" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD15" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE15" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF15" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG15" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH15" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI15" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ15" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK15" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL15" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM15" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN15" t="inlineStr"/>
+      <c r="DO15" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP15" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ15" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR15" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS15" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT15" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU15" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV15" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW15" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX15" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY15" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ15" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA15" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB15" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC15" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED15" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE15" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF15" t="inlineStr"/>
+      <c r="EG15" t="inlineStr"/>
+      <c r="EH15" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI15" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ15" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK15" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05/06/2026, 16:44:39</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>84</v>
+      </c>
+      <c r="D16" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E16" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L16" t="n">
+        <v>408</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O16" t="n">
+        <v>408</v>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q16" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R16" t="n">
+        <v>1780688196</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>16:36</t>
+        </is>
+      </c>
+      <c r="U16" t="inlineStr">
+        <is>
+          <t>05/06/2026 16:36</t>
+        </is>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W16" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X16" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y16" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z16" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA16" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC16" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD16" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE16" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF16" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG16" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH16" t="inlineStr"/>
+      <c r="AI16" t="inlineStr"/>
+      <c r="AJ16" t="inlineStr"/>
+      <c r="AK16" t="inlineStr"/>
+      <c r="AL16" t="inlineStr"/>
+      <c r="AM16" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN16" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO16" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP16" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR16" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS16" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT16" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU16" t="inlineStr"/>
+      <c r="AV16" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW16" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX16" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY16" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ16" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA16" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB16" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC16" t="inlineStr"/>
+      <c r="BD16" t="inlineStr"/>
+      <c r="BE16" t="inlineStr"/>
+      <c r="BF16" t="inlineStr"/>
+      <c r="BG16" t="inlineStr"/>
+      <c r="BH16" t="inlineStr"/>
+      <c r="BI16" t="inlineStr"/>
+      <c r="BJ16" t="inlineStr"/>
+      <c r="BK16" t="inlineStr"/>
+      <c r="BL16" t="inlineStr"/>
+      <c r="BM16" t="inlineStr"/>
+      <c r="BN16" t="inlineStr"/>
+      <c r="BO16" t="inlineStr"/>
+      <c r="BP16" t="inlineStr"/>
+      <c r="BQ16" t="inlineStr"/>
+      <c r="BR16" t="inlineStr"/>
+      <c r="BS16" t="inlineStr"/>
+      <c r="BT16" t="inlineStr"/>
+      <c r="BU16" t="inlineStr"/>
+      <c r="BV16" t="inlineStr"/>
+      <c r="BW16" t="inlineStr"/>
+      <c r="BX16" t="inlineStr"/>
+      <c r="BY16" t="inlineStr"/>
+      <c r="BZ16" t="inlineStr"/>
+      <c r="CA16" t="inlineStr"/>
+      <c r="CB16" t="inlineStr"/>
+      <c r="CC16" t="inlineStr"/>
+      <c r="CD16" t="inlineStr"/>
+      <c r="CE16" t="inlineStr"/>
+      <c r="CF16" t="inlineStr"/>
+      <c r="CG16" t="inlineStr"/>
+      <c r="CH16" t="inlineStr"/>
+      <c r="CI16" t="inlineStr"/>
+      <c r="CJ16" t="inlineStr"/>
+      <c r="CK16" t="inlineStr"/>
+      <c r="CL16" t="inlineStr"/>
+      <c r="CM16" t="inlineStr"/>
+      <c r="CN16" t="inlineStr"/>
+      <c r="CO16" t="inlineStr"/>
+      <c r="CP16" t="inlineStr"/>
+      <c r="CQ16" t="inlineStr"/>
+      <c r="CR16" t="inlineStr"/>
+      <c r="CS16" t="inlineStr"/>
+      <c r="CT16" t="inlineStr"/>
+      <c r="CU16" t="inlineStr"/>
+      <c r="CV16" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW16" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX16" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY16" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ16" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA16" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB16" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC16" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD16" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE16" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF16" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG16" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH16" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI16" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ16" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK16" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL16" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM16" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN16" t="inlineStr"/>
+      <c r="DO16" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP16" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ16" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR16" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS16" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT16" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU16" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV16" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW16" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX16" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY16" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ16" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA16" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB16" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC16" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED16" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE16" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF16" t="inlineStr"/>
+      <c r="EG16" t="inlineStr"/>
+      <c r="EH16" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI16" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ16" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK16" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>05/06/2026, 17:04:12</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>84</v>
+      </c>
+      <c r="D17" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F17" t="n">
+        <v>1</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L17" t="n">
+        <v>408</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O17" t="n">
+        <v>408</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q17" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R17" t="n">
+        <v>1780689369</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>16:56</t>
+        </is>
+      </c>
+      <c r="U17" t="inlineStr">
+        <is>
+          <t>05/06/2026 16:56</t>
+        </is>
+      </c>
+      <c r="V17" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W17" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X17" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y17" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z17" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA17" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB17" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC17" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD17" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE17" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF17" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG17" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH17" t="inlineStr"/>
+      <c r="AI17" t="inlineStr"/>
+      <c r="AJ17" t="inlineStr"/>
+      <c r="AK17" t="inlineStr"/>
+      <c r="AL17" t="inlineStr"/>
+      <c r="AM17" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN17" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO17" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP17" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ17" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR17" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS17" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT17" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU17" t="inlineStr"/>
+      <c r="AV17" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW17" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX17" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY17" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ17" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA17" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB17" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC17" t="inlineStr"/>
+      <c r="BD17" t="inlineStr"/>
+      <c r="BE17" t="inlineStr"/>
+      <c r="BF17" t="inlineStr"/>
+      <c r="BG17" t="inlineStr"/>
+      <c r="BH17" t="inlineStr"/>
+      <c r="BI17" t="inlineStr"/>
+      <c r="BJ17" t="inlineStr"/>
+      <c r="BK17" t="inlineStr"/>
+      <c r="BL17" t="inlineStr"/>
+      <c r="BM17" t="inlineStr"/>
+      <c r="BN17" t="inlineStr"/>
+      <c r="BO17" t="inlineStr"/>
+      <c r="BP17" t="inlineStr"/>
+      <c r="BQ17" t="inlineStr"/>
+      <c r="BR17" t="inlineStr"/>
+      <c r="BS17" t="inlineStr"/>
+      <c r="BT17" t="inlineStr"/>
+      <c r="BU17" t="inlineStr"/>
+      <c r="BV17" t="inlineStr"/>
+      <c r="BW17" t="inlineStr"/>
+      <c r="BX17" t="inlineStr"/>
+      <c r="BY17" t="inlineStr"/>
+      <c r="BZ17" t="inlineStr"/>
+      <c r="CA17" t="inlineStr"/>
+      <c r="CB17" t="inlineStr"/>
+      <c r="CC17" t="inlineStr"/>
+      <c r="CD17" t="inlineStr"/>
+      <c r="CE17" t="inlineStr"/>
+      <c r="CF17" t="inlineStr"/>
+      <c r="CG17" t="inlineStr"/>
+      <c r="CH17" t="inlineStr"/>
+      <c r="CI17" t="inlineStr"/>
+      <c r="CJ17" t="inlineStr"/>
+      <c r="CK17" t="inlineStr"/>
+      <c r="CL17" t="inlineStr"/>
+      <c r="CM17" t="inlineStr"/>
+      <c r="CN17" t="inlineStr"/>
+      <c r="CO17" t="inlineStr"/>
+      <c r="CP17" t="inlineStr"/>
+      <c r="CQ17" t="inlineStr"/>
+      <c r="CR17" t="inlineStr"/>
+      <c r="CS17" t="inlineStr"/>
+      <c r="CT17" t="inlineStr"/>
+      <c r="CU17" t="inlineStr"/>
+      <c r="CV17" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW17" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX17" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY17" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ17" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA17" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB17" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC17" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD17" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE17" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF17" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG17" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH17" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI17" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ17" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK17" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL17" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM17" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN17" t="inlineStr"/>
+      <c r="DO17" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP17" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ17" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR17" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS17" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT17" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU17" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV17" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW17" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX17" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY17" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ17" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA17" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB17" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC17" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED17" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE17" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF17" t="inlineStr"/>
+      <c r="EG17" t="inlineStr"/>
+      <c r="EH17" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI17" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ17" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK17" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>05/06/2026, 17:17:06</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>1780628400</t>
+        </is>
+      </c>
+      <c r="R18" t="inlineStr">
+        <is>
+          <t>1780690142</t>
+        </is>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>05/06/2026</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>17:09</t>
+        </is>
+      </c>
+      <c r="U18" t="inlineStr">
+        <is>
+          <t>05/06/2026 17:09</t>
+        </is>
+      </c>
+      <c r="V18" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W18" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X18" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y18" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z18" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC18" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD18" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE18" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF18" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG18" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
+      <c r="AL18" t="inlineStr"/>
+      <c r="AM18" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN18" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO18" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP18" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ18" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR18" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS18" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT18" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU18" t="inlineStr"/>
+      <c r="AV18" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW18" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX18" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY18" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ18" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA18" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB18" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC18" t="inlineStr"/>
+      <c r="BD18" t="inlineStr"/>
+      <c r="BE18" t="inlineStr"/>
+      <c r="BF18" t="inlineStr"/>
+      <c r="BG18" t="inlineStr"/>
+      <c r="BH18" t="inlineStr"/>
+      <c r="BI18" t="inlineStr"/>
+      <c r="BJ18" t="inlineStr"/>
+      <c r="BK18" t="inlineStr"/>
+      <c r="BL18" t="inlineStr"/>
+      <c r="BM18" t="inlineStr"/>
+      <c r="BN18" t="inlineStr"/>
+      <c r="BO18" t="inlineStr"/>
+      <c r="BP18" t="inlineStr"/>
+      <c r="BQ18" t="inlineStr"/>
+      <c r="BR18" t="inlineStr"/>
+      <c r="BS18" t="inlineStr"/>
+      <c r="BT18" t="inlineStr"/>
+      <c r="BU18" t="inlineStr"/>
+      <c r="BV18" t="inlineStr"/>
+      <c r="BW18" t="inlineStr"/>
+      <c r="BX18" t="inlineStr"/>
+      <c r="BY18" t="inlineStr"/>
+      <c r="BZ18" t="inlineStr"/>
+      <c r="CA18" t="inlineStr"/>
+      <c r="CB18" t="inlineStr"/>
+      <c r="CC18" t="inlineStr"/>
+      <c r="CD18" t="inlineStr"/>
+      <c r="CE18" t="inlineStr"/>
+      <c r="CF18" t="inlineStr"/>
+      <c r="CG18" t="inlineStr"/>
+      <c r="CH18" t="inlineStr"/>
+      <c r="CI18" t="inlineStr"/>
+      <c r="CJ18" t="inlineStr"/>
+      <c r="CK18" t="inlineStr"/>
+      <c r="CL18" t="inlineStr"/>
+      <c r="CM18" t="inlineStr"/>
+      <c r="CN18" t="inlineStr"/>
+      <c r="CO18" t="inlineStr"/>
+      <c r="CP18" t="inlineStr"/>
+      <c r="CQ18" t="inlineStr"/>
+      <c r="CR18" t="inlineStr"/>
+      <c r="CS18" t="inlineStr"/>
+      <c r="CT18" t="inlineStr"/>
+      <c r="CU18" t="inlineStr"/>
+      <c r="CV18" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW18" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX18" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY18" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ18" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA18" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB18" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC18" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD18" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE18" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF18" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG18" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH18" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI18" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ18" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK18" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL18" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM18" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN18" t="inlineStr"/>
+      <c r="DO18" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP18" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ18" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR18" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS18" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT18" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU18" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV18" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW18" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX18" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY18" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ18" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA18" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB18" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC18" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED18" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE18" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF18" t="inlineStr"/>
+      <c r="EG18" t="inlineStr"/>
+      <c r="EH18" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI18" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ18" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK18" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL18" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B5FCC50092DEF84396333E47DAEFEB5E" ma:contentTypeVersion="13" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3f5dff31fa7a2b799118bc7c00128ae3">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" xmlns:ns3="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a22452f93ee1f3c8f432c572ea5d732" ns2:_="" ns3:_="">
+    <xsd:import namespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51"/>
+    <xsd:import namespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4410abd1-e841-4d52-8c09-cc5936d54c0f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{78d918e0-dd2a-4d55-9cd7-b9c5d47e1b97}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5df11fd7-6aff-4cc6-9d69-481ebafd3f51">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E5362F9-87DC-4D00-AC6A-0D4FA0E11BC8}"/>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60550303-CF0E-48C3-9117-6FA69E4BED68}"/>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F51F449-F139-4018-8D77-64162D58004A}"/>
 </file>
</xml_diff>

<commit_message>
Refactor HTML contract template with improved structure and styling
- Revamp `modelo_contrato.html` with a cleaner, modular style
- Enhance layout and typography for improved readability
- Use semantic HTML5 elements and responsive design techniques
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL18"/>
+  <dimension ref="A1:EL26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8299,47 +8299,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C18" t="n">
+        <v>84</v>
+      </c>
+      <c r="D18" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E18" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F18" t="n">
+        <v>1</v>
       </c>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I18" t="n">
+        <v>0</v>
+      </c>
+      <c r="J18" t="n">
+        <v>22133</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L18" t="n">
+        <v>408</v>
       </c>
       <c r="M18" t="inlineStr">
         <is>
@@ -8351,25 +8337,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O18" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O18" t="n">
+        <v>408</v>
       </c>
       <c r="P18" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q18" t="inlineStr">
-        <is>
-          <t>1780628400</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>1780690142</t>
-        </is>
+      <c r="Q18" t="n">
+        <v>1780628400</v>
+      </c>
+      <c r="R18" t="n">
+        <v>1780690142</v>
       </c>
       <c r="S18" t="inlineStr">
         <is>
@@ -8391,10 +8371,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W18" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W18" t="n">
+        <v>22133</v>
       </c>
       <c r="X18" t="inlineStr">
         <is>
@@ -8406,35 +8384,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z18" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z18" t="n">
+        <v>127857</v>
       </c>
       <c r="AA18" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB18" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC18" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB18" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC18" t="n">
+        <v>487</v>
       </c>
       <c r="AD18" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE18" t="n">
+        <v>121</v>
       </c>
       <c r="AF18" t="inlineStr">
         <is>
@@ -8451,10 +8421,8 @@
       <c r="AJ18" t="inlineStr"/>
       <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="inlineStr"/>
-      <c r="AM18" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM18" t="n">
+        <v>127857</v>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
@@ -8486,10 +8454,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT18" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT18" t="n">
+        <v>3500</v>
       </c>
       <c r="AU18" t="inlineStr"/>
       <c r="AV18" t="inlineStr">
@@ -8617,10 +8583,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE18" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE18" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF18" t="inlineStr">
         <is>
@@ -8637,15 +8601,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI18" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ18" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI18" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ18" t="n">
+        <v>12344</v>
       </c>
       <c r="DK18" t="inlineStr">
         <is>
@@ -8657,10 +8617,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM18" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM18" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN18" t="inlineStr"/>
       <c r="DO18" t="inlineStr">
@@ -8678,15 +8636,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR18" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS18" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR18" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS18" t="n">
+        <v>3144</v>
       </c>
       <c r="DT18" t="inlineStr">
         <is>
@@ -8703,10 +8657,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW18" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW18" t="n">
+        <v>124</v>
       </c>
       <c r="DX18" t="inlineStr">
         <is>
@@ -8771,6 +8723,3542 @@
         </is>
       </c>
       <c r="EL18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>08/06/2026, 09:00:42</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>84</v>
+      </c>
+      <c r="D19" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E19" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L19" t="n">
+        <v>408</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O19" t="n">
+        <v>408</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q19" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R19" t="n">
+        <v>1780919542</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>08:52</t>
+        </is>
+      </c>
+      <c r="U19" t="inlineStr">
+        <is>
+          <t>08/06/2026 08:52</t>
+        </is>
+      </c>
+      <c r="V19" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W19" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X19" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y19" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z19" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA19" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB19" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC19" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD19" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE19" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF19" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG19" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH19" t="inlineStr"/>
+      <c r="AI19" t="inlineStr"/>
+      <c r="AJ19" t="inlineStr"/>
+      <c r="AK19" t="inlineStr"/>
+      <c r="AL19" t="inlineStr"/>
+      <c r="AM19" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN19" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO19" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP19" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ19" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR19" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS19" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT19" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU19" t="inlineStr"/>
+      <c r="AV19" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW19" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX19" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY19" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ19" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA19" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB19" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC19" t="inlineStr"/>
+      <c r="BD19" t="inlineStr"/>
+      <c r="BE19" t="inlineStr"/>
+      <c r="BF19" t="inlineStr"/>
+      <c r="BG19" t="inlineStr"/>
+      <c r="BH19" t="inlineStr"/>
+      <c r="BI19" t="inlineStr"/>
+      <c r="BJ19" t="inlineStr"/>
+      <c r="BK19" t="inlineStr"/>
+      <c r="BL19" t="inlineStr"/>
+      <c r="BM19" t="inlineStr"/>
+      <c r="BN19" t="inlineStr"/>
+      <c r="BO19" t="inlineStr"/>
+      <c r="BP19" t="inlineStr"/>
+      <c r="BQ19" t="inlineStr"/>
+      <c r="BR19" t="inlineStr"/>
+      <c r="BS19" t="inlineStr"/>
+      <c r="BT19" t="inlineStr"/>
+      <c r="BU19" t="inlineStr"/>
+      <c r="BV19" t="inlineStr"/>
+      <c r="BW19" t="inlineStr"/>
+      <c r="BX19" t="inlineStr"/>
+      <c r="BY19" t="inlineStr"/>
+      <c r="BZ19" t="inlineStr"/>
+      <c r="CA19" t="inlineStr"/>
+      <c r="CB19" t="inlineStr"/>
+      <c r="CC19" t="inlineStr"/>
+      <c r="CD19" t="inlineStr"/>
+      <c r="CE19" t="inlineStr"/>
+      <c r="CF19" t="inlineStr"/>
+      <c r="CG19" t="inlineStr"/>
+      <c r="CH19" t="inlineStr"/>
+      <c r="CI19" t="inlineStr"/>
+      <c r="CJ19" t="inlineStr"/>
+      <c r="CK19" t="inlineStr"/>
+      <c r="CL19" t="inlineStr"/>
+      <c r="CM19" t="inlineStr"/>
+      <c r="CN19" t="inlineStr"/>
+      <c r="CO19" t="inlineStr"/>
+      <c r="CP19" t="inlineStr"/>
+      <c r="CQ19" t="inlineStr"/>
+      <c r="CR19" t="inlineStr"/>
+      <c r="CS19" t="inlineStr"/>
+      <c r="CT19" t="inlineStr"/>
+      <c r="CU19" t="inlineStr"/>
+      <c r="CV19" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW19" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX19" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY19" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ19" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA19" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB19" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC19" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD19" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE19" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF19" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG19" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH19" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI19" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ19" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK19" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL19" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM19" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN19" t="inlineStr"/>
+      <c r="DO19" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP19" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ19" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR19" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS19" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT19" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU19" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV19" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW19" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX19" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY19" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ19" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA19" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB19" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC19" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED19" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE19" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF19" t="inlineStr"/>
+      <c r="EG19" t="inlineStr"/>
+      <c r="EH19" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI19" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ19" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK19" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>08/06/2026, 09:07:11</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>84</v>
+      </c>
+      <c r="D20" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E20" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F20" t="n">
+        <v>1</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="n">
+        <v>0</v>
+      </c>
+      <c r="J20" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L20" t="n">
+        <v>408</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O20" t="n">
+        <v>408</v>
+      </c>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q20" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R20" t="n">
+        <v>1780919931</v>
+      </c>
+      <c r="S20" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T20" t="inlineStr">
+        <is>
+          <t>08:58</t>
+        </is>
+      </c>
+      <c r="U20" t="inlineStr">
+        <is>
+          <t>08/06/2026 08:58</t>
+        </is>
+      </c>
+      <c r="V20" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W20" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X20" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y20" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z20" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB20" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC20" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD20" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE20" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF20" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG20" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH20" t="inlineStr"/>
+      <c r="AI20" t="inlineStr"/>
+      <c r="AJ20" t="inlineStr"/>
+      <c r="AK20" t="inlineStr"/>
+      <c r="AL20" t="inlineStr"/>
+      <c r="AM20" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN20" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO20" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP20" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ20" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR20" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS20" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT20" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU20" t="inlineStr"/>
+      <c r="AV20" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW20" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX20" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY20" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ20" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA20" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB20" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC20" t="inlineStr"/>
+      <c r="BD20" t="inlineStr"/>
+      <c r="BE20" t="inlineStr"/>
+      <c r="BF20" t="inlineStr"/>
+      <c r="BG20" t="inlineStr"/>
+      <c r="BH20" t="inlineStr"/>
+      <c r="BI20" t="inlineStr"/>
+      <c r="BJ20" t="inlineStr"/>
+      <c r="BK20" t="inlineStr"/>
+      <c r="BL20" t="inlineStr"/>
+      <c r="BM20" t="inlineStr"/>
+      <c r="BN20" t="inlineStr"/>
+      <c r="BO20" t="inlineStr"/>
+      <c r="BP20" t="inlineStr"/>
+      <c r="BQ20" t="inlineStr"/>
+      <c r="BR20" t="inlineStr"/>
+      <c r="BS20" t="inlineStr"/>
+      <c r="BT20" t="inlineStr"/>
+      <c r="BU20" t="inlineStr"/>
+      <c r="BV20" t="inlineStr"/>
+      <c r="BW20" t="inlineStr"/>
+      <c r="BX20" t="inlineStr"/>
+      <c r="BY20" t="inlineStr"/>
+      <c r="BZ20" t="inlineStr"/>
+      <c r="CA20" t="inlineStr"/>
+      <c r="CB20" t="inlineStr"/>
+      <c r="CC20" t="inlineStr"/>
+      <c r="CD20" t="inlineStr"/>
+      <c r="CE20" t="inlineStr"/>
+      <c r="CF20" t="inlineStr"/>
+      <c r="CG20" t="inlineStr"/>
+      <c r="CH20" t="inlineStr"/>
+      <c r="CI20" t="inlineStr"/>
+      <c r="CJ20" t="inlineStr"/>
+      <c r="CK20" t="inlineStr"/>
+      <c r="CL20" t="inlineStr"/>
+      <c r="CM20" t="inlineStr"/>
+      <c r="CN20" t="inlineStr"/>
+      <c r="CO20" t="inlineStr"/>
+      <c r="CP20" t="inlineStr"/>
+      <c r="CQ20" t="inlineStr"/>
+      <c r="CR20" t="inlineStr"/>
+      <c r="CS20" t="inlineStr"/>
+      <c r="CT20" t="inlineStr"/>
+      <c r="CU20" t="inlineStr"/>
+      <c r="CV20" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW20" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX20" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY20" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ20" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA20" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB20" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC20" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD20" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE20" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF20" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG20" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH20" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI20" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ20" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK20" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL20" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM20" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN20" t="inlineStr"/>
+      <c r="DO20" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP20" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ20" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR20" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS20" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT20" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU20" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV20" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW20" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX20" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY20" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ20" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA20" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB20" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC20" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED20" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE20" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF20" t="inlineStr"/>
+      <c r="EG20" t="inlineStr"/>
+      <c r="EH20" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI20" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ20" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK20" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>08/06/2026, 12:16:38</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C21" t="n">
+        <v>84</v>
+      </c>
+      <c r="D21" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E21" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="n">
+        <v>0</v>
+      </c>
+      <c r="J21" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L21" t="n">
+        <v>408</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O21" t="n">
+        <v>408</v>
+      </c>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q21" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R21" t="n">
+        <v>1780931293</v>
+      </c>
+      <c r="S21" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T21" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="U21" t="inlineStr">
+        <is>
+          <t>08/06/2026 12:08</t>
+        </is>
+      </c>
+      <c r="V21" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W21" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X21" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y21" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z21" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA21" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC21" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD21" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE21" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF21" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG21" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH21" t="inlineStr"/>
+      <c r="AI21" t="inlineStr"/>
+      <c r="AJ21" t="inlineStr"/>
+      <c r="AK21" t="inlineStr"/>
+      <c r="AL21" t="inlineStr"/>
+      <c r="AM21" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN21" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO21" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP21" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ21" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR21" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS21" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT21" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU21" t="inlineStr"/>
+      <c r="AV21" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW21" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX21" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY21" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ21" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA21" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB21" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC21" t="inlineStr"/>
+      <c r="BD21" t="inlineStr"/>
+      <c r="BE21" t="inlineStr"/>
+      <c r="BF21" t="inlineStr"/>
+      <c r="BG21" t="inlineStr"/>
+      <c r="BH21" t="inlineStr"/>
+      <c r="BI21" t="inlineStr"/>
+      <c r="BJ21" t="inlineStr"/>
+      <c r="BK21" t="inlineStr"/>
+      <c r="BL21" t="inlineStr"/>
+      <c r="BM21" t="inlineStr"/>
+      <c r="BN21" t="inlineStr"/>
+      <c r="BO21" t="inlineStr"/>
+      <c r="BP21" t="inlineStr"/>
+      <c r="BQ21" t="inlineStr"/>
+      <c r="BR21" t="inlineStr"/>
+      <c r="BS21" t="inlineStr"/>
+      <c r="BT21" t="inlineStr"/>
+      <c r="BU21" t="inlineStr"/>
+      <c r="BV21" t="inlineStr"/>
+      <c r="BW21" t="inlineStr"/>
+      <c r="BX21" t="inlineStr"/>
+      <c r="BY21" t="inlineStr"/>
+      <c r="BZ21" t="inlineStr"/>
+      <c r="CA21" t="inlineStr"/>
+      <c r="CB21" t="inlineStr"/>
+      <c r="CC21" t="inlineStr"/>
+      <c r="CD21" t="inlineStr"/>
+      <c r="CE21" t="inlineStr"/>
+      <c r="CF21" t="inlineStr"/>
+      <c r="CG21" t="inlineStr"/>
+      <c r="CH21" t="inlineStr"/>
+      <c r="CI21" t="inlineStr"/>
+      <c r="CJ21" t="inlineStr"/>
+      <c r="CK21" t="inlineStr"/>
+      <c r="CL21" t="inlineStr"/>
+      <c r="CM21" t="inlineStr"/>
+      <c r="CN21" t="inlineStr"/>
+      <c r="CO21" t="inlineStr"/>
+      <c r="CP21" t="inlineStr"/>
+      <c r="CQ21" t="inlineStr"/>
+      <c r="CR21" t="inlineStr"/>
+      <c r="CS21" t="inlineStr"/>
+      <c r="CT21" t="inlineStr"/>
+      <c r="CU21" t="inlineStr"/>
+      <c r="CV21" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW21" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX21" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY21" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ21" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA21" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB21" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC21" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD21" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE21" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF21" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG21" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH21" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI21" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ21" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK21" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL21" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM21" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN21" t="inlineStr"/>
+      <c r="DO21" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP21" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ21" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR21" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS21" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT21" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU21" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV21" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW21" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX21" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY21" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ21" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA21" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB21" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC21" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED21" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE21" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF21" t="inlineStr"/>
+      <c r="EG21" t="inlineStr"/>
+      <c r="EH21" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI21" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ21" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK21" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>08/06/2026, 12:17:55</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C22" t="n">
+        <v>84</v>
+      </c>
+      <c r="D22" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E22" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="n">
+        <v>0</v>
+      </c>
+      <c r="J22" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L22" t="n">
+        <v>408</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O22" t="n">
+        <v>408</v>
+      </c>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q22" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R22" t="n">
+        <v>1780931370</v>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>12:09</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>08/06/2026 12:09</t>
+        </is>
+      </c>
+      <c r="V22" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W22" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X22" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y22" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z22" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE22" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH22" t="inlineStr"/>
+      <c r="AI22" t="inlineStr"/>
+      <c r="AJ22" t="inlineStr"/>
+      <c r="AK22" t="inlineStr"/>
+      <c r="AL22" t="inlineStr"/>
+      <c r="AM22" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP22" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ22" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR22" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT22" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU22" t="inlineStr"/>
+      <c r="AV22" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW22" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY22" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ22" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA22" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB22" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC22" t="inlineStr"/>
+      <c r="BD22" t="inlineStr"/>
+      <c r="BE22" t="inlineStr"/>
+      <c r="BF22" t="inlineStr"/>
+      <c r="BG22" t="inlineStr"/>
+      <c r="BH22" t="inlineStr"/>
+      <c r="BI22" t="inlineStr"/>
+      <c r="BJ22" t="inlineStr"/>
+      <c r="BK22" t="inlineStr"/>
+      <c r="BL22" t="inlineStr"/>
+      <c r="BM22" t="inlineStr"/>
+      <c r="BN22" t="inlineStr"/>
+      <c r="BO22" t="inlineStr"/>
+      <c r="BP22" t="inlineStr"/>
+      <c r="BQ22" t="inlineStr"/>
+      <c r="BR22" t="inlineStr"/>
+      <c r="BS22" t="inlineStr"/>
+      <c r="BT22" t="inlineStr"/>
+      <c r="BU22" t="inlineStr"/>
+      <c r="BV22" t="inlineStr"/>
+      <c r="BW22" t="inlineStr"/>
+      <c r="BX22" t="inlineStr"/>
+      <c r="BY22" t="inlineStr"/>
+      <c r="BZ22" t="inlineStr"/>
+      <c r="CA22" t="inlineStr"/>
+      <c r="CB22" t="inlineStr"/>
+      <c r="CC22" t="inlineStr"/>
+      <c r="CD22" t="inlineStr"/>
+      <c r="CE22" t="inlineStr"/>
+      <c r="CF22" t="inlineStr"/>
+      <c r="CG22" t="inlineStr"/>
+      <c r="CH22" t="inlineStr"/>
+      <c r="CI22" t="inlineStr"/>
+      <c r="CJ22" t="inlineStr"/>
+      <c r="CK22" t="inlineStr"/>
+      <c r="CL22" t="inlineStr"/>
+      <c r="CM22" t="inlineStr"/>
+      <c r="CN22" t="inlineStr"/>
+      <c r="CO22" t="inlineStr"/>
+      <c r="CP22" t="inlineStr"/>
+      <c r="CQ22" t="inlineStr"/>
+      <c r="CR22" t="inlineStr"/>
+      <c r="CS22" t="inlineStr"/>
+      <c r="CT22" t="inlineStr"/>
+      <c r="CU22" t="inlineStr"/>
+      <c r="CV22" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW22" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX22" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY22" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ22" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA22" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB22" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC22" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD22" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE22" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF22" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG22" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH22" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI22" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ22" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK22" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL22" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM22" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN22" t="inlineStr"/>
+      <c r="DO22" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP22" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ22" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR22" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS22" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT22" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU22" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV22" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW22" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX22" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY22" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ22" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA22" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB22" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC22" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED22" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE22" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF22" t="inlineStr"/>
+      <c r="EG22" t="inlineStr"/>
+      <c r="EH22" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI22" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ22" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK22" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>08/06/2026, 12:22:00</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>84</v>
+      </c>
+      <c r="D23" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E23" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L23" t="n">
+        <v>408</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O23" t="n">
+        <v>408</v>
+      </c>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q23" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1780931615</v>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>08/06/2026 12:13</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W23" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z23" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA23" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE23" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH23" t="inlineStr"/>
+      <c r="AI23" t="inlineStr"/>
+      <c r="AJ23" t="inlineStr"/>
+      <c r="AK23" t="inlineStr"/>
+      <c r="AL23" t="inlineStr"/>
+      <c r="AM23" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP23" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ23" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR23" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT23" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU23" t="inlineStr"/>
+      <c r="AV23" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW23" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY23" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ23" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA23" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB23" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC23" t="inlineStr"/>
+      <c r="BD23" t="inlineStr"/>
+      <c r="BE23" t="inlineStr"/>
+      <c r="BF23" t="inlineStr"/>
+      <c r="BG23" t="inlineStr"/>
+      <c r="BH23" t="inlineStr"/>
+      <c r="BI23" t="inlineStr"/>
+      <c r="BJ23" t="inlineStr"/>
+      <c r="BK23" t="inlineStr"/>
+      <c r="BL23" t="inlineStr"/>
+      <c r="BM23" t="inlineStr"/>
+      <c r="BN23" t="inlineStr"/>
+      <c r="BO23" t="inlineStr"/>
+      <c r="BP23" t="inlineStr"/>
+      <c r="BQ23" t="inlineStr"/>
+      <c r="BR23" t="inlineStr"/>
+      <c r="BS23" t="inlineStr"/>
+      <c r="BT23" t="inlineStr"/>
+      <c r="BU23" t="inlineStr"/>
+      <c r="BV23" t="inlineStr"/>
+      <c r="BW23" t="inlineStr"/>
+      <c r="BX23" t="inlineStr"/>
+      <c r="BY23" t="inlineStr"/>
+      <c r="BZ23" t="inlineStr"/>
+      <c r="CA23" t="inlineStr"/>
+      <c r="CB23" t="inlineStr"/>
+      <c r="CC23" t="inlineStr"/>
+      <c r="CD23" t="inlineStr"/>
+      <c r="CE23" t="inlineStr"/>
+      <c r="CF23" t="inlineStr"/>
+      <c r="CG23" t="inlineStr"/>
+      <c r="CH23" t="inlineStr"/>
+      <c r="CI23" t="inlineStr"/>
+      <c r="CJ23" t="inlineStr"/>
+      <c r="CK23" t="inlineStr"/>
+      <c r="CL23" t="inlineStr"/>
+      <c r="CM23" t="inlineStr"/>
+      <c r="CN23" t="inlineStr"/>
+      <c r="CO23" t="inlineStr"/>
+      <c r="CP23" t="inlineStr"/>
+      <c r="CQ23" t="inlineStr"/>
+      <c r="CR23" t="inlineStr"/>
+      <c r="CS23" t="inlineStr"/>
+      <c r="CT23" t="inlineStr"/>
+      <c r="CU23" t="inlineStr"/>
+      <c r="CV23" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW23" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX23" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY23" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ23" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA23" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB23" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC23" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD23" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE23" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF23" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG23" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH23" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI23" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ23" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK23" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL23" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM23" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN23" t="inlineStr"/>
+      <c r="DO23" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP23" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ23" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR23" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS23" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT23" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU23" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV23" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW23" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX23" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY23" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ23" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA23" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB23" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC23" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED23" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE23" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF23" t="inlineStr"/>
+      <c r="EG23" t="inlineStr"/>
+      <c r="EH23" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI23" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ23" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK23" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>08/06/2026, 14:30:41</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>84</v>
+      </c>
+      <c r="D24" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E24" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="n">
+        <v>0</v>
+      </c>
+      <c r="J24" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L24" t="n">
+        <v>408</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O24" t="n">
+        <v>408</v>
+      </c>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q24" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R24" t="n">
+        <v>1780939335</v>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>08/06/2026 14:22</t>
+        </is>
+      </c>
+      <c r="V24" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W24" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X24" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y24" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z24" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA24" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE24" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH24" t="inlineStr"/>
+      <c r="AI24" t="inlineStr"/>
+      <c r="AJ24" t="inlineStr"/>
+      <c r="AK24" t="inlineStr"/>
+      <c r="AL24" t="inlineStr"/>
+      <c r="AM24" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP24" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ24" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR24" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT24" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU24" t="inlineStr"/>
+      <c r="AV24" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW24" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY24" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ24" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA24" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB24" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC24" t="inlineStr"/>
+      <c r="BD24" t="inlineStr"/>
+      <c r="BE24" t="inlineStr"/>
+      <c r="BF24" t="inlineStr"/>
+      <c r="BG24" t="inlineStr"/>
+      <c r="BH24" t="inlineStr"/>
+      <c r="BI24" t="inlineStr"/>
+      <c r="BJ24" t="inlineStr"/>
+      <c r="BK24" t="inlineStr"/>
+      <c r="BL24" t="inlineStr"/>
+      <c r="BM24" t="inlineStr"/>
+      <c r="BN24" t="inlineStr"/>
+      <c r="BO24" t="inlineStr"/>
+      <c r="BP24" t="inlineStr"/>
+      <c r="BQ24" t="inlineStr"/>
+      <c r="BR24" t="inlineStr"/>
+      <c r="BS24" t="inlineStr"/>
+      <c r="BT24" t="inlineStr"/>
+      <c r="BU24" t="inlineStr"/>
+      <c r="BV24" t="inlineStr"/>
+      <c r="BW24" t="inlineStr"/>
+      <c r="BX24" t="inlineStr"/>
+      <c r="BY24" t="inlineStr"/>
+      <c r="BZ24" t="inlineStr"/>
+      <c r="CA24" t="inlineStr"/>
+      <c r="CB24" t="inlineStr"/>
+      <c r="CC24" t="inlineStr"/>
+      <c r="CD24" t="inlineStr"/>
+      <c r="CE24" t="inlineStr"/>
+      <c r="CF24" t="inlineStr"/>
+      <c r="CG24" t="inlineStr"/>
+      <c r="CH24" t="inlineStr"/>
+      <c r="CI24" t="inlineStr"/>
+      <c r="CJ24" t="inlineStr"/>
+      <c r="CK24" t="inlineStr"/>
+      <c r="CL24" t="inlineStr"/>
+      <c r="CM24" t="inlineStr"/>
+      <c r="CN24" t="inlineStr"/>
+      <c r="CO24" t="inlineStr"/>
+      <c r="CP24" t="inlineStr"/>
+      <c r="CQ24" t="inlineStr"/>
+      <c r="CR24" t="inlineStr"/>
+      <c r="CS24" t="inlineStr"/>
+      <c r="CT24" t="inlineStr"/>
+      <c r="CU24" t="inlineStr"/>
+      <c r="CV24" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW24" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX24" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY24" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ24" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA24" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB24" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC24" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD24" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE24" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF24" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG24" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH24" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI24" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ24" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK24" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL24" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM24" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN24" t="inlineStr"/>
+      <c r="DO24" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP24" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ24" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR24" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS24" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT24" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU24" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV24" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW24" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX24" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY24" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ24" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA24" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB24" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC24" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED24" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE24" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF24" t="inlineStr"/>
+      <c r="EG24" t="inlineStr"/>
+      <c r="EH24" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI24" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ24" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK24" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>08/06/2026, 14:38:09</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>84</v>
+      </c>
+      <c r="D25" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E25" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F25" t="n">
+        <v>1</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J25" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L25" t="n">
+        <v>408</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O25" t="n">
+        <v>408</v>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q25" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R25" t="n">
+        <v>1780939784</v>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>14:29</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>08/06/2026 14:29</t>
+        </is>
+      </c>
+      <c r="V25" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W25" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X25" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y25" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z25" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA25" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE25" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH25" t="inlineStr"/>
+      <c r="AI25" t="inlineStr"/>
+      <c r="AJ25" t="inlineStr"/>
+      <c r="AK25" t="inlineStr"/>
+      <c r="AL25" t="inlineStr"/>
+      <c r="AM25" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP25" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ25" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR25" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT25" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU25" t="inlineStr"/>
+      <c r="AV25" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW25" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY25" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ25" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA25" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB25" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC25" t="inlineStr"/>
+      <c r="BD25" t="inlineStr"/>
+      <c r="BE25" t="inlineStr"/>
+      <c r="BF25" t="inlineStr"/>
+      <c r="BG25" t="inlineStr"/>
+      <c r="BH25" t="inlineStr"/>
+      <c r="BI25" t="inlineStr"/>
+      <c r="BJ25" t="inlineStr"/>
+      <c r="BK25" t="inlineStr"/>
+      <c r="BL25" t="inlineStr"/>
+      <c r="BM25" t="inlineStr"/>
+      <c r="BN25" t="inlineStr"/>
+      <c r="BO25" t="inlineStr"/>
+      <c r="BP25" t="inlineStr"/>
+      <c r="BQ25" t="inlineStr"/>
+      <c r="BR25" t="inlineStr"/>
+      <c r="BS25" t="inlineStr"/>
+      <c r="BT25" t="inlineStr"/>
+      <c r="BU25" t="inlineStr"/>
+      <c r="BV25" t="inlineStr"/>
+      <c r="BW25" t="inlineStr"/>
+      <c r="BX25" t="inlineStr"/>
+      <c r="BY25" t="inlineStr"/>
+      <c r="BZ25" t="inlineStr"/>
+      <c r="CA25" t="inlineStr"/>
+      <c r="CB25" t="inlineStr"/>
+      <c r="CC25" t="inlineStr"/>
+      <c r="CD25" t="inlineStr"/>
+      <c r="CE25" t="inlineStr"/>
+      <c r="CF25" t="inlineStr"/>
+      <c r="CG25" t="inlineStr"/>
+      <c r="CH25" t="inlineStr"/>
+      <c r="CI25" t="inlineStr"/>
+      <c r="CJ25" t="inlineStr"/>
+      <c r="CK25" t="inlineStr"/>
+      <c r="CL25" t="inlineStr"/>
+      <c r="CM25" t="inlineStr"/>
+      <c r="CN25" t="inlineStr"/>
+      <c r="CO25" t="inlineStr"/>
+      <c r="CP25" t="inlineStr"/>
+      <c r="CQ25" t="inlineStr"/>
+      <c r="CR25" t="inlineStr"/>
+      <c r="CS25" t="inlineStr"/>
+      <c r="CT25" t="inlineStr"/>
+      <c r="CU25" t="inlineStr"/>
+      <c r="CV25" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW25" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX25" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY25" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ25" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA25" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB25" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC25" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD25" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE25" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF25" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG25" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH25" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI25" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ25" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK25" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL25" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM25" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN25" t="inlineStr"/>
+      <c r="DO25" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP25" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ25" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR25" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS25" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT25" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU25" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV25" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW25" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX25" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY25" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ25" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA25" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB25" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC25" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED25" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE25" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF25" t="inlineStr"/>
+      <c r="EG25" t="inlineStr"/>
+      <c r="EH25" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI25" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ25" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK25" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>08/06/2026, 14:45:04</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1780887600</t>
+        </is>
+      </c>
+      <c r="R26" t="inlineStr">
+        <is>
+          <t>1780940198</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>08/06/2026 14:36</t>
+        </is>
+      </c>
+      <c r="V26" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W26" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X26" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y26" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA26" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB26" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC26" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH26" t="inlineStr"/>
+      <c r="AI26" t="inlineStr"/>
+      <c r="AJ26" t="inlineStr"/>
+      <c r="AK26" t="inlineStr"/>
+      <c r="AL26" t="inlineStr"/>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP26" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ26" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR26" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT26" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU26" t="inlineStr"/>
+      <c r="AV26" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW26" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY26" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ26" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA26" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB26" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC26" t="inlineStr"/>
+      <c r="BD26" t="inlineStr"/>
+      <c r="BE26" t="inlineStr"/>
+      <c r="BF26" t="inlineStr"/>
+      <c r="BG26" t="inlineStr"/>
+      <c r="BH26" t="inlineStr"/>
+      <c r="BI26" t="inlineStr"/>
+      <c r="BJ26" t="inlineStr"/>
+      <c r="BK26" t="inlineStr"/>
+      <c r="BL26" t="inlineStr"/>
+      <c r="BM26" t="inlineStr"/>
+      <c r="BN26" t="inlineStr"/>
+      <c r="BO26" t="inlineStr"/>
+      <c r="BP26" t="inlineStr"/>
+      <c r="BQ26" t="inlineStr"/>
+      <c r="BR26" t="inlineStr"/>
+      <c r="BS26" t="inlineStr"/>
+      <c r="BT26" t="inlineStr"/>
+      <c r="BU26" t="inlineStr"/>
+      <c r="BV26" t="inlineStr"/>
+      <c r="BW26" t="inlineStr"/>
+      <c r="BX26" t="inlineStr"/>
+      <c r="BY26" t="inlineStr"/>
+      <c r="BZ26" t="inlineStr"/>
+      <c r="CA26" t="inlineStr"/>
+      <c r="CB26" t="inlineStr"/>
+      <c r="CC26" t="inlineStr"/>
+      <c r="CD26" t="inlineStr"/>
+      <c r="CE26" t="inlineStr"/>
+      <c r="CF26" t="inlineStr"/>
+      <c r="CG26" t="inlineStr"/>
+      <c r="CH26" t="inlineStr"/>
+      <c r="CI26" t="inlineStr"/>
+      <c r="CJ26" t="inlineStr"/>
+      <c r="CK26" t="inlineStr"/>
+      <c r="CL26" t="inlineStr"/>
+      <c r="CM26" t="inlineStr"/>
+      <c r="CN26" t="inlineStr"/>
+      <c r="CO26" t="inlineStr"/>
+      <c r="CP26" t="inlineStr"/>
+      <c r="CQ26" t="inlineStr"/>
+      <c r="CR26" t="inlineStr"/>
+      <c r="CS26" t="inlineStr"/>
+      <c r="CT26" t="inlineStr"/>
+      <c r="CU26" t="inlineStr"/>
+      <c r="CV26" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW26" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX26" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY26" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ26" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA26" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB26" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC26" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD26" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE26" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF26" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG26" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH26" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI26" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ26" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK26" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL26" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM26" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN26" t="inlineStr"/>
+      <c r="DO26" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP26" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ26" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR26" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS26" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT26" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU26" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV26" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW26" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX26" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY26" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ26" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA26" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB26" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC26" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED26" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE26" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF26" t="inlineStr"/>
+      <c r="EG26" t="inlineStr"/>
+      <c r="EH26" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI26" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ26" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK26" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL26" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9005,13 +12493,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2E5362F9-87DC-4D00-AC6A-0D4FA0E11BC8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B6294CC-8429-4C63-A44E-44A628E2ACE5}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{60550303-CF0E-48C3-9117-6FA69E4BED68}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{311BAE5D-3F8F-438D-BB80-DF8E8CD7C837}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6F51F449-F139-4018-8D77-64162D58004A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{6A122744-7312-4534-8A32-66E24F2B507E}"/>
 </file>
</xml_diff>

<commit_message>
Update `modelo_contrato.html` with enhanced print styles and layout refinements
- Introduce A4 page setup for print compatibility.
- Add footer with firm contact details.
- Refactor CSS for layout consistency and improved page break handling.
- Update `dados_formulario_atual.json` with new extraction timestamps and formatted data.
- Modify linked data files (`dados_formularios.xlsx`, `Contrato_alex_de_Niterói.pdf`).
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL37"/>
+  <dimension ref="A1:EL38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16583,47 +16583,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E37" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C37" t="n">
+        <v>84</v>
+      </c>
+      <c r="D37" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E37" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
       </c>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
-      <c r="I37" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I37" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" t="n">
+        <v>22133</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L37" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L37" t="n">
+        <v>408</v>
       </c>
       <c r="M37" t="inlineStr">
         <is>
@@ -16635,25 +16621,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O37" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O37" t="n">
+        <v>408</v>
       </c>
       <c r="P37" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q37" t="inlineStr">
-        <is>
-          <t>1780887600</t>
-        </is>
-      </c>
-      <c r="R37" t="inlineStr">
-        <is>
-          <t>1780946198</t>
-        </is>
+      <c r="Q37" t="n">
+        <v>1780887600</v>
+      </c>
+      <c r="R37" t="n">
+        <v>1780946198</v>
       </c>
       <c r="S37" t="inlineStr">
         <is>
@@ -16675,10 +16655,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W37" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W37" t="n">
+        <v>22133</v>
       </c>
       <c r="X37" t="inlineStr">
         <is>
@@ -16690,35 +16668,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z37" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z37" t="n">
+        <v>127857</v>
       </c>
       <c r="AA37" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB37" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC37" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB37" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC37" t="n">
+        <v>487</v>
       </c>
       <c r="AD37" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE37" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE37" t="n">
+        <v>121</v>
       </c>
       <c r="AF37" t="inlineStr">
         <is>
@@ -16735,10 +16705,8 @@
       <c r="AJ37" t="inlineStr"/>
       <c r="AK37" t="inlineStr"/>
       <c r="AL37" t="inlineStr"/>
-      <c r="AM37" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM37" t="n">
+        <v>127857</v>
       </c>
       <c r="AN37" t="inlineStr">
         <is>
@@ -16770,10 +16738,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT37" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT37" t="n">
+        <v>3500</v>
       </c>
       <c r="AU37" t="inlineStr"/>
       <c r="AV37" t="inlineStr">
@@ -16901,10 +16867,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE37" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE37" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF37" t="inlineStr">
         <is>
@@ -16921,15 +16885,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI37" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ37" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI37" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ37" t="n">
+        <v>12344</v>
       </c>
       <c r="DK37" t="inlineStr">
         <is>
@@ -16941,10 +16901,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM37" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM37" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN37" t="inlineStr"/>
       <c r="DO37" t="inlineStr">
@@ -16962,15 +16920,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR37" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS37" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR37" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS37" t="n">
+        <v>3144</v>
       </c>
       <c r="DT37" t="inlineStr">
         <is>
@@ -16987,10 +16941,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW37" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW37" t="n">
+        <v>124</v>
       </c>
       <c r="DX37" t="inlineStr">
         <is>
@@ -17055,6 +17007,490 @@
         </is>
       </c>
       <c r="EL37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>08/06/2026, 16:41:31</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>1780887600</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr">
+        <is>
+          <t>1780947185</t>
+        </is>
+      </c>
+      <c r="S38" t="inlineStr">
+        <is>
+          <t>08/06/2026</t>
+        </is>
+      </c>
+      <c r="T38" t="inlineStr">
+        <is>
+          <t>16:33</t>
+        </is>
+      </c>
+      <c r="U38" t="inlineStr">
+        <is>
+          <t>08/06/2026 16:33</t>
+        </is>
+      </c>
+      <c r="V38" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W38" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X38" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y38" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z38" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA38" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB38" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC38" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD38" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE38" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF38" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG38" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH38" t="inlineStr"/>
+      <c r="AI38" t="inlineStr"/>
+      <c r="AJ38" t="inlineStr"/>
+      <c r="AK38" t="inlineStr"/>
+      <c r="AL38" t="inlineStr"/>
+      <c r="AM38" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN38" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO38" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP38" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ38" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR38" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS38" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT38" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU38" t="inlineStr"/>
+      <c r="AV38" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW38" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX38" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY38" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ38" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA38" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB38" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC38" t="inlineStr"/>
+      <c r="BD38" t="inlineStr"/>
+      <c r="BE38" t="inlineStr"/>
+      <c r="BF38" t="inlineStr"/>
+      <c r="BG38" t="inlineStr"/>
+      <c r="BH38" t="inlineStr"/>
+      <c r="BI38" t="inlineStr"/>
+      <c r="BJ38" t="inlineStr"/>
+      <c r="BK38" t="inlineStr"/>
+      <c r="BL38" t="inlineStr"/>
+      <c r="BM38" t="inlineStr"/>
+      <c r="BN38" t="inlineStr"/>
+      <c r="BO38" t="inlineStr"/>
+      <c r="BP38" t="inlineStr"/>
+      <c r="BQ38" t="inlineStr"/>
+      <c r="BR38" t="inlineStr"/>
+      <c r="BS38" t="inlineStr"/>
+      <c r="BT38" t="inlineStr"/>
+      <c r="BU38" t="inlineStr"/>
+      <c r="BV38" t="inlineStr"/>
+      <c r="BW38" t="inlineStr"/>
+      <c r="BX38" t="inlineStr"/>
+      <c r="BY38" t="inlineStr"/>
+      <c r="BZ38" t="inlineStr"/>
+      <c r="CA38" t="inlineStr"/>
+      <c r="CB38" t="inlineStr"/>
+      <c r="CC38" t="inlineStr"/>
+      <c r="CD38" t="inlineStr"/>
+      <c r="CE38" t="inlineStr"/>
+      <c r="CF38" t="inlineStr"/>
+      <c r="CG38" t="inlineStr"/>
+      <c r="CH38" t="inlineStr"/>
+      <c r="CI38" t="inlineStr"/>
+      <c r="CJ38" t="inlineStr"/>
+      <c r="CK38" t="inlineStr"/>
+      <c r="CL38" t="inlineStr"/>
+      <c r="CM38" t="inlineStr"/>
+      <c r="CN38" t="inlineStr"/>
+      <c r="CO38" t="inlineStr"/>
+      <c r="CP38" t="inlineStr"/>
+      <c r="CQ38" t="inlineStr"/>
+      <c r="CR38" t="inlineStr"/>
+      <c r="CS38" t="inlineStr"/>
+      <c r="CT38" t="inlineStr"/>
+      <c r="CU38" t="inlineStr"/>
+      <c r="CV38" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW38" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX38" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY38" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ38" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA38" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB38" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC38" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD38" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE38" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF38" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG38" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH38" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI38" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ38" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK38" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL38" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM38" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN38" t="inlineStr"/>
+      <c r="DO38" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP38" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ38" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR38" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS38" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT38" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU38" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV38" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW38" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX38" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY38" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ38" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA38" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB38" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC38" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED38" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE38" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF38" t="inlineStr"/>
+      <c r="EG38" t="inlineStr"/>
+      <c r="EH38" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI38" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ38" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK38" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL38" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -17289,13 +17725,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EE751E45-8382-40E1-801A-0A2FC209627A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9162617-93AF-40BB-9DCB-EBC8E391BA75}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{55EDDF23-E659-4E27-95CB-CE6FF0CB7BA8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78CF7E72-26DD-410D-9C19-B1F12050467C}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{470B21B9-7EA8-4B86-B102-AA8A96485515}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BED12907-72DE-4F09-AD72-39393081ED76}"/>
 </file>
</xml_diff>

<commit_message>
Remove unused `modelo_contrato.txt` file
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL51"/>
+  <dimension ref="A1:EL59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -22687,47 +22687,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>84</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>01210000010</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C51" t="n">
+        <v>84</v>
+      </c>
+      <c r="D51" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E51" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
       </c>
       <c r="G51" t="inlineStr"/>
       <c r="H51" t="inlineStr"/>
-      <c r="I51" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J51" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="I51" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" t="n">
+        <v>22133</v>
       </c>
       <c r="K51" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L51" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L51" t="n">
+        <v>408</v>
       </c>
       <c r="M51" t="inlineStr">
         <is>
@@ -22739,25 +22725,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O51" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O51" t="n">
+        <v>408</v>
       </c>
       <c r="P51" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q51" t="inlineStr">
-        <is>
-          <t>1780974000</t>
-        </is>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>1781053687</t>
-        </is>
+      <c r="Q51" t="n">
+        <v>1780974000</v>
+      </c>
+      <c r="R51" t="n">
+        <v>1781053687</v>
       </c>
       <c r="S51" t="inlineStr">
         <is>
@@ -22779,10 +22759,8 @@
           <t>03/06/2026 17:13</t>
         </is>
       </c>
-      <c r="W51" t="inlineStr">
-        <is>
-          <t>22133</t>
-        </is>
+      <c r="W51" t="n">
+        <v>22133</v>
       </c>
       <c r="X51" t="inlineStr">
         <is>
@@ -22794,35 +22772,27 @@
           <t>04/06/2026 17:25</t>
         </is>
       </c>
-      <c r="Z51" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="Z51" t="n">
+        <v>127857</v>
       </c>
       <c r="AA51" t="inlineStr">
         <is>
           <t>08 - Confecção e assinatura (Contrato)</t>
         </is>
       </c>
-      <c r="AB51" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC51" t="inlineStr">
-        <is>
-          <t>487</t>
-        </is>
+      <c r="AB51" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC51" t="n">
+        <v>487</v>
       </c>
       <c r="AD51" t="inlineStr">
         <is>
           <t>Pedro Santana</t>
         </is>
       </c>
-      <c r="AE51" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE51" t="n">
+        <v>121</v>
       </c>
       <c r="AF51" t="inlineStr">
         <is>
@@ -22839,10 +22809,8 @@
       <c r="AJ51" t="inlineStr"/>
       <c r="AK51" t="inlineStr"/>
       <c r="AL51" t="inlineStr"/>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t>127857</t>
-        </is>
+      <c r="AM51" t="n">
+        <v>127857</v>
       </c>
       <c r="AN51" t="inlineStr">
         <is>
@@ -22874,10 +22842,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT51" t="inlineStr">
-        <is>
-          <t>3500.00</t>
-        </is>
+      <c r="AT51" t="n">
+        <v>3500</v>
       </c>
       <c r="AU51" t="inlineStr"/>
       <c r="AV51" t="inlineStr">
@@ -23005,10 +22971,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE51" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE51" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF51" t="inlineStr">
         <is>
@@ -23025,15 +22989,11 @@
           <t>Namorado(a)</t>
         </is>
       </c>
-      <c r="DI51" t="inlineStr">
-        <is>
-          <t>212122</t>
-        </is>
-      </c>
-      <c r="DJ51" t="inlineStr">
-        <is>
-          <t>12344</t>
-        </is>
+      <c r="DI51" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ51" t="n">
+        <v>12344</v>
       </c>
       <c r="DK51" t="inlineStr">
         <is>
@@ -23045,10 +23005,8 @@
           <t>pedro.santana@folhatech.com.br</t>
         </is>
       </c>
-      <c r="DM51" t="inlineStr">
-        <is>
-          <t>121212212112</t>
-        </is>
+      <c r="DM51" t="n">
+        <v>121212212112</v>
       </c>
       <c r="DN51" t="inlineStr"/>
       <c r="DO51" t="inlineStr">
@@ -23066,15 +23024,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR51" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS51" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR51" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS51" t="n">
+        <v>3144</v>
       </c>
       <c r="DT51" t="inlineStr">
         <is>
@@ -23091,10 +23045,8 @@
           <t>etetetet</t>
         </is>
       </c>
-      <c r="DW51" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW51" t="n">
+        <v>124</v>
       </c>
       <c r="DX51" t="inlineStr">
         <is>
@@ -23159,6 +23111,3542 @@
         </is>
       </c>
       <c r="EL51" t="inlineStr"/>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>10/06/2026, 08:48:09</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C52" t="n">
+        <v>84</v>
+      </c>
+      <c r="D52" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E52" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F52" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="n">
+        <v>0</v>
+      </c>
+      <c r="J52" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L52" t="n">
+        <v>408</v>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O52" t="n">
+        <v>408</v>
+      </c>
+      <c r="P52" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q52" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R52" t="n">
+        <v>1781091571</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>08:39</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>10/06/2026 08:39</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W52" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X52" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y52" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z52" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA52" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB52" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC52" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD52" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE52" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF52" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG52" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH52" t="inlineStr"/>
+      <c r="AI52" t="inlineStr"/>
+      <c r="AJ52" t="inlineStr"/>
+      <c r="AK52" t="inlineStr"/>
+      <c r="AL52" t="inlineStr"/>
+      <c r="AM52" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN52" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO52" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP52" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ52" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR52" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS52" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT52" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU52" t="inlineStr"/>
+      <c r="AV52" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW52" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX52" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY52" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ52" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA52" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB52" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC52" t="inlineStr"/>
+      <c r="BD52" t="inlineStr"/>
+      <c r="BE52" t="inlineStr"/>
+      <c r="BF52" t="inlineStr"/>
+      <c r="BG52" t="inlineStr"/>
+      <c r="BH52" t="inlineStr"/>
+      <c r="BI52" t="inlineStr"/>
+      <c r="BJ52" t="inlineStr"/>
+      <c r="BK52" t="inlineStr"/>
+      <c r="BL52" t="inlineStr"/>
+      <c r="BM52" t="inlineStr"/>
+      <c r="BN52" t="inlineStr"/>
+      <c r="BO52" t="inlineStr"/>
+      <c r="BP52" t="inlineStr"/>
+      <c r="BQ52" t="inlineStr"/>
+      <c r="BR52" t="inlineStr"/>
+      <c r="BS52" t="inlineStr"/>
+      <c r="BT52" t="inlineStr"/>
+      <c r="BU52" t="inlineStr"/>
+      <c r="BV52" t="inlineStr"/>
+      <c r="BW52" t="inlineStr"/>
+      <c r="BX52" t="inlineStr"/>
+      <c r="BY52" t="inlineStr"/>
+      <c r="BZ52" t="inlineStr"/>
+      <c r="CA52" t="inlineStr"/>
+      <c r="CB52" t="inlineStr"/>
+      <c r="CC52" t="inlineStr"/>
+      <c r="CD52" t="inlineStr"/>
+      <c r="CE52" t="inlineStr"/>
+      <c r="CF52" t="inlineStr"/>
+      <c r="CG52" t="inlineStr"/>
+      <c r="CH52" t="inlineStr"/>
+      <c r="CI52" t="inlineStr"/>
+      <c r="CJ52" t="inlineStr"/>
+      <c r="CK52" t="inlineStr"/>
+      <c r="CL52" t="inlineStr"/>
+      <c r="CM52" t="inlineStr"/>
+      <c r="CN52" t="inlineStr"/>
+      <c r="CO52" t="inlineStr"/>
+      <c r="CP52" t="inlineStr"/>
+      <c r="CQ52" t="inlineStr"/>
+      <c r="CR52" t="inlineStr"/>
+      <c r="CS52" t="inlineStr"/>
+      <c r="CT52" t="inlineStr"/>
+      <c r="CU52" t="inlineStr"/>
+      <c r="CV52" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW52" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX52" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY52" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ52" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA52" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB52" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC52" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD52" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE52" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF52" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG52" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH52" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI52" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ52" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK52" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL52" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM52" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN52" t="inlineStr"/>
+      <c r="DO52" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP52" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ52" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR52" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS52" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT52" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU52" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV52" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW52" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX52" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY52" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ52" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA52" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB52" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC52" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED52" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE52" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF52" t="inlineStr"/>
+      <c r="EG52" t="inlineStr"/>
+      <c r="EH52" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI52" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ52" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK52" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL52" t="inlineStr"/>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>10/06/2026, 08:52:40</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C53" t="n">
+        <v>84</v>
+      </c>
+      <c r="D53" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E53" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="n">
+        <v>0</v>
+      </c>
+      <c r="J53" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L53" t="n">
+        <v>408</v>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O53" t="n">
+        <v>408</v>
+      </c>
+      <c r="P53" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q53" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R53" t="n">
+        <v>1781091842</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>08:44</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>10/06/2026 08:44</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W53" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X53" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y53" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z53" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA53" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB53" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC53" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD53" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE53" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF53" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG53" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH53" t="inlineStr"/>
+      <c r="AI53" t="inlineStr"/>
+      <c r="AJ53" t="inlineStr"/>
+      <c r="AK53" t="inlineStr"/>
+      <c r="AL53" t="inlineStr"/>
+      <c r="AM53" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN53" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO53" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP53" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ53" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR53" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS53" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT53" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU53" t="inlineStr"/>
+      <c r="AV53" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW53" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX53" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY53" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ53" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA53" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB53" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC53" t="inlineStr"/>
+      <c r="BD53" t="inlineStr"/>
+      <c r="BE53" t="inlineStr"/>
+      <c r="BF53" t="inlineStr"/>
+      <c r="BG53" t="inlineStr"/>
+      <c r="BH53" t="inlineStr"/>
+      <c r="BI53" t="inlineStr"/>
+      <c r="BJ53" t="inlineStr"/>
+      <c r="BK53" t="inlineStr"/>
+      <c r="BL53" t="inlineStr"/>
+      <c r="BM53" t="inlineStr"/>
+      <c r="BN53" t="inlineStr"/>
+      <c r="BO53" t="inlineStr"/>
+      <c r="BP53" t="inlineStr"/>
+      <c r="BQ53" t="inlineStr"/>
+      <c r="BR53" t="inlineStr"/>
+      <c r="BS53" t="inlineStr"/>
+      <c r="BT53" t="inlineStr"/>
+      <c r="BU53" t="inlineStr"/>
+      <c r="BV53" t="inlineStr"/>
+      <c r="BW53" t="inlineStr"/>
+      <c r="BX53" t="inlineStr"/>
+      <c r="BY53" t="inlineStr"/>
+      <c r="BZ53" t="inlineStr"/>
+      <c r="CA53" t="inlineStr"/>
+      <c r="CB53" t="inlineStr"/>
+      <c r="CC53" t="inlineStr"/>
+      <c r="CD53" t="inlineStr"/>
+      <c r="CE53" t="inlineStr"/>
+      <c r="CF53" t="inlineStr"/>
+      <c r="CG53" t="inlineStr"/>
+      <c r="CH53" t="inlineStr"/>
+      <c r="CI53" t="inlineStr"/>
+      <c r="CJ53" t="inlineStr"/>
+      <c r="CK53" t="inlineStr"/>
+      <c r="CL53" t="inlineStr"/>
+      <c r="CM53" t="inlineStr"/>
+      <c r="CN53" t="inlineStr"/>
+      <c r="CO53" t="inlineStr"/>
+      <c r="CP53" t="inlineStr"/>
+      <c r="CQ53" t="inlineStr"/>
+      <c r="CR53" t="inlineStr"/>
+      <c r="CS53" t="inlineStr"/>
+      <c r="CT53" t="inlineStr"/>
+      <c r="CU53" t="inlineStr"/>
+      <c r="CV53" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW53" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX53" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY53" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ53" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA53" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB53" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC53" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD53" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE53" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF53" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG53" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH53" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI53" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ53" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK53" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL53" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM53" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN53" t="inlineStr"/>
+      <c r="DO53" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP53" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ53" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR53" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS53" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT53" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU53" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV53" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW53" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX53" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY53" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ53" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA53" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB53" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC53" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED53" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE53" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF53" t="inlineStr"/>
+      <c r="EG53" t="inlineStr"/>
+      <c r="EH53" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI53" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ53" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK53" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL53" t="inlineStr"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:08:41</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C54" t="n">
+        <v>84</v>
+      </c>
+      <c r="D54" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E54" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="n">
+        <v>0</v>
+      </c>
+      <c r="J54" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L54" t="n">
+        <v>408</v>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O54" t="n">
+        <v>408</v>
+      </c>
+      <c r="P54" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q54" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R54" t="n">
+        <v>1781092803</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:00</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W54" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X54" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y54" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z54" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA54" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB54" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC54" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD54" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE54" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF54" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG54" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH54" t="inlineStr"/>
+      <c r="AI54" t="inlineStr"/>
+      <c r="AJ54" t="inlineStr"/>
+      <c r="AK54" t="inlineStr"/>
+      <c r="AL54" t="inlineStr"/>
+      <c r="AM54" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN54" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO54" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP54" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ54" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR54" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS54" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT54" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU54" t="inlineStr"/>
+      <c r="AV54" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW54" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX54" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY54" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ54" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA54" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB54" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC54" t="inlineStr"/>
+      <c r="BD54" t="inlineStr"/>
+      <c r="BE54" t="inlineStr"/>
+      <c r="BF54" t="inlineStr"/>
+      <c r="BG54" t="inlineStr"/>
+      <c r="BH54" t="inlineStr"/>
+      <c r="BI54" t="inlineStr"/>
+      <c r="BJ54" t="inlineStr"/>
+      <c r="BK54" t="inlineStr"/>
+      <c r="BL54" t="inlineStr"/>
+      <c r="BM54" t="inlineStr"/>
+      <c r="BN54" t="inlineStr"/>
+      <c r="BO54" t="inlineStr"/>
+      <c r="BP54" t="inlineStr"/>
+      <c r="BQ54" t="inlineStr"/>
+      <c r="BR54" t="inlineStr"/>
+      <c r="BS54" t="inlineStr"/>
+      <c r="BT54" t="inlineStr"/>
+      <c r="BU54" t="inlineStr"/>
+      <c r="BV54" t="inlineStr"/>
+      <c r="BW54" t="inlineStr"/>
+      <c r="BX54" t="inlineStr"/>
+      <c r="BY54" t="inlineStr"/>
+      <c r="BZ54" t="inlineStr"/>
+      <c r="CA54" t="inlineStr"/>
+      <c r="CB54" t="inlineStr"/>
+      <c r="CC54" t="inlineStr"/>
+      <c r="CD54" t="inlineStr"/>
+      <c r="CE54" t="inlineStr"/>
+      <c r="CF54" t="inlineStr"/>
+      <c r="CG54" t="inlineStr"/>
+      <c r="CH54" t="inlineStr"/>
+      <c r="CI54" t="inlineStr"/>
+      <c r="CJ54" t="inlineStr"/>
+      <c r="CK54" t="inlineStr"/>
+      <c r="CL54" t="inlineStr"/>
+      <c r="CM54" t="inlineStr"/>
+      <c r="CN54" t="inlineStr"/>
+      <c r="CO54" t="inlineStr"/>
+      <c r="CP54" t="inlineStr"/>
+      <c r="CQ54" t="inlineStr"/>
+      <c r="CR54" t="inlineStr"/>
+      <c r="CS54" t="inlineStr"/>
+      <c r="CT54" t="inlineStr"/>
+      <c r="CU54" t="inlineStr"/>
+      <c r="CV54" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW54" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX54" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY54" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ54" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA54" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB54" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC54" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD54" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE54" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF54" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG54" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH54" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI54" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ54" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK54" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL54" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM54" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN54" t="inlineStr"/>
+      <c r="DO54" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP54" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ54" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR54" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS54" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT54" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU54" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV54" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW54" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX54" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY54" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ54" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA54" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB54" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC54" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED54" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE54" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF54" t="inlineStr"/>
+      <c r="EG54" t="inlineStr"/>
+      <c r="EH54" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI54" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ54" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK54" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL54" t="inlineStr"/>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:10:49</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C55" t="n">
+        <v>84</v>
+      </c>
+      <c r="D55" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E55" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="n">
+        <v>0</v>
+      </c>
+      <c r="J55" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L55" t="n">
+        <v>408</v>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O55" t="n">
+        <v>408</v>
+      </c>
+      <c r="P55" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q55" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R55" t="n">
+        <v>1781092931</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>09:02</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:02</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W55" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X55" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y55" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z55" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA55" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB55" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC55" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD55" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE55" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF55" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG55" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH55" t="inlineStr"/>
+      <c r="AI55" t="inlineStr"/>
+      <c r="AJ55" t="inlineStr"/>
+      <c r="AK55" t="inlineStr"/>
+      <c r="AL55" t="inlineStr"/>
+      <c r="AM55" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN55" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO55" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP55" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ55" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR55" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS55" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT55" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU55" t="inlineStr"/>
+      <c r="AV55" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW55" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX55" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY55" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ55" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA55" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB55" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC55" t="inlineStr"/>
+      <c r="BD55" t="inlineStr"/>
+      <c r="BE55" t="inlineStr"/>
+      <c r="BF55" t="inlineStr"/>
+      <c r="BG55" t="inlineStr"/>
+      <c r="BH55" t="inlineStr"/>
+      <c r="BI55" t="inlineStr"/>
+      <c r="BJ55" t="inlineStr"/>
+      <c r="BK55" t="inlineStr"/>
+      <c r="BL55" t="inlineStr"/>
+      <c r="BM55" t="inlineStr"/>
+      <c r="BN55" t="inlineStr"/>
+      <c r="BO55" t="inlineStr"/>
+      <c r="BP55" t="inlineStr"/>
+      <c r="BQ55" t="inlineStr"/>
+      <c r="BR55" t="inlineStr"/>
+      <c r="BS55" t="inlineStr"/>
+      <c r="BT55" t="inlineStr"/>
+      <c r="BU55" t="inlineStr"/>
+      <c r="BV55" t="inlineStr"/>
+      <c r="BW55" t="inlineStr"/>
+      <c r="BX55" t="inlineStr"/>
+      <c r="BY55" t="inlineStr"/>
+      <c r="BZ55" t="inlineStr"/>
+      <c r="CA55" t="inlineStr"/>
+      <c r="CB55" t="inlineStr"/>
+      <c r="CC55" t="inlineStr"/>
+      <c r="CD55" t="inlineStr"/>
+      <c r="CE55" t="inlineStr"/>
+      <c r="CF55" t="inlineStr"/>
+      <c r="CG55" t="inlineStr"/>
+      <c r="CH55" t="inlineStr"/>
+      <c r="CI55" t="inlineStr"/>
+      <c r="CJ55" t="inlineStr"/>
+      <c r="CK55" t="inlineStr"/>
+      <c r="CL55" t="inlineStr"/>
+      <c r="CM55" t="inlineStr"/>
+      <c r="CN55" t="inlineStr"/>
+      <c r="CO55" t="inlineStr"/>
+      <c r="CP55" t="inlineStr"/>
+      <c r="CQ55" t="inlineStr"/>
+      <c r="CR55" t="inlineStr"/>
+      <c r="CS55" t="inlineStr"/>
+      <c r="CT55" t="inlineStr"/>
+      <c r="CU55" t="inlineStr"/>
+      <c r="CV55" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW55" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX55" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY55" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ55" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA55" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB55" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC55" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD55" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE55" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF55" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG55" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH55" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI55" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ55" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK55" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL55" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM55" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN55" t="inlineStr"/>
+      <c r="DO55" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP55" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ55" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR55" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS55" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT55" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU55" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV55" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW55" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX55" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY55" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ55" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA55" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB55" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC55" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED55" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE55" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF55" t="inlineStr"/>
+      <c r="EG55" t="inlineStr"/>
+      <c r="EH55" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI55" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ55" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK55" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL55" t="inlineStr"/>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:19:19</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C56" t="n">
+        <v>84</v>
+      </c>
+      <c r="D56" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E56" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L56" t="n">
+        <v>408</v>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O56" t="n">
+        <v>408</v>
+      </c>
+      <c r="P56" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q56" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R56" t="n">
+        <v>1781093441</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>09:10</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:10</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W56" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X56" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y56" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z56" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA56" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB56" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC56" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD56" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE56" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF56" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG56" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH56" t="inlineStr"/>
+      <c r="AI56" t="inlineStr"/>
+      <c r="AJ56" t="inlineStr"/>
+      <c r="AK56" t="inlineStr"/>
+      <c r="AL56" t="inlineStr"/>
+      <c r="AM56" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN56" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO56" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP56" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ56" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR56" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS56" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT56" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU56" t="inlineStr"/>
+      <c r="AV56" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW56" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX56" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY56" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ56" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA56" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB56" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC56" t="inlineStr"/>
+      <c r="BD56" t="inlineStr"/>
+      <c r="BE56" t="inlineStr"/>
+      <c r="BF56" t="inlineStr"/>
+      <c r="BG56" t="inlineStr"/>
+      <c r="BH56" t="inlineStr"/>
+      <c r="BI56" t="inlineStr"/>
+      <c r="BJ56" t="inlineStr"/>
+      <c r="BK56" t="inlineStr"/>
+      <c r="BL56" t="inlineStr"/>
+      <c r="BM56" t="inlineStr"/>
+      <c r="BN56" t="inlineStr"/>
+      <c r="BO56" t="inlineStr"/>
+      <c r="BP56" t="inlineStr"/>
+      <c r="BQ56" t="inlineStr"/>
+      <c r="BR56" t="inlineStr"/>
+      <c r="BS56" t="inlineStr"/>
+      <c r="BT56" t="inlineStr"/>
+      <c r="BU56" t="inlineStr"/>
+      <c r="BV56" t="inlineStr"/>
+      <c r="BW56" t="inlineStr"/>
+      <c r="BX56" t="inlineStr"/>
+      <c r="BY56" t="inlineStr"/>
+      <c r="BZ56" t="inlineStr"/>
+      <c r="CA56" t="inlineStr"/>
+      <c r="CB56" t="inlineStr"/>
+      <c r="CC56" t="inlineStr"/>
+      <c r="CD56" t="inlineStr"/>
+      <c r="CE56" t="inlineStr"/>
+      <c r="CF56" t="inlineStr"/>
+      <c r="CG56" t="inlineStr"/>
+      <c r="CH56" t="inlineStr"/>
+      <c r="CI56" t="inlineStr"/>
+      <c r="CJ56" t="inlineStr"/>
+      <c r="CK56" t="inlineStr"/>
+      <c r="CL56" t="inlineStr"/>
+      <c r="CM56" t="inlineStr"/>
+      <c r="CN56" t="inlineStr"/>
+      <c r="CO56" t="inlineStr"/>
+      <c r="CP56" t="inlineStr"/>
+      <c r="CQ56" t="inlineStr"/>
+      <c r="CR56" t="inlineStr"/>
+      <c r="CS56" t="inlineStr"/>
+      <c r="CT56" t="inlineStr"/>
+      <c r="CU56" t="inlineStr"/>
+      <c r="CV56" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW56" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX56" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY56" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ56" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA56" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB56" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC56" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD56" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE56" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF56" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG56" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH56" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI56" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ56" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK56" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL56" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM56" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN56" t="inlineStr"/>
+      <c r="DO56" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP56" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ56" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR56" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS56" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT56" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU56" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV56" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW56" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX56" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY56" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ56" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA56" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB56" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC56" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED56" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE56" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF56" t="inlineStr"/>
+      <c r="EG56" t="inlineStr"/>
+      <c r="EH56" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI56" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ56" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK56" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL56" t="inlineStr"/>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:22:37</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C57" t="n">
+        <v>84</v>
+      </c>
+      <c r="D57" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E57" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L57" t="n">
+        <v>408</v>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O57" t="n">
+        <v>408</v>
+      </c>
+      <c r="P57" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q57" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R57" t="n">
+        <v>1781093639</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>09:13</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:13</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W57" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X57" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y57" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z57" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA57" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB57" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC57" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD57" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE57" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF57" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG57" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH57" t="inlineStr"/>
+      <c r="AI57" t="inlineStr"/>
+      <c r="AJ57" t="inlineStr"/>
+      <c r="AK57" t="inlineStr"/>
+      <c r="AL57" t="inlineStr"/>
+      <c r="AM57" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN57" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO57" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP57" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ57" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR57" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS57" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT57" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU57" t="inlineStr"/>
+      <c r="AV57" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW57" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX57" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY57" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ57" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA57" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB57" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC57" t="inlineStr"/>
+      <c r="BD57" t="inlineStr"/>
+      <c r="BE57" t="inlineStr"/>
+      <c r="BF57" t="inlineStr"/>
+      <c r="BG57" t="inlineStr"/>
+      <c r="BH57" t="inlineStr"/>
+      <c r="BI57" t="inlineStr"/>
+      <c r="BJ57" t="inlineStr"/>
+      <c r="BK57" t="inlineStr"/>
+      <c r="BL57" t="inlineStr"/>
+      <c r="BM57" t="inlineStr"/>
+      <c r="BN57" t="inlineStr"/>
+      <c r="BO57" t="inlineStr"/>
+      <c r="BP57" t="inlineStr"/>
+      <c r="BQ57" t="inlineStr"/>
+      <c r="BR57" t="inlineStr"/>
+      <c r="BS57" t="inlineStr"/>
+      <c r="BT57" t="inlineStr"/>
+      <c r="BU57" t="inlineStr"/>
+      <c r="BV57" t="inlineStr"/>
+      <c r="BW57" t="inlineStr"/>
+      <c r="BX57" t="inlineStr"/>
+      <c r="BY57" t="inlineStr"/>
+      <c r="BZ57" t="inlineStr"/>
+      <c r="CA57" t="inlineStr"/>
+      <c r="CB57" t="inlineStr"/>
+      <c r="CC57" t="inlineStr"/>
+      <c r="CD57" t="inlineStr"/>
+      <c r="CE57" t="inlineStr"/>
+      <c r="CF57" t="inlineStr"/>
+      <c r="CG57" t="inlineStr"/>
+      <c r="CH57" t="inlineStr"/>
+      <c r="CI57" t="inlineStr"/>
+      <c r="CJ57" t="inlineStr"/>
+      <c r="CK57" t="inlineStr"/>
+      <c r="CL57" t="inlineStr"/>
+      <c r="CM57" t="inlineStr"/>
+      <c r="CN57" t="inlineStr"/>
+      <c r="CO57" t="inlineStr"/>
+      <c r="CP57" t="inlineStr"/>
+      <c r="CQ57" t="inlineStr"/>
+      <c r="CR57" t="inlineStr"/>
+      <c r="CS57" t="inlineStr"/>
+      <c r="CT57" t="inlineStr"/>
+      <c r="CU57" t="inlineStr"/>
+      <c r="CV57" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW57" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX57" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY57" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ57" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA57" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB57" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC57" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD57" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE57" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF57" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG57" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH57" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI57" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ57" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK57" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL57" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM57" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN57" t="inlineStr"/>
+      <c r="DO57" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP57" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ57" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR57" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS57" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT57" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU57" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV57" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW57" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX57" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY57" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ57" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA57" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB57" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC57" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED57" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE57" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF57" t="inlineStr"/>
+      <c r="EG57" t="inlineStr"/>
+      <c r="EH57" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI57" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ57" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK57" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL57" t="inlineStr"/>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:24:19</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C58" t="n">
+        <v>84</v>
+      </c>
+      <c r="D58" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E58" t="n">
+        <v>1210000010</v>
+      </c>
+      <c r="F58" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="n">
+        <v>0</v>
+      </c>
+      <c r="J58" t="n">
+        <v>22133</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L58" t="n">
+        <v>408</v>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O58" t="n">
+        <v>408</v>
+      </c>
+      <c r="P58" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q58" t="n">
+        <v>1781060400</v>
+      </c>
+      <c r="R58" t="n">
+        <v>1781093741</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:15</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W58" t="n">
+        <v>22133</v>
+      </c>
+      <c r="X58" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y58" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z58" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AA58" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB58" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC58" t="n">
+        <v>487</v>
+      </c>
+      <c r="AD58" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE58" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF58" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG58" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH58" t="inlineStr"/>
+      <c r="AI58" t="inlineStr"/>
+      <c r="AJ58" t="inlineStr"/>
+      <c r="AK58" t="inlineStr"/>
+      <c r="AL58" t="inlineStr"/>
+      <c r="AM58" t="n">
+        <v>127857</v>
+      </c>
+      <c r="AN58" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO58" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP58" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ58" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR58" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS58" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT58" t="n">
+        <v>3500</v>
+      </c>
+      <c r="AU58" t="inlineStr"/>
+      <c r="AV58" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW58" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX58" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY58" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ58" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA58" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB58" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC58" t="inlineStr"/>
+      <c r="BD58" t="inlineStr"/>
+      <c r="BE58" t="inlineStr"/>
+      <c r="BF58" t="inlineStr"/>
+      <c r="BG58" t="inlineStr"/>
+      <c r="BH58" t="inlineStr"/>
+      <c r="BI58" t="inlineStr"/>
+      <c r="BJ58" t="inlineStr"/>
+      <c r="BK58" t="inlineStr"/>
+      <c r="BL58" t="inlineStr"/>
+      <c r="BM58" t="inlineStr"/>
+      <c r="BN58" t="inlineStr"/>
+      <c r="BO58" t="inlineStr"/>
+      <c r="BP58" t="inlineStr"/>
+      <c r="BQ58" t="inlineStr"/>
+      <c r="BR58" t="inlineStr"/>
+      <c r="BS58" t="inlineStr"/>
+      <c r="BT58" t="inlineStr"/>
+      <c r="BU58" t="inlineStr"/>
+      <c r="BV58" t="inlineStr"/>
+      <c r="BW58" t="inlineStr"/>
+      <c r="BX58" t="inlineStr"/>
+      <c r="BY58" t="inlineStr"/>
+      <c r="BZ58" t="inlineStr"/>
+      <c r="CA58" t="inlineStr"/>
+      <c r="CB58" t="inlineStr"/>
+      <c r="CC58" t="inlineStr"/>
+      <c r="CD58" t="inlineStr"/>
+      <c r="CE58" t="inlineStr"/>
+      <c r="CF58" t="inlineStr"/>
+      <c r="CG58" t="inlineStr"/>
+      <c r="CH58" t="inlineStr"/>
+      <c r="CI58" t="inlineStr"/>
+      <c r="CJ58" t="inlineStr"/>
+      <c r="CK58" t="inlineStr"/>
+      <c r="CL58" t="inlineStr"/>
+      <c r="CM58" t="inlineStr"/>
+      <c r="CN58" t="inlineStr"/>
+      <c r="CO58" t="inlineStr"/>
+      <c r="CP58" t="inlineStr"/>
+      <c r="CQ58" t="inlineStr"/>
+      <c r="CR58" t="inlineStr"/>
+      <c r="CS58" t="inlineStr"/>
+      <c r="CT58" t="inlineStr"/>
+      <c r="CU58" t="inlineStr"/>
+      <c r="CV58" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW58" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX58" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY58" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ58" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA58" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB58" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC58" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD58" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE58" t="n">
+        <v>1121029128</v>
+      </c>
+      <c r="DF58" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG58" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH58" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI58" t="n">
+        <v>212122</v>
+      </c>
+      <c r="DJ58" t="n">
+        <v>12344</v>
+      </c>
+      <c r="DK58" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL58" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM58" t="n">
+        <v>121212212112</v>
+      </c>
+      <c r="DN58" t="inlineStr"/>
+      <c r="DO58" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP58" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ58" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR58" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS58" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT58" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU58" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV58" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW58" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX58" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY58" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ58" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA58" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB58" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC58" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED58" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE58" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF58" t="inlineStr"/>
+      <c r="EG58" t="inlineStr"/>
+      <c r="EH58" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI58" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ58" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK58" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL58" t="inlineStr"/>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>10/06/2026, 09:25:20</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>84</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>01210000010</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr"/>
+      <c r="H59" t="inlineStr"/>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P59" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q59" t="inlineStr">
+        <is>
+          <t>1781060400</t>
+        </is>
+      </c>
+      <c r="R59" t="inlineStr">
+        <is>
+          <t>1781093802</t>
+        </is>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>09:16</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>10/06/2026 09:16</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:13</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>22133</t>
+        </is>
+      </c>
+      <c r="X59" t="inlineStr">
+        <is>
+          <t>03/06/2026 17:24</t>
+        </is>
+      </c>
+      <c r="Y59" t="inlineStr">
+        <is>
+          <t>04/06/2026 17:25</t>
+        </is>
+      </c>
+      <c r="Z59" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AA59" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB59" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC59" t="inlineStr">
+        <is>
+          <t>487</t>
+        </is>
+      </c>
+      <c r="AD59" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AE59" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF59" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG59" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH59" t="inlineStr"/>
+      <c r="AI59" t="inlineStr"/>
+      <c r="AJ59" t="inlineStr"/>
+      <c r="AK59" t="inlineStr"/>
+      <c r="AL59" t="inlineStr"/>
+      <c r="AM59" t="inlineStr">
+        <is>
+          <t>127857</t>
+        </is>
+      </c>
+      <c r="AN59" t="inlineStr">
+        <is>
+          <t>Pedro Santana</t>
+        </is>
+      </c>
+      <c r="AO59" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP59" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ59" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR59" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS59" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT59" t="inlineStr">
+        <is>
+          <t>3500.00</t>
+        </is>
+      </c>
+      <c r="AU59" t="inlineStr"/>
+      <c r="AV59" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW59" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX59" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY59" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ59" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA59" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB59" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC59" t="inlineStr"/>
+      <c r="BD59" t="inlineStr"/>
+      <c r="BE59" t="inlineStr"/>
+      <c r="BF59" t="inlineStr"/>
+      <c r="BG59" t="inlineStr"/>
+      <c r="BH59" t="inlineStr"/>
+      <c r="BI59" t="inlineStr"/>
+      <c r="BJ59" t="inlineStr"/>
+      <c r="BK59" t="inlineStr"/>
+      <c r="BL59" t="inlineStr"/>
+      <c r="BM59" t="inlineStr"/>
+      <c r="BN59" t="inlineStr"/>
+      <c r="BO59" t="inlineStr"/>
+      <c r="BP59" t="inlineStr"/>
+      <c r="BQ59" t="inlineStr"/>
+      <c r="BR59" t="inlineStr"/>
+      <c r="BS59" t="inlineStr"/>
+      <c r="BT59" t="inlineStr"/>
+      <c r="BU59" t="inlineStr"/>
+      <c r="BV59" t="inlineStr"/>
+      <c r="BW59" t="inlineStr"/>
+      <c r="BX59" t="inlineStr"/>
+      <c r="BY59" t="inlineStr"/>
+      <c r="BZ59" t="inlineStr"/>
+      <c r="CA59" t="inlineStr"/>
+      <c r="CB59" t="inlineStr"/>
+      <c r="CC59" t="inlineStr"/>
+      <c r="CD59" t="inlineStr"/>
+      <c r="CE59" t="inlineStr"/>
+      <c r="CF59" t="inlineStr"/>
+      <c r="CG59" t="inlineStr"/>
+      <c r="CH59" t="inlineStr"/>
+      <c r="CI59" t="inlineStr"/>
+      <c r="CJ59" t="inlineStr"/>
+      <c r="CK59" t="inlineStr"/>
+      <c r="CL59" t="inlineStr"/>
+      <c r="CM59" t="inlineStr"/>
+      <c r="CN59" t="inlineStr"/>
+      <c r="CO59" t="inlineStr"/>
+      <c r="CP59" t="inlineStr"/>
+      <c r="CQ59" t="inlineStr"/>
+      <c r="CR59" t="inlineStr"/>
+      <c r="CS59" t="inlineStr"/>
+      <c r="CT59" t="inlineStr"/>
+      <c r="CU59" t="inlineStr"/>
+      <c r="CV59" t="inlineStr">
+        <is>
+          <t>alex de Niterói</t>
+        </is>
+      </c>
+      <c r="CW59" t="inlineStr">
+        <is>
+          <t>15/12/1985</t>
+        </is>
+      </c>
+      <c r="CX59" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY59" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ59" t="inlineStr">
+        <is>
+          <t>Jackson</t>
+        </is>
+      </c>
+      <c r="DA59" t="inlineStr">
+        <is>
+          <t>Maria</t>
+        </is>
+      </c>
+      <c r="DB59" t="inlineStr">
+        <is>
+          <t>jackson</t>
+        </is>
+      </c>
+      <c r="DC59" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD59" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE59" t="inlineStr">
+        <is>
+          <t>1121029128</t>
+        </is>
+      </c>
+      <c r="DF59" t="inlineStr">
+        <is>
+          <t>maria</t>
+        </is>
+      </c>
+      <c r="DG59" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DH59" t="inlineStr">
+        <is>
+          <t>Namorado(a)</t>
+        </is>
+      </c>
+      <c r="DI59" t="inlineStr">
+        <is>
+          <t>212122</t>
+        </is>
+      </c>
+      <c r="DJ59" t="inlineStr">
+        <is>
+          <t>12344</t>
+        </is>
+      </c>
+      <c r="DK59" t="inlineStr">
+        <is>
+          <t>042.815.546-45</t>
+        </is>
+      </c>
+      <c r="DL59" t="inlineStr">
+        <is>
+          <t>pedro.santana@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="DM59" t="inlineStr">
+        <is>
+          <t>121212212112</t>
+        </is>
+      </c>
+      <c r="DN59" t="inlineStr"/>
+      <c r="DO59" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP59" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ59" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR59" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS59" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT59" t="inlineStr">
+        <is>
+          <t>dadadqr</t>
+        </is>
+      </c>
+      <c r="DU59" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV59" t="inlineStr">
+        <is>
+          <t>etetetet</t>
+        </is>
+      </c>
+      <c r="DW59" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX59" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY59" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ59" t="inlineStr">
+        <is>
+          <t>wrwrwrw</t>
+        </is>
+      </c>
+      <c r="EA59" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB59" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC59" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED59" t="inlineStr">
+        <is>
+          <t>aaa</t>
+        </is>
+      </c>
+      <c r="EE59" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF59" t="inlineStr"/>
+      <c r="EG59" t="inlineStr"/>
+      <c r="EH59" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Eduardo Rocha - {{2026-06-03 17:24:17}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-03 17:23:48}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Proposta&lt;br&gt;Adrielly Santana - {{2026-06-03 17:23:29}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;avançar &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-06-03 17:21:57}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;teste &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;Pedro Santana - {{2026-06-03 17:20:42}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aprovado &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-03 17:20:13}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02.5 - Aprovação Recrutamento&lt;br&gt;Fernando Andrade - {{2026-06-03 17:17:36}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-03 17:15:35}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;prosseguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;Pedro Santana - {{2026-06-03 17:14:43}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;prosseguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI59" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção e assinatura (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ59" t="inlineStr">
+        <is>
+          <t>08 - Confecção e assinatura (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK59" t="inlineStr">
+        <is>
+          <t>Alexzinho de Niterói</t>
+        </is>
+      </c>
+      <c r="EL59" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -23393,13 +26881,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F0AD173E-02E4-44B4-B9A9-35A413A9532A}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C2A788E-BB37-4653-AD65-3C999FF24002}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{09A9F1D5-FB0F-446E-A87A-7CDF91E228EB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8AA4E6DB-2AC6-4FB4-A24F-B38DFC99D9AB}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0336733E-B746-4DDA-B755-3AF2BC5749A3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ADDB313E-B6AC-45C9-A851-3A4EE982B7B3}"/>
 </file>
</xml_diff>

<commit_message>
Add task definitions for VS Code and Zed editors
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL62"/>
+  <dimension ref="A1:EL63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -27575,47 +27575,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>102</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E62" t="inlineStr">
-        <is>
-          <t>01210000013</t>
-        </is>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C62" t="n">
+        <v>102</v>
+      </c>
+      <c r="D62" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E62" t="n">
+        <v>1210000013</v>
+      </c>
+      <c r="F62" t="n">
+        <v>1</v>
       </c>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>22250</t>
-        </is>
+      <c r="I62" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" t="n">
+        <v>22250</v>
       </c>
       <c r="K62" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L62" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L62" t="n">
+        <v>408</v>
       </c>
       <c r="M62" t="inlineStr">
         <is>
@@ -27627,25 +27613,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O62" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O62" t="n">
+        <v>408</v>
       </c>
       <c r="P62" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q62" t="inlineStr">
-        <is>
-          <t>1781492400</t>
-        </is>
-      </c>
-      <c r="R62" t="inlineStr">
-        <is>
-          <t>1781529474</t>
-        </is>
+      <c r="Q62" t="n">
+        <v>1781492400</v>
+      </c>
+      <c r="R62" t="n">
+        <v>1781529474</v>
       </c>
       <c r="S62" t="inlineStr">
         <is>
@@ -27667,10 +27647,8 @@
           <t>10/06/2026 11:40</t>
         </is>
       </c>
-      <c r="W62" t="inlineStr">
-        <is>
-          <t>22250</t>
-        </is>
+      <c r="W62" t="n">
+        <v>22250</v>
       </c>
       <c r="X62" t="inlineStr">
         <is>
@@ -27682,35 +27660,27 @@
           <t>11/06/2026 11:46</t>
         </is>
       </c>
-      <c r="Z62" t="inlineStr">
-        <is>
-          <t>128496</t>
-        </is>
+      <c r="Z62" t="n">
+        <v>128496</v>
       </c>
       <c r="AA62" t="inlineStr">
         <is>
           <t>05.1 - Confecção Proposta</t>
         </is>
       </c>
-      <c r="AB62" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC62" t="inlineStr">
-        <is>
-          <t>363</t>
-        </is>
+      <c r="AB62" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC62" t="n">
+        <v>363</v>
       </c>
       <c r="AD62" t="inlineStr">
         <is>
           <t>Karolina Navarro</t>
         </is>
       </c>
-      <c r="AE62" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE62" t="n">
+        <v>121</v>
       </c>
       <c r="AF62" t="inlineStr">
         <is>
@@ -27727,10 +27697,8 @@
       <c r="AJ62" t="inlineStr"/>
       <c r="AK62" t="inlineStr"/>
       <c r="AL62" t="inlineStr"/>
-      <c r="AM62" t="inlineStr">
-        <is>
-          <t>128496</t>
-        </is>
+      <c r="AM62" t="n">
+        <v>128496</v>
       </c>
       <c r="AN62" t="inlineStr">
         <is>
@@ -27762,10 +27730,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT62" t="inlineStr">
-        <is>
-          <t>20000.00</t>
-        </is>
+      <c r="AT62" t="n">
+        <v>20000</v>
       </c>
       <c r="AU62" t="inlineStr"/>
       <c r="AV62" t="inlineStr">
@@ -27997,10 +27963,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE62" t="inlineStr">
-        <is>
-          <t>1121029128</t>
-        </is>
+      <c r="DE62" t="n">
+        <v>1121029128</v>
       </c>
       <c r="DF62" t="inlineStr"/>
       <c r="DG62" t="inlineStr">
@@ -28013,15 +27977,11 @@
           <t>- Selecione algo -</t>
         </is>
       </c>
-      <c r="DI62" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="DJ62" t="inlineStr">
-        <is>
-          <t>392003077</t>
-        </is>
+      <c r="DI62" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ62" t="n">
+        <v>392003077</v>
       </c>
       <c r="DK62" t="inlineStr">
         <is>
@@ -28033,10 +27993,8 @@
           <t>alessandra.maite.rocha@hardquality.com.br</t>
         </is>
       </c>
-      <c r="DM62" t="inlineStr">
-        <is>
-          <t>27999923013</t>
-        </is>
+      <c r="DM62" t="n">
+        <v>27999923013</v>
       </c>
       <c r="DN62" t="inlineStr"/>
       <c r="DO62" t="inlineStr">
@@ -28054,15 +28012,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR62" t="inlineStr">
-        <is>
-          <t>302</t>
-        </is>
-      </c>
-      <c r="DS62" t="inlineStr">
-        <is>
-          <t>10517413</t>
-        </is>
+      <c r="DR62" t="n">
+        <v>302</v>
+      </c>
+      <c r="DS62" t="n">
+        <v>10517413</v>
       </c>
       <c r="DT62" t="inlineStr">
         <is>
@@ -28079,10 +28033,8 @@
           <t>Rua Seis</t>
         </is>
       </c>
-      <c r="DW62" t="inlineStr">
-        <is>
-          <t>808</t>
-        </is>
+      <c r="DW62" t="n">
+        <v>808</v>
       </c>
       <c r="DX62" t="inlineStr"/>
       <c r="DY62" t="inlineStr">
@@ -28139,247 +28091,586 @@
       </c>
       <c r="EK62" t="inlineStr"/>
       <c r="EL62" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>24/06/2026, 09:52:42</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>01210000013</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>22612</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q63" t="inlineStr">
+        <is>
+          <t>1782270000</t>
+        </is>
+      </c>
+      <c r="R63" t="inlineStr">
+        <is>
+          <t>1782304941</t>
+        </is>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>24/06/2026</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>09:42</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:42</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:10</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>22612</t>
+        </is>
+      </c>
+      <c r="X63" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:20</t>
+        </is>
+      </c>
+      <c r="Y63" t="inlineStr">
+        <is>
+          <t>25/06/2026 09:21</t>
+        </is>
+      </c>
+      <c r="Z63" t="inlineStr">
+        <is>
+          <t>130404</t>
+        </is>
+      </c>
+      <c r="AA63" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="AB63" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC63" t="inlineStr">
+        <is>
+          <t>427</t>
+        </is>
+      </c>
+      <c r="AD63" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE63" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF63" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG63" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH63" t="inlineStr"/>
+      <c r="AI63" t="inlineStr"/>
+      <c r="AJ63" t="inlineStr"/>
+      <c r="AK63" t="inlineStr"/>
+      <c r="AL63" t="inlineStr"/>
+      <c r="AM63" t="inlineStr">
+        <is>
+          <t>130404</t>
+        </is>
+      </c>
+      <c r="AN63" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO63" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP63" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ63" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR63" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS63" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT63" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="AU63" t="inlineStr"/>
+      <c r="AV63" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW63" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX63" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY63" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ63" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA63" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB63" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC63" t="inlineStr">
+        <is>
+          <t>[x] Notebook</t>
+        </is>
+      </c>
+      <c r="BD63" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BE63" t="inlineStr"/>
+      <c r="BF63" t="inlineStr">
+        <is>
+          <t>[x] Celular</t>
+        </is>
+      </c>
+      <c r="BG63" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BH63" t="inlineStr"/>
+      <c r="BI63" t="inlineStr">
+        <is>
+          <t>[ ] Teclado</t>
+        </is>
+      </c>
+      <c r="BJ63" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK63" t="inlineStr"/>
+      <c r="BL63" t="inlineStr">
+        <is>
+          <t>[ ] Mouse</t>
+        </is>
+      </c>
+      <c r="BM63" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN63" t="inlineStr"/>
+      <c r="BO63" t="inlineStr">
+        <is>
+          <t>[ ] Fone</t>
+        </is>
+      </c>
+      <c r="BP63" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ63" t="inlineStr"/>
+      <c r="BR63" t="inlineStr">
+        <is>
+          <t>[ ] Linha móvel</t>
+        </is>
+      </c>
+      <c r="BS63" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT63" t="inlineStr"/>
+      <c r="BU63" t="inlineStr">
+        <is>
+          <t>[x] 365</t>
+        </is>
+      </c>
+      <c r="BV63" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW63" t="inlineStr"/>
+      <c r="BX63" t="inlineStr">
+        <is>
+          <t>[x] LegalOne</t>
+        </is>
+      </c>
+      <c r="BY63" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BZ63" t="inlineStr"/>
+      <c r="CA63" t="inlineStr">
+        <is>
+          <t>[ ] MKTZap</t>
+        </is>
+      </c>
+      <c r="CB63" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC63" t="inlineStr"/>
+      <c r="CD63" t="inlineStr">
+        <is>
+          <t>[ ] WorkFlow</t>
+        </is>
+      </c>
+      <c r="CE63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF63" t="inlineStr"/>
+      <c r="CG63" t="inlineStr">
+        <is>
+          <t>[ ] Doc9/Whom</t>
+        </is>
+      </c>
+      <c r="CH63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI63" t="inlineStr"/>
+      <c r="CJ63" t="inlineStr">
+        <is>
+          <t>[ ] Dominio</t>
+        </is>
+      </c>
+      <c r="CK63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL63" t="inlineStr"/>
+      <c r="CM63" t="inlineStr">
+        <is>
+          <t>[ ] RD Station</t>
+        </is>
+      </c>
+      <c r="CN63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO63" t="inlineStr"/>
+      <c r="CP63" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - PowerBI</t>
+        </is>
+      </c>
+      <c r="CQ63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR63" t="inlineStr"/>
+      <c r="CS63" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - Power Automate</t>
+        </is>
+      </c>
+      <c r="CT63" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU63" t="inlineStr"/>
+      <c r="CV63" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="CW63" t="inlineStr">
+        <is>
+          <t>14/05/1998</t>
+        </is>
+      </c>
+      <c r="CX63" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CY63" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CZ63" t="inlineStr">
+        <is>
+          <t>Pedro Henrique Anthony Roberto Vieira</t>
+        </is>
+      </c>
+      <c r="DA63" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DB63" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DC63" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DD63" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DE63" t="inlineStr">
+        <is>
+          <t>79999552575</t>
+        </is>
+      </c>
+      <c r="DF63" t="inlineStr"/>
+      <c r="DG63" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH63" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI63" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DJ63" t="inlineStr">
+        <is>
+          <t>339799149</t>
+        </is>
+      </c>
+      <c r="DK63" t="inlineStr">
+        <is>
+          <t>009.510.135-72</t>
+        </is>
+      </c>
+      <c r="DL63" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DM63" t="inlineStr">
+        <is>
+          <t>69994528502</t>
+        </is>
+      </c>
+      <c r="DN63" t="inlineStr">
+        <is>
+          <t>43.169.616/0001-01</t>
+        </is>
+      </c>
+      <c r="DO63" t="inlineStr">
+        <is>
+          <t>Itau</t>
+        </is>
+      </c>
+      <c r="DP63" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ63" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR63" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
+      <c r="DS63" t="inlineStr">
+        <is>
+          <t>324401</t>
+        </is>
+      </c>
+      <c r="DT63" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DU63" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="DV63" t="inlineStr">
+        <is>
+          <t>Rua A</t>
+        </is>
+      </c>
+      <c r="DW63" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX63" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY63" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ63" t="inlineStr">
+        <is>
+          <t>Jabotiana</t>
+        </is>
+      </c>
+      <c r="EA63" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB63" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC63" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED63" t="inlineStr">
+        <is>
+          <t>Mecanica</t>
+        </is>
+      </c>
+      <c r="EE63" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF63" t="inlineStr"/>
+      <c r="EG63" t="inlineStr"/>
+      <c r="EH63" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-24 09:20:15}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-06-24 09:19:59}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-24 09:19:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-24 09:11:53}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-06-24 09:11:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI63" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ63" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="EK63" t="inlineStr"/>
+      <c r="EL63" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100B5FCC50092DEF84396333E47DAEFEB5E" ma:contentTypeVersion="13" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="3f5dff31fa7a2b799118bc7c00128ae3">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" xmlns:ns3="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5a22452f93ee1f3c8f432c572ea5d732" ns2:_="" ns3:_="">
-    <xsd:import namespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51"/>
-    <xsd:import namespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db"/>
-    <xsd:element name="properties">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element name="documentManagement">
-            <xsd:complexType>
-              <xsd:all>
-                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
-                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
-                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
-                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
-              </xsd:all>
-            </xsd:complexType>
-          </xsd:element>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="5df11fd7-6aff-4cc6-9d69-481ebafd3f51" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceSearchProperties" ma:index="10" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="11" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="13" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Marcações de imagem" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="4410abd1-e841-4d52-8c09-cc5936d54c0f" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
-      <xsd:complexType>
-        <xsd:sequence>
-          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
-        </xsd:sequence>
-      </xsd:complexType>
-    </xsd:element>
-    <xsd:element name="MediaServiceDateTaken" ma:index="15" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceOCR" ma:index="16" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Note">
-          <xsd:maxLength value="255"/>
-        </xsd:restriction>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceGenerationTime" ma:index="17" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceEventHashCode" ma:index="18" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaServiceLocation" ma:index="19" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Text"/>
-      </xsd:simpleType>
-    </xsd:element>
-    <xsd:element name="MediaLengthInSeconds" ma:index="20" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
-      <xsd:simpleType>
-        <xsd:restriction base="dms:Unknown"/>
-      </xsd:simpleType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" elementFormDefault="qualified">
-    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="TaxCatchAll" ma:index="14" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{78d918e0-dd2a-4d55-9cd7-b9c5d47e1b97}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db">
-      <xsd:complexType>
-        <xsd:complexContent>
-          <xsd:extension base="dms:MultiChoiceLookup">
-            <xsd:sequence>
-              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
-            </xsd:sequence>
-          </xsd:extension>
-        </xsd:complexContent>
-      </xsd:complexType>
-    </xsd:element>
-  </xsd:schema>
-  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
-    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
-    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
-    <xsd:element name="coreProperties" type="CT_coreProperties"/>
-    <xsd:complexType name="CT_coreProperties">
-      <xsd:all>
-        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Tipo de Conteúdo"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Título"/>
-        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
-        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
-          <xsd:annotation>
-            <xsd:documentation>
-                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
-                    </xsd:documentation>
-          </xsd:annotation>
-        </xsd:element>
-        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
-      </xsd:all>
-    </xsd:complexType>
-  </xsd:schema>
-  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
-    <xs:element name="Person">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:DisplayName" minOccurs="0"/>
-          <xs:element ref="pc:AccountId" minOccurs="0"/>
-          <xs:element ref="pc:AccountType" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="DisplayName" type="xs:string"/>
-    <xs:element name="AccountId" type="xs:string"/>
-    <xs:element name="AccountType" type="xs:string"/>
-    <xs:element name="BDCAssociatedEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-        <xs:attribute ref="pc:EntityNamespace"/>
-        <xs:attribute ref="pc:EntityName"/>
-        <xs:attribute ref="pc:SystemInstanceName"/>
-        <xs:attribute ref="pc:AssociationName"/>
-      </xs:complexType>
-    </xs:element>
-    <xs:attribute name="EntityNamespace" type="xs:string"/>
-    <xs:attribute name="EntityName" type="xs:string"/>
-    <xs:attribute name="SystemInstanceName" type="xs:string"/>
-    <xs:attribute name="AssociationName" type="xs:string"/>
-    <xs:element name="BDCEntity">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
-          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
-          <xs:element ref="pc:EntityId1" minOccurs="0"/>
-          <xs:element ref="pc:EntityId2" minOccurs="0"/>
-          <xs:element ref="pc:EntityId3" minOccurs="0"/>
-          <xs:element ref="pc:EntityId4" minOccurs="0"/>
-          <xs:element ref="pc:EntityId5" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="EntityDisplayName" type="xs:string"/>
-    <xs:element name="EntityInstanceReference" type="xs:string"/>
-    <xs:element name="EntityId1" type="xs:string"/>
-    <xs:element name="EntityId2" type="xs:string"/>
-    <xs:element name="EntityId3" type="xs:string"/>
-    <xs:element name="EntityId4" type="xs:string"/>
-    <xs:element name="EntityId5" type="xs:string"/>
-    <xs:element name="Terms">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermInfo">
-      <xs:complexType>
-        <xs:sequence>
-          <xs:element ref="pc:TermName" minOccurs="0"/>
-          <xs:element ref="pc:TermId" minOccurs="0"/>
-        </xs:sequence>
-      </xs:complexType>
-    </xs:element>
-    <xs:element name="TermName" type="xs:string"/>
-    <xs:element name="TermId" type="xs:string"/>
-  </xs:schema>
-</ct:contentTypeSchema>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ba98ff8d-cf9c-4574-b9ff-8782fca0b7db" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5df11fd7-6aff-4cc6-9d69-481ebafd3f51">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B807571-995F-4DD0-8353-F6F31947D694}"/>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EAEBDD51-810A-46D5-A7EB-DE0197B4B33A}"/>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A965ED70-0358-4620-ACC7-2A7AECBE31FE}"/>
 </file>
</xml_diff>

<commit_message>
feat(workflows): add finalize proposal workflow to complete Triata task after ZapSign
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EL63"/>
+  <dimension ref="A1:EL65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28103,47 +28103,33 @@
           <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>108</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>01210000013</t>
-        </is>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C63" t="n">
+        <v>108</v>
+      </c>
+      <c r="D63" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E63" t="n">
+        <v>1210000013</v>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
       </c>
       <c r="G63" t="inlineStr"/>
       <c r="H63" t="inlineStr"/>
-      <c r="I63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>22612</t>
-        </is>
+      <c r="I63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J63" t="n">
+        <v>22612</v>
       </c>
       <c r="K63" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L63" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L63" t="n">
+        <v>408</v>
       </c>
       <c r="M63" t="inlineStr">
         <is>
@@ -28155,25 +28141,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O63" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O63" t="n">
+        <v>408</v>
       </c>
       <c r="P63" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q63" t="inlineStr">
-        <is>
-          <t>1782270000</t>
-        </is>
-      </c>
-      <c r="R63" t="inlineStr">
-        <is>
-          <t>1782304941</t>
-        </is>
+      <c r="Q63" t="n">
+        <v>1782270000</v>
+      </c>
+      <c r="R63" t="n">
+        <v>1782304941</v>
       </c>
       <c r="S63" t="inlineStr">
         <is>
@@ -28195,10 +28175,8 @@
           <t>24/06/2026 09:10</t>
         </is>
       </c>
-      <c r="W63" t="inlineStr">
-        <is>
-          <t>22612</t>
-        </is>
+      <c r="W63" t="n">
+        <v>22612</v>
       </c>
       <c r="X63" t="inlineStr">
         <is>
@@ -28210,35 +28188,27 @@
           <t>25/06/2026 09:21</t>
         </is>
       </c>
-      <c r="Z63" t="inlineStr">
-        <is>
-          <t>130404</t>
-        </is>
+      <c r="Z63" t="n">
+        <v>130404</v>
       </c>
       <c r="AA63" t="inlineStr">
         <is>
           <t>05.1 - Confecção Proposta</t>
         </is>
       </c>
-      <c r="AB63" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC63" t="inlineStr">
-        <is>
-          <t>427</t>
-        </is>
+      <c r="AB63" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC63" t="n">
+        <v>427</v>
       </c>
       <c r="AD63" t="inlineStr">
         <is>
           <t>tiago izaias</t>
         </is>
       </c>
-      <c r="AE63" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE63" t="n">
+        <v>121</v>
       </c>
       <c r="AF63" t="inlineStr">
         <is>
@@ -28255,10 +28225,8 @@
       <c r="AJ63" t="inlineStr"/>
       <c r="AK63" t="inlineStr"/>
       <c r="AL63" t="inlineStr"/>
-      <c r="AM63" t="inlineStr">
-        <is>
-          <t>130404</t>
-        </is>
+      <c r="AM63" t="n">
+        <v>130404</v>
       </c>
       <c r="AN63" t="inlineStr">
         <is>
@@ -28290,10 +28258,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT63" t="inlineStr">
-        <is>
-          <t>50000.00</t>
-        </is>
+      <c r="AT63" t="n">
+        <v>50000</v>
       </c>
       <c r="AU63" t="inlineStr"/>
       <c r="AV63" t="inlineStr">
@@ -28367,7 +28333,7 @@
           <t>[ ] Mouse</t>
         </is>
       </c>
-      <c r="BM63" t="b">
+      <c r="BM63" t="n">
         <v>0</v>
       </c>
       <c r="BN63" t="inlineStr"/>
@@ -28376,7 +28342,7 @@
           <t>[ ] Fone</t>
         </is>
       </c>
-      <c r="BP63" t="b">
+      <c r="BP63" t="n">
         <v>0</v>
       </c>
       <c r="BQ63" t="inlineStr"/>
@@ -28519,10 +28485,8 @@
           <t>Mãe</t>
         </is>
       </c>
-      <c r="DE63" t="inlineStr">
-        <is>
-          <t>79999552575</t>
-        </is>
+      <c r="DE63" t="n">
+        <v>79999552575</v>
       </c>
       <c r="DF63" t="inlineStr"/>
       <c r="DG63" t="inlineStr">
@@ -28535,15 +28499,11 @@
           <t>- Selecione algo -</t>
         </is>
       </c>
-      <c r="DI63" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="DJ63" t="inlineStr">
-        <is>
-          <t>339799149</t>
-        </is>
+      <c r="DI63" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ63" t="n">
+        <v>339799149</v>
       </c>
       <c r="DK63" t="inlineStr">
         <is>
@@ -28555,10 +28515,8 @@
           <t>sergionicolasvieira@tursi.com.br</t>
         </is>
       </c>
-      <c r="DM63" t="inlineStr">
-        <is>
-          <t>69994528502</t>
-        </is>
+      <c r="DM63" t="n">
+        <v>69994528502</v>
       </c>
       <c r="DN63" t="inlineStr">
         <is>
@@ -28580,15 +28538,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR63" t="inlineStr">
-        <is>
-          <t>1650</t>
-        </is>
-      </c>
-      <c r="DS63" t="inlineStr">
-        <is>
-          <t>324401</t>
-        </is>
+      <c r="DR63" t="n">
+        <v>1650</v>
+      </c>
+      <c r="DS63" t="n">
+        <v>324401</v>
       </c>
       <c r="DT63" t="inlineStr">
         <is>
@@ -28605,10 +28559,8 @@
           <t>Rua A</t>
         </is>
       </c>
-      <c r="DW63" t="inlineStr">
-        <is>
-          <t>124</t>
-        </is>
+      <c r="DW63" t="n">
+        <v>124</v>
       </c>
       <c r="DX63" t="inlineStr">
         <is>
@@ -28669,6 +28621,1114 @@
       </c>
       <c r="EK63" t="inlineStr"/>
       <c r="EL63" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>29/06/2026, 13:04:54</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C64" t="n">
+        <v>108</v>
+      </c>
+      <c r="D64" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E64" t="n">
+        <v>1210000013</v>
+      </c>
+      <c r="F64" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="n">
+        <v>0</v>
+      </c>
+      <c r="J64" t="n">
+        <v>22612</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L64" t="n">
+        <v>408</v>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O64" t="n">
+        <v>408</v>
+      </c>
+      <c r="P64" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q64" t="n">
+        <v>1782702000</v>
+      </c>
+      <c r="R64" t="n">
+        <v>1782748434</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>29/06/2026 12:53</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:10</t>
+        </is>
+      </c>
+      <c r="W64" t="n">
+        <v>22612</v>
+      </c>
+      <c r="X64" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:20</t>
+        </is>
+      </c>
+      <c r="Y64" t="inlineStr">
+        <is>
+          <t>25/06/2026 09:21</t>
+        </is>
+      </c>
+      <c r="Z64" t="n">
+        <v>130404</v>
+      </c>
+      <c r="AA64" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="AB64" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC64" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD64" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE64" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF64" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG64" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH64" t="inlineStr"/>
+      <c r="AI64" t="inlineStr"/>
+      <c r="AJ64" t="inlineStr"/>
+      <c r="AK64" t="inlineStr"/>
+      <c r="AL64" t="inlineStr"/>
+      <c r="AM64" t="n">
+        <v>130404</v>
+      </c>
+      <c r="AN64" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO64" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP64" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ64" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR64" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS64" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT64" t="n">
+        <v>50000</v>
+      </c>
+      <c r="AU64" t="inlineStr"/>
+      <c r="AV64" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW64" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX64" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY64" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ64" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA64" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB64" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC64" t="inlineStr">
+        <is>
+          <t>[x] Notebook</t>
+        </is>
+      </c>
+      <c r="BD64" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BE64" t="inlineStr"/>
+      <c r="BF64" t="inlineStr">
+        <is>
+          <t>[x] Celular</t>
+        </is>
+      </c>
+      <c r="BG64" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BH64" t="inlineStr"/>
+      <c r="BI64" t="inlineStr">
+        <is>
+          <t>[ ] Teclado</t>
+        </is>
+      </c>
+      <c r="BJ64" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK64" t="inlineStr"/>
+      <c r="BL64" t="inlineStr">
+        <is>
+          <t>[ ] Mouse</t>
+        </is>
+      </c>
+      <c r="BM64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN64" t="inlineStr"/>
+      <c r="BO64" t="inlineStr">
+        <is>
+          <t>[ ] Fone</t>
+        </is>
+      </c>
+      <c r="BP64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BQ64" t="inlineStr"/>
+      <c r="BR64" t="inlineStr">
+        <is>
+          <t>[ ] Linha móvel</t>
+        </is>
+      </c>
+      <c r="BS64" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT64" t="inlineStr"/>
+      <c r="BU64" t="inlineStr">
+        <is>
+          <t>[x] 365</t>
+        </is>
+      </c>
+      <c r="BV64" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW64" t="inlineStr"/>
+      <c r="BX64" t="inlineStr">
+        <is>
+          <t>[x] LegalOne</t>
+        </is>
+      </c>
+      <c r="BY64" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BZ64" t="inlineStr"/>
+      <c r="CA64" t="inlineStr">
+        <is>
+          <t>[ ] MKTZap</t>
+        </is>
+      </c>
+      <c r="CB64" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC64" t="inlineStr"/>
+      <c r="CD64" t="inlineStr">
+        <is>
+          <t>[ ] WorkFlow</t>
+        </is>
+      </c>
+      <c r="CE64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF64" t="inlineStr"/>
+      <c r="CG64" t="inlineStr">
+        <is>
+          <t>[ ] Doc9/Whom</t>
+        </is>
+      </c>
+      <c r="CH64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI64" t="inlineStr"/>
+      <c r="CJ64" t="inlineStr">
+        <is>
+          <t>[ ] Dominio</t>
+        </is>
+      </c>
+      <c r="CK64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL64" t="inlineStr"/>
+      <c r="CM64" t="inlineStr">
+        <is>
+          <t>[ ] RD Station</t>
+        </is>
+      </c>
+      <c r="CN64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO64" t="inlineStr"/>
+      <c r="CP64" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - PowerBI</t>
+        </is>
+      </c>
+      <c r="CQ64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR64" t="inlineStr"/>
+      <c r="CS64" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - Power Automate</t>
+        </is>
+      </c>
+      <c r="CT64" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU64" t="inlineStr"/>
+      <c r="CV64" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="CW64" t="inlineStr">
+        <is>
+          <t>14/05/1998</t>
+        </is>
+      </c>
+      <c r="CX64" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CY64" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CZ64" t="inlineStr">
+        <is>
+          <t>Pedro Henrique Anthony Roberto Vieira</t>
+        </is>
+      </c>
+      <c r="DA64" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DB64" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DC64" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DD64" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DE64" t="n">
+        <v>79999552575</v>
+      </c>
+      <c r="DF64" t="inlineStr"/>
+      <c r="DG64" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH64" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI64" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ64" t="n">
+        <v>339799149</v>
+      </c>
+      <c r="DK64" t="inlineStr">
+        <is>
+          <t>009.510.135-72</t>
+        </is>
+      </c>
+      <c r="DL64" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DM64" t="n">
+        <v>69994528502</v>
+      </c>
+      <c r="DN64" t="inlineStr">
+        <is>
+          <t>43.169.616/0001-01</t>
+        </is>
+      </c>
+      <c r="DO64" t="inlineStr">
+        <is>
+          <t>Itau</t>
+        </is>
+      </c>
+      <c r="DP64" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ64" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR64" t="n">
+        <v>1650</v>
+      </c>
+      <c r="DS64" t="n">
+        <v>324401</v>
+      </c>
+      <c r="DT64" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DU64" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="DV64" t="inlineStr">
+        <is>
+          <t>Rua A</t>
+        </is>
+      </c>
+      <c r="DW64" t="n">
+        <v>124</v>
+      </c>
+      <c r="DX64" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY64" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ64" t="inlineStr">
+        <is>
+          <t>Jabotiana</t>
+        </is>
+      </c>
+      <c r="EA64" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB64" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC64" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED64" t="inlineStr">
+        <is>
+          <t>Mecanica</t>
+        </is>
+      </c>
+      <c r="EE64" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF64" t="inlineStr"/>
+      <c r="EG64" t="inlineStr"/>
+      <c r="EH64" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-24 09:20:15}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-06-24 09:19:59}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-24 09:19:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-24 09:11:53}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-06-24 09:11:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI64" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ64" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="EK64" t="inlineStr"/>
+      <c r="EL64" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>29/06/2026, 13:07:51</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>108</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>01210000013</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>22612</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q65" t="inlineStr">
+        <is>
+          <t>1782702000</t>
+        </is>
+      </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>1782748611</t>
+        </is>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>29/06/2026</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>12:56</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>29/06/2026 12:56</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:10</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>22612</t>
+        </is>
+      </c>
+      <c r="X65" t="inlineStr">
+        <is>
+          <t>24/06/2026 09:20</t>
+        </is>
+      </c>
+      <c r="Y65" t="inlineStr">
+        <is>
+          <t>25/06/2026 09:21</t>
+        </is>
+      </c>
+      <c r="Z65" t="inlineStr">
+        <is>
+          <t>130404</t>
+        </is>
+      </c>
+      <c r="AA65" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="AB65" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC65" t="inlineStr">
+        <is>
+          <t>427</t>
+        </is>
+      </c>
+      <c r="AD65" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE65" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF65" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG65" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH65" t="inlineStr"/>
+      <c r="AI65" t="inlineStr"/>
+      <c r="AJ65" t="inlineStr"/>
+      <c r="AK65" t="inlineStr"/>
+      <c r="AL65" t="inlineStr"/>
+      <c r="AM65" t="inlineStr">
+        <is>
+          <t>130404</t>
+        </is>
+      </c>
+      <c r="AN65" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO65" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP65" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ65" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR65" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS65" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT65" t="inlineStr">
+        <is>
+          <t>50000.00</t>
+        </is>
+      </c>
+      <c r="AU65" t="inlineStr"/>
+      <c r="AV65" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW65" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX65" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY65" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ65" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA65" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB65" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC65" t="inlineStr">
+        <is>
+          <t>[x] Notebook</t>
+        </is>
+      </c>
+      <c r="BD65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BE65" t="inlineStr"/>
+      <c r="BF65" t="inlineStr">
+        <is>
+          <t>[x] Celular</t>
+        </is>
+      </c>
+      <c r="BG65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BH65" t="inlineStr"/>
+      <c r="BI65" t="inlineStr">
+        <is>
+          <t>[ ] Teclado</t>
+        </is>
+      </c>
+      <c r="BJ65" t="b">
+        <v>0</v>
+      </c>
+      <c r="BK65" t="inlineStr"/>
+      <c r="BL65" t="inlineStr">
+        <is>
+          <t>[ ] Mouse</t>
+        </is>
+      </c>
+      <c r="BM65" t="b">
+        <v>0</v>
+      </c>
+      <c r="BN65" t="inlineStr"/>
+      <c r="BO65" t="inlineStr">
+        <is>
+          <t>[ ] Fone</t>
+        </is>
+      </c>
+      <c r="BP65" t="b">
+        <v>0</v>
+      </c>
+      <c r="BQ65" t="inlineStr"/>
+      <c r="BR65" t="inlineStr">
+        <is>
+          <t>[ ] Linha móvel</t>
+        </is>
+      </c>
+      <c r="BS65" t="n">
+        <v>0</v>
+      </c>
+      <c r="BT65" t="inlineStr"/>
+      <c r="BU65" t="inlineStr">
+        <is>
+          <t>[x] 365</t>
+        </is>
+      </c>
+      <c r="BV65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BW65" t="inlineStr"/>
+      <c r="BX65" t="inlineStr">
+        <is>
+          <t>[x] LegalOne</t>
+        </is>
+      </c>
+      <c r="BY65" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="BZ65" t="inlineStr"/>
+      <c r="CA65" t="inlineStr">
+        <is>
+          <t>[ ] MKTZap</t>
+        </is>
+      </c>
+      <c r="CB65" t="b">
+        <v>0</v>
+      </c>
+      <c r="CC65" t="inlineStr"/>
+      <c r="CD65" t="inlineStr">
+        <is>
+          <t>[ ] WorkFlow</t>
+        </is>
+      </c>
+      <c r="CE65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CF65" t="inlineStr"/>
+      <c r="CG65" t="inlineStr">
+        <is>
+          <t>[ ] Doc9/Whom</t>
+        </is>
+      </c>
+      <c r="CH65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CI65" t="inlineStr"/>
+      <c r="CJ65" t="inlineStr">
+        <is>
+          <t>[ ] Dominio</t>
+        </is>
+      </c>
+      <c r="CK65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CL65" t="inlineStr"/>
+      <c r="CM65" t="inlineStr">
+        <is>
+          <t>[ ] RD Station</t>
+        </is>
+      </c>
+      <c r="CN65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CO65" t="inlineStr"/>
+      <c r="CP65" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - PowerBI</t>
+        </is>
+      </c>
+      <c r="CQ65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CR65" t="inlineStr"/>
+      <c r="CS65" t="inlineStr">
+        <is>
+          <t>[ ] Adicional - Power Automate</t>
+        </is>
+      </c>
+      <c r="CT65" t="n">
+        <v>0</v>
+      </c>
+      <c r="CU65" t="inlineStr"/>
+      <c r="CV65" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="CW65" t="inlineStr">
+        <is>
+          <t>14/05/1998</t>
+        </is>
+      </c>
+      <c r="CX65" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CY65" t="inlineStr">
+        <is>
+          <t>Casado</t>
+        </is>
+      </c>
+      <c r="CZ65" t="inlineStr">
+        <is>
+          <t>Pedro Henrique Anthony Roberto Vieira</t>
+        </is>
+      </c>
+      <c r="DA65" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DB65" t="inlineStr">
+        <is>
+          <t>Adriana Isabelle</t>
+        </is>
+      </c>
+      <c r="DC65" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DD65" t="inlineStr">
+        <is>
+          <t>Mãe</t>
+        </is>
+      </c>
+      <c r="DE65" t="inlineStr">
+        <is>
+          <t>79999552575</t>
+        </is>
+      </c>
+      <c r="DF65" t="inlineStr"/>
+      <c r="DG65" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH65" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI65" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DJ65" t="inlineStr">
+        <is>
+          <t>339799149</t>
+        </is>
+      </c>
+      <c r="DK65" t="inlineStr">
+        <is>
+          <t>009.510.135-72</t>
+        </is>
+      </c>
+      <c r="DL65" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DM65" t="inlineStr">
+        <is>
+          <t>69994528502</t>
+        </is>
+      </c>
+      <c r="DN65" t="inlineStr">
+        <is>
+          <t>43.169.616/0001-01</t>
+        </is>
+      </c>
+      <c r="DO65" t="inlineStr">
+        <is>
+          <t>Itau</t>
+        </is>
+      </c>
+      <c r="DP65" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ65" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR65" t="inlineStr">
+        <is>
+          <t>1650</t>
+        </is>
+      </c>
+      <c r="DS65" t="inlineStr">
+        <is>
+          <t>324401</t>
+        </is>
+      </c>
+      <c r="DT65" t="inlineStr">
+        <is>
+          <t>sergionicolasvieira@tursi.com.br</t>
+        </is>
+      </c>
+      <c r="DU65" t="inlineStr">
+        <is>
+          <t>Sérgio Nicolas Vieira</t>
+        </is>
+      </c>
+      <c r="DV65" t="inlineStr">
+        <is>
+          <t>Rua A</t>
+        </is>
+      </c>
+      <c r="DW65" t="inlineStr">
+        <is>
+          <t>124</t>
+        </is>
+      </c>
+      <c r="DX65" t="inlineStr">
+        <is>
+          <t>fwfwee</t>
+        </is>
+      </c>
+      <c r="DY65" t="inlineStr">
+        <is>
+          <t>43242-523</t>
+        </is>
+      </c>
+      <c r="DZ65" t="inlineStr">
+        <is>
+          <t>Jabotiana</t>
+        </is>
+      </c>
+      <c r="EA65" t="inlineStr">
+        <is>
+          <t>são paulo</t>
+        </is>
+      </c>
+      <c r="EB65" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC65" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED65" t="inlineStr">
+        <is>
+          <t>Mecanica</t>
+        </is>
+      </c>
+      <c r="EE65" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF65" t="inlineStr"/>
+      <c r="EG65" t="inlineStr"/>
+      <c r="EH65" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-06-24 09:20:15}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-06-24 09:19:59}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-06-24 09:19:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-06-24 09:11:53}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;Seguir &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-06-24 09:11:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;Seguir &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI65" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ65" t="inlineStr">
+        <is>
+          <t>05.1 - Confecção Proposta</t>
+        </is>
+      </c>
+      <c r="EK65" t="inlineStr"/>
+      <c r="EL65" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(workflows): add processar_fila full-queue workflow
enviar_assinatura and finalizar_proposta now accept processo_id to read
from dados/<id>_<slug>.json, enabling processing of all queue candidates
rather than just the last one.
</commit_message>
<xml_diff>
--- a/dados_formularios.xlsx
+++ b/dados_formularios.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:EQ93"/>
+  <dimension ref="A1:EQ99"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -43403,47 +43403,33 @@
           <t>https://workflow.folhatech.com.br//triata/Sistema.php</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>147</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>0121000</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>01210000016</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+      <c r="C93" t="n">
+        <v>147</v>
+      </c>
+      <c r="D93" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E93" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F93" t="n">
+        <v>1</v>
       </c>
       <c r="G93" t="inlineStr"/>
       <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="J93" t="inlineStr">
-        <is>
-          <t>22820</t>
-        </is>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>22820</v>
       </c>
       <c r="K93" t="inlineStr">
         <is>
           <t>C</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="L93" t="n">
+        <v>408</v>
       </c>
       <c r="M93" t="inlineStr">
         <is>
@@ -43455,25 +43441,19 @@
           <t>robo.relatorio@folhatech.com.br</t>
         </is>
       </c>
-      <c r="O93" t="inlineStr">
-        <is>
-          <t>408</t>
-        </is>
+      <c r="O93" t="n">
+        <v>408</v>
       </c>
       <c r="P93" t="inlineStr">
         <is>
           <t>Robo Cadastro Cliente</t>
         </is>
       </c>
-      <c r="Q93" t="inlineStr">
-        <is>
-          <t>1782961200</t>
-        </is>
-      </c>
-      <c r="R93" t="inlineStr">
-        <is>
-          <t>1783021839</t>
-        </is>
+      <c r="Q93" t="n">
+        <v>1782961200</v>
+      </c>
+      <c r="R93" t="n">
+        <v>1783021839</v>
       </c>
       <c r="S93" t="inlineStr">
         <is>
@@ -43495,10 +43475,8 @@
           <t>01/07/2026 09:31</t>
         </is>
       </c>
-      <c r="W93" t="inlineStr">
-        <is>
-          <t>22820</t>
-        </is>
+      <c r="W93" t="n">
+        <v>22820</v>
       </c>
       <c r="X93" t="inlineStr">
         <is>
@@ -43510,35 +43488,27 @@
           <t>02/07/2026 16:18</t>
         </is>
       </c>
-      <c r="Z93" t="inlineStr">
-        <is>
-          <t>131607</t>
-        </is>
+      <c r="Z93" t="n">
+        <v>131607</v>
       </c>
       <c r="AA93" t="inlineStr">
         <is>
           <t>08 - Confecção 30 dias (Contrato)</t>
         </is>
       </c>
-      <c r="AB93" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="AC93" t="inlineStr">
-        <is>
-          <t>427</t>
-        </is>
+      <c r="AB93" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC93" t="n">
+        <v>427</v>
       </c>
       <c r="AD93" t="inlineStr">
         <is>
           <t>tiago izaias</t>
         </is>
       </c>
-      <c r="AE93" t="inlineStr">
-        <is>
-          <t>0121</t>
-        </is>
+      <c r="AE93" t="n">
+        <v>121</v>
       </c>
       <c r="AF93" t="inlineStr">
         <is>
@@ -43555,10 +43525,8 @@
       <c r="AJ93" t="inlineStr"/>
       <c r="AK93" t="inlineStr"/>
       <c r="AL93" t="inlineStr"/>
-      <c r="AM93" t="inlineStr">
-        <is>
-          <t>131607</t>
-        </is>
+      <c r="AM93" t="n">
+        <v>131607</v>
       </c>
       <c r="AN93" t="inlineStr">
         <is>
@@ -43590,10 +43558,8 @@
           <t>Aumento de quadro</t>
         </is>
       </c>
-      <c r="AT93" t="inlineStr">
-        <is>
-          <t>12700.00</t>
-        </is>
+      <c r="AT93" t="n">
+        <v>12700</v>
       </c>
       <c r="AU93" t="inlineStr"/>
       <c r="AV93" t="inlineStr">
@@ -43721,10 +43687,8 @@
           <t>Pai</t>
         </is>
       </c>
-      <c r="DE93" t="inlineStr">
-        <is>
-          <t>312423424</t>
-        </is>
+      <c r="DE93" t="n">
+        <v>312423424</v>
       </c>
       <c r="DF93" t="inlineStr"/>
       <c r="DG93" t="inlineStr">
@@ -43737,15 +43701,11 @@
           <t>- Selecione algo -</t>
         </is>
       </c>
-      <c r="DI93" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="DJ93" t="inlineStr">
-        <is>
-          <t>174280130</t>
-        </is>
+      <c r="DI93" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ93" t="n">
+        <v>174280130</v>
       </c>
       <c r="DK93" t="inlineStr">
         <is>
@@ -43757,10 +43717,8 @@
           <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
         </is>
       </c>
-      <c r="DM93" t="inlineStr">
-        <is>
-          <t>1234242354</t>
-        </is>
+      <c r="DM93" t="n">
+        <v>1234242354</v>
       </c>
       <c r="DN93" t="inlineStr">
         <is>
@@ -43782,15 +43740,11 @@
           <t>Conta Corrente</t>
         </is>
       </c>
-      <c r="DR93" t="inlineStr">
-        <is>
-          <t>12121</t>
-        </is>
-      </c>
-      <c r="DS93" t="inlineStr">
-        <is>
-          <t>3144</t>
-        </is>
+      <c r="DR93" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS93" t="n">
+        <v>3144</v>
       </c>
       <c r="DT93" t="inlineStr">
         <is>
@@ -43807,10 +43761,8 @@
           <t>Alameda dos Pescadores 202 Loja 28</t>
         </is>
       </c>
-      <c r="DW93" t="inlineStr">
-        <is>
-          <t>762</t>
-        </is>
+      <c r="DW93" t="n">
+        <v>762</v>
       </c>
       <c r="DX93" t="inlineStr"/>
       <c r="DY93" t="inlineStr">
@@ -43888,6 +43840,2772 @@
         </is>
       </c>
       <c r="EQ93" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>03/07/2026, 15:24:44</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C94" t="n">
+        <v>147</v>
+      </c>
+      <c r="D94" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E94" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F94" t="n">
+        <v>1</v>
+      </c>
+      <c r="G94" t="inlineStr"/>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="n">
+        <v>0</v>
+      </c>
+      <c r="J94" t="n">
+        <v>22820</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L94" t="n">
+        <v>408</v>
+      </c>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O94" t="n">
+        <v>408</v>
+      </c>
+      <c r="P94" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q94" t="n">
+        <v>1783047600</v>
+      </c>
+      <c r="R94" t="n">
+        <v>1783102953</v>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>15:22</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>03/07/2026 15:22</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W94" t="n">
+        <v>22820</v>
+      </c>
+      <c r="X94" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y94" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z94" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AA94" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB94" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC94" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD94" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE94" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF94" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG94" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH94" t="inlineStr"/>
+      <c r="AI94" t="inlineStr"/>
+      <c r="AJ94" t="inlineStr"/>
+      <c r="AK94" t="inlineStr"/>
+      <c r="AL94" t="inlineStr"/>
+      <c r="AM94" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AN94" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO94" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP94" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ94" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR94" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS94" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT94" t="n">
+        <v>12700</v>
+      </c>
+      <c r="AU94" t="inlineStr"/>
+      <c r="AV94" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW94" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX94" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY94" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ94" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA94" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB94" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC94" t="inlineStr"/>
+      <c r="BD94" t="inlineStr"/>
+      <c r="BE94" t="inlineStr"/>
+      <c r="BF94" t="inlineStr"/>
+      <c r="BG94" t="inlineStr"/>
+      <c r="BH94" t="inlineStr"/>
+      <c r="BI94" t="inlineStr"/>
+      <c r="BJ94" t="inlineStr"/>
+      <c r="BK94" t="inlineStr"/>
+      <c r="BL94" t="inlineStr"/>
+      <c r="BM94" t="inlineStr"/>
+      <c r="BN94" t="inlineStr"/>
+      <c r="BO94" t="inlineStr"/>
+      <c r="BP94" t="inlineStr"/>
+      <c r="BQ94" t="inlineStr"/>
+      <c r="BR94" t="inlineStr"/>
+      <c r="BS94" t="inlineStr"/>
+      <c r="BT94" t="inlineStr"/>
+      <c r="BU94" t="inlineStr"/>
+      <c r="BV94" t="inlineStr"/>
+      <c r="BW94" t="inlineStr"/>
+      <c r="BX94" t="inlineStr"/>
+      <c r="BY94" t="inlineStr"/>
+      <c r="BZ94" t="inlineStr"/>
+      <c r="CA94" t="inlineStr"/>
+      <c r="CB94" t="inlineStr"/>
+      <c r="CC94" t="inlineStr"/>
+      <c r="CD94" t="inlineStr"/>
+      <c r="CE94" t="inlineStr"/>
+      <c r="CF94" t="inlineStr"/>
+      <c r="CG94" t="inlineStr"/>
+      <c r="CH94" t="inlineStr"/>
+      <c r="CI94" t="inlineStr"/>
+      <c r="CJ94" t="inlineStr"/>
+      <c r="CK94" t="inlineStr"/>
+      <c r="CL94" t="inlineStr"/>
+      <c r="CM94" t="inlineStr"/>
+      <c r="CN94" t="inlineStr"/>
+      <c r="CO94" t="inlineStr"/>
+      <c r="CP94" t="inlineStr"/>
+      <c r="CQ94" t="inlineStr"/>
+      <c r="CR94" t="inlineStr"/>
+      <c r="CS94" t="inlineStr"/>
+      <c r="CT94" t="inlineStr"/>
+      <c r="CU94" t="inlineStr"/>
+      <c r="CV94" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW94" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX94" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY94" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ94" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA94" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB94" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC94" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD94" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE94" t="n">
+        <v>312423424</v>
+      </c>
+      <c r="DF94" t="inlineStr"/>
+      <c r="DG94" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH94" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI94" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ94" t="n">
+        <v>174280130</v>
+      </c>
+      <c r="DK94" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL94" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM94" t="n">
+        <v>1234242354</v>
+      </c>
+      <c r="DN94" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO94" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP94" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ94" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR94" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS94" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT94" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU94" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV94" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW94" t="n">
+        <v>762</v>
+      </c>
+      <c r="DX94" t="inlineStr"/>
+      <c r="DY94" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ94" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA94" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB94" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC94" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED94" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE94" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF94" t="inlineStr"/>
+      <c r="EG94" t="inlineStr"/>
+      <c r="EH94" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI94" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ94" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK94" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL94" t="inlineStr"/>
+      <c r="EM94" t="inlineStr"/>
+      <c r="EN94" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO94" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP94" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ94" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>03/07/2026, 15:56:16</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C95" t="n">
+        <v>147</v>
+      </c>
+      <c r="D95" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E95" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F95" t="n">
+        <v>1</v>
+      </c>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="n">
+        <v>0</v>
+      </c>
+      <c r="J95" t="n">
+        <v>22820</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L95" t="n">
+        <v>408</v>
+      </c>
+      <c r="M95" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O95" t="n">
+        <v>408</v>
+      </c>
+      <c r="P95" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q95" t="n">
+        <v>1783047600</v>
+      </c>
+      <c r="R95" t="n">
+        <v>1783104845</v>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>15:54</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>03/07/2026 15:54</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W95" t="n">
+        <v>22820</v>
+      </c>
+      <c r="X95" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y95" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z95" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AA95" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB95" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC95" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD95" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE95" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF95" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG95" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH95" t="inlineStr"/>
+      <c r="AI95" t="inlineStr"/>
+      <c r="AJ95" t="inlineStr"/>
+      <c r="AK95" t="inlineStr"/>
+      <c r="AL95" t="inlineStr"/>
+      <c r="AM95" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AN95" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO95" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP95" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ95" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR95" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS95" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT95" t="n">
+        <v>12700</v>
+      </c>
+      <c r="AU95" t="inlineStr"/>
+      <c r="AV95" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW95" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX95" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY95" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ95" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA95" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB95" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC95" t="inlineStr"/>
+      <c r="BD95" t="inlineStr"/>
+      <c r="BE95" t="inlineStr"/>
+      <c r="BF95" t="inlineStr"/>
+      <c r="BG95" t="inlineStr"/>
+      <c r="BH95" t="inlineStr"/>
+      <c r="BI95" t="inlineStr"/>
+      <c r="BJ95" t="inlineStr"/>
+      <c r="BK95" t="inlineStr"/>
+      <c r="BL95" t="inlineStr"/>
+      <c r="BM95" t="inlineStr"/>
+      <c r="BN95" t="inlineStr"/>
+      <c r="BO95" t="inlineStr"/>
+      <c r="BP95" t="inlineStr"/>
+      <c r="BQ95" t="inlineStr"/>
+      <c r="BR95" t="inlineStr"/>
+      <c r="BS95" t="inlineStr"/>
+      <c r="BT95" t="inlineStr"/>
+      <c r="BU95" t="inlineStr"/>
+      <c r="BV95" t="inlineStr"/>
+      <c r="BW95" t="inlineStr"/>
+      <c r="BX95" t="inlineStr"/>
+      <c r="BY95" t="inlineStr"/>
+      <c r="BZ95" t="inlineStr"/>
+      <c r="CA95" t="inlineStr"/>
+      <c r="CB95" t="inlineStr"/>
+      <c r="CC95" t="inlineStr"/>
+      <c r="CD95" t="inlineStr"/>
+      <c r="CE95" t="inlineStr"/>
+      <c r="CF95" t="inlineStr"/>
+      <c r="CG95" t="inlineStr"/>
+      <c r="CH95" t="inlineStr"/>
+      <c r="CI95" t="inlineStr"/>
+      <c r="CJ95" t="inlineStr"/>
+      <c r="CK95" t="inlineStr"/>
+      <c r="CL95" t="inlineStr"/>
+      <c r="CM95" t="inlineStr"/>
+      <c r="CN95" t="inlineStr"/>
+      <c r="CO95" t="inlineStr"/>
+      <c r="CP95" t="inlineStr"/>
+      <c r="CQ95" t="inlineStr"/>
+      <c r="CR95" t="inlineStr"/>
+      <c r="CS95" t="inlineStr"/>
+      <c r="CT95" t="inlineStr"/>
+      <c r="CU95" t="inlineStr"/>
+      <c r="CV95" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW95" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX95" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY95" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ95" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA95" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB95" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC95" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD95" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE95" t="n">
+        <v>312423424</v>
+      </c>
+      <c r="DF95" t="inlineStr"/>
+      <c r="DG95" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH95" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI95" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ95" t="n">
+        <v>174280130</v>
+      </c>
+      <c r="DK95" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL95" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM95" t="n">
+        <v>1234242354</v>
+      </c>
+      <c r="DN95" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO95" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP95" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ95" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR95" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS95" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT95" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU95" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV95" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW95" t="n">
+        <v>762</v>
+      </c>
+      <c r="DX95" t="inlineStr"/>
+      <c r="DY95" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ95" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA95" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB95" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC95" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED95" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE95" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF95" t="inlineStr"/>
+      <c r="EG95" t="inlineStr"/>
+      <c r="EH95" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI95" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ95" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK95" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL95" t="inlineStr"/>
+      <c r="EM95" t="inlineStr"/>
+      <c r="EN95" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO95" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP95" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ95" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>03/07/2026, 16:10:33</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C96" t="n">
+        <v>147</v>
+      </c>
+      <c r="D96" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E96" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F96" t="n">
+        <v>1</v>
+      </c>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="n">
+        <v>0</v>
+      </c>
+      <c r="J96" t="n">
+        <v>22820</v>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L96" t="n">
+        <v>408</v>
+      </c>
+      <c r="M96" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O96" t="n">
+        <v>408</v>
+      </c>
+      <c r="P96" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q96" t="n">
+        <v>1783047600</v>
+      </c>
+      <c r="R96" t="n">
+        <v>1783105702</v>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>16:08</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>03/07/2026 16:08</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W96" t="n">
+        <v>22820</v>
+      </c>
+      <c r="X96" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y96" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z96" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AA96" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB96" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC96" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD96" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE96" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF96" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG96" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH96" t="inlineStr"/>
+      <c r="AI96" t="inlineStr"/>
+      <c r="AJ96" t="inlineStr"/>
+      <c r="AK96" t="inlineStr"/>
+      <c r="AL96" t="inlineStr"/>
+      <c r="AM96" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AN96" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO96" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP96" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ96" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR96" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS96" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT96" t="n">
+        <v>12700</v>
+      </c>
+      <c r="AU96" t="inlineStr"/>
+      <c r="AV96" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW96" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX96" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY96" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ96" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA96" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB96" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC96" t="inlineStr"/>
+      <c r="BD96" t="inlineStr"/>
+      <c r="BE96" t="inlineStr"/>
+      <c r="BF96" t="inlineStr"/>
+      <c r="BG96" t="inlineStr"/>
+      <c r="BH96" t="inlineStr"/>
+      <c r="BI96" t="inlineStr"/>
+      <c r="BJ96" t="inlineStr"/>
+      <c r="BK96" t="inlineStr"/>
+      <c r="BL96" t="inlineStr"/>
+      <c r="BM96" t="inlineStr"/>
+      <c r="BN96" t="inlineStr"/>
+      <c r="BO96" t="inlineStr"/>
+      <c r="BP96" t="inlineStr"/>
+      <c r="BQ96" t="inlineStr"/>
+      <c r="BR96" t="inlineStr"/>
+      <c r="BS96" t="inlineStr"/>
+      <c r="BT96" t="inlineStr"/>
+      <c r="BU96" t="inlineStr"/>
+      <c r="BV96" t="inlineStr"/>
+      <c r="BW96" t="inlineStr"/>
+      <c r="BX96" t="inlineStr"/>
+      <c r="BY96" t="inlineStr"/>
+      <c r="BZ96" t="inlineStr"/>
+      <c r="CA96" t="inlineStr"/>
+      <c r="CB96" t="inlineStr"/>
+      <c r="CC96" t="inlineStr"/>
+      <c r="CD96" t="inlineStr"/>
+      <c r="CE96" t="inlineStr"/>
+      <c r="CF96" t="inlineStr"/>
+      <c r="CG96" t="inlineStr"/>
+      <c r="CH96" t="inlineStr"/>
+      <c r="CI96" t="inlineStr"/>
+      <c r="CJ96" t="inlineStr"/>
+      <c r="CK96" t="inlineStr"/>
+      <c r="CL96" t="inlineStr"/>
+      <c r="CM96" t="inlineStr"/>
+      <c r="CN96" t="inlineStr"/>
+      <c r="CO96" t="inlineStr"/>
+      <c r="CP96" t="inlineStr"/>
+      <c r="CQ96" t="inlineStr"/>
+      <c r="CR96" t="inlineStr"/>
+      <c r="CS96" t="inlineStr"/>
+      <c r="CT96" t="inlineStr"/>
+      <c r="CU96" t="inlineStr"/>
+      <c r="CV96" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW96" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX96" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY96" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ96" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA96" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB96" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC96" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD96" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE96" t="n">
+        <v>312423424</v>
+      </c>
+      <c r="DF96" t="inlineStr"/>
+      <c r="DG96" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH96" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI96" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ96" t="n">
+        <v>174280130</v>
+      </c>
+      <c r="DK96" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL96" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM96" t="n">
+        <v>1234242354</v>
+      </c>
+      <c r="DN96" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO96" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP96" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ96" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR96" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS96" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT96" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU96" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV96" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW96" t="n">
+        <v>762</v>
+      </c>
+      <c r="DX96" t="inlineStr"/>
+      <c r="DY96" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ96" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA96" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB96" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC96" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED96" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE96" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF96" t="inlineStr"/>
+      <c r="EG96" t="inlineStr"/>
+      <c r="EH96" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI96" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ96" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK96" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL96" t="inlineStr"/>
+      <c r="EM96" t="inlineStr"/>
+      <c r="EN96" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO96" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP96" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ96" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>03/07/2026, 16:14:35</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C97" t="n">
+        <v>147</v>
+      </c>
+      <c r="D97" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E97" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F97" t="n">
+        <v>1</v>
+      </c>
+      <c r="G97" t="inlineStr"/>
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="n">
+        <v>0</v>
+      </c>
+      <c r="J97" t="n">
+        <v>22820</v>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L97" t="n">
+        <v>408</v>
+      </c>
+      <c r="M97" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O97" t="n">
+        <v>408</v>
+      </c>
+      <c r="P97" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q97" t="n">
+        <v>1783047600</v>
+      </c>
+      <c r="R97" t="n">
+        <v>1783105943</v>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>16:12</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>03/07/2026 16:12</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W97" t="n">
+        <v>22820</v>
+      </c>
+      <c r="X97" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y97" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z97" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AA97" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB97" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC97" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD97" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE97" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF97" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG97" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH97" t="inlineStr"/>
+      <c r="AI97" t="inlineStr"/>
+      <c r="AJ97" t="inlineStr"/>
+      <c r="AK97" t="inlineStr"/>
+      <c r="AL97" t="inlineStr"/>
+      <c r="AM97" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AN97" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO97" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP97" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ97" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR97" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS97" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT97" t="n">
+        <v>12700</v>
+      </c>
+      <c r="AU97" t="inlineStr"/>
+      <c r="AV97" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW97" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX97" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY97" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ97" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA97" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB97" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC97" t="inlineStr"/>
+      <c r="BD97" t="inlineStr"/>
+      <c r="BE97" t="inlineStr"/>
+      <c r="BF97" t="inlineStr"/>
+      <c r="BG97" t="inlineStr"/>
+      <c r="BH97" t="inlineStr"/>
+      <c r="BI97" t="inlineStr"/>
+      <c r="BJ97" t="inlineStr"/>
+      <c r="BK97" t="inlineStr"/>
+      <c r="BL97" t="inlineStr"/>
+      <c r="BM97" t="inlineStr"/>
+      <c r="BN97" t="inlineStr"/>
+      <c r="BO97" t="inlineStr"/>
+      <c r="BP97" t="inlineStr"/>
+      <c r="BQ97" t="inlineStr"/>
+      <c r="BR97" t="inlineStr"/>
+      <c r="BS97" t="inlineStr"/>
+      <c r="BT97" t="inlineStr"/>
+      <c r="BU97" t="inlineStr"/>
+      <c r="BV97" t="inlineStr"/>
+      <c r="BW97" t="inlineStr"/>
+      <c r="BX97" t="inlineStr"/>
+      <c r="BY97" t="inlineStr"/>
+      <c r="BZ97" t="inlineStr"/>
+      <c r="CA97" t="inlineStr"/>
+      <c r="CB97" t="inlineStr"/>
+      <c r="CC97" t="inlineStr"/>
+      <c r="CD97" t="inlineStr"/>
+      <c r="CE97" t="inlineStr"/>
+      <c r="CF97" t="inlineStr"/>
+      <c r="CG97" t="inlineStr"/>
+      <c r="CH97" t="inlineStr"/>
+      <c r="CI97" t="inlineStr"/>
+      <c r="CJ97" t="inlineStr"/>
+      <c r="CK97" t="inlineStr"/>
+      <c r="CL97" t="inlineStr"/>
+      <c r="CM97" t="inlineStr"/>
+      <c r="CN97" t="inlineStr"/>
+      <c r="CO97" t="inlineStr"/>
+      <c r="CP97" t="inlineStr"/>
+      <c r="CQ97" t="inlineStr"/>
+      <c r="CR97" t="inlineStr"/>
+      <c r="CS97" t="inlineStr"/>
+      <c r="CT97" t="inlineStr"/>
+      <c r="CU97" t="inlineStr"/>
+      <c r="CV97" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW97" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX97" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY97" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ97" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA97" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB97" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC97" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD97" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE97" t="n">
+        <v>312423424</v>
+      </c>
+      <c r="DF97" t="inlineStr"/>
+      <c r="DG97" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH97" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI97" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ97" t="n">
+        <v>174280130</v>
+      </c>
+      <c r="DK97" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL97" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM97" t="n">
+        <v>1234242354</v>
+      </c>
+      <c r="DN97" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO97" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP97" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ97" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR97" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS97" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT97" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU97" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV97" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW97" t="n">
+        <v>762</v>
+      </c>
+      <c r="DX97" t="inlineStr"/>
+      <c r="DY97" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ97" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA97" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB97" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC97" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED97" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE97" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF97" t="inlineStr"/>
+      <c r="EG97" t="inlineStr"/>
+      <c r="EH97" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI97" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ97" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK97" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL97" t="inlineStr"/>
+      <c r="EM97" t="inlineStr"/>
+      <c r="EN97" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO97" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP97" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ97" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>03/07/2026, 16:44:16</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C98" t="n">
+        <v>147</v>
+      </c>
+      <c r="D98" t="n">
+        <v>121000</v>
+      </c>
+      <c r="E98" t="n">
+        <v>1210000016</v>
+      </c>
+      <c r="F98" t="n">
+        <v>1</v>
+      </c>
+      <c r="G98" t="inlineStr"/>
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="n">
+        <v>0</v>
+      </c>
+      <c r="J98" t="n">
+        <v>22820</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L98" t="n">
+        <v>408</v>
+      </c>
+      <c r="M98" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O98" t="n">
+        <v>408</v>
+      </c>
+      <c r="P98" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q98" t="n">
+        <v>1783047600</v>
+      </c>
+      <c r="R98" t="n">
+        <v>1783107724</v>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>16:42</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>03/07/2026 16:42</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W98" t="n">
+        <v>22820</v>
+      </c>
+      <c r="X98" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y98" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z98" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AA98" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB98" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC98" t="n">
+        <v>427</v>
+      </c>
+      <c r="AD98" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE98" t="n">
+        <v>121</v>
+      </c>
+      <c r="AF98" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG98" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH98" t="inlineStr"/>
+      <c r="AI98" t="inlineStr"/>
+      <c r="AJ98" t="inlineStr"/>
+      <c r="AK98" t="inlineStr"/>
+      <c r="AL98" t="inlineStr"/>
+      <c r="AM98" t="n">
+        <v>131607</v>
+      </c>
+      <c r="AN98" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO98" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP98" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ98" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR98" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS98" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT98" t="n">
+        <v>12700</v>
+      </c>
+      <c r="AU98" t="inlineStr"/>
+      <c r="AV98" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW98" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX98" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY98" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ98" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA98" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB98" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC98" t="inlineStr"/>
+      <c r="BD98" t="inlineStr"/>
+      <c r="BE98" t="inlineStr"/>
+      <c r="BF98" t="inlineStr"/>
+      <c r="BG98" t="inlineStr"/>
+      <c r="BH98" t="inlineStr"/>
+      <c r="BI98" t="inlineStr"/>
+      <c r="BJ98" t="inlineStr"/>
+      <c r="BK98" t="inlineStr"/>
+      <c r="BL98" t="inlineStr"/>
+      <c r="BM98" t="inlineStr"/>
+      <c r="BN98" t="inlineStr"/>
+      <c r="BO98" t="inlineStr"/>
+      <c r="BP98" t="inlineStr"/>
+      <c r="BQ98" t="inlineStr"/>
+      <c r="BR98" t="inlineStr"/>
+      <c r="BS98" t="inlineStr"/>
+      <c r="BT98" t="inlineStr"/>
+      <c r="BU98" t="inlineStr"/>
+      <c r="BV98" t="inlineStr"/>
+      <c r="BW98" t="inlineStr"/>
+      <c r="BX98" t="inlineStr"/>
+      <c r="BY98" t="inlineStr"/>
+      <c r="BZ98" t="inlineStr"/>
+      <c r="CA98" t="inlineStr"/>
+      <c r="CB98" t="inlineStr"/>
+      <c r="CC98" t="inlineStr"/>
+      <c r="CD98" t="inlineStr"/>
+      <c r="CE98" t="inlineStr"/>
+      <c r="CF98" t="inlineStr"/>
+      <c r="CG98" t="inlineStr"/>
+      <c r="CH98" t="inlineStr"/>
+      <c r="CI98" t="inlineStr"/>
+      <c r="CJ98" t="inlineStr"/>
+      <c r="CK98" t="inlineStr"/>
+      <c r="CL98" t="inlineStr"/>
+      <c r="CM98" t="inlineStr"/>
+      <c r="CN98" t="inlineStr"/>
+      <c r="CO98" t="inlineStr"/>
+      <c r="CP98" t="inlineStr"/>
+      <c r="CQ98" t="inlineStr"/>
+      <c r="CR98" t="inlineStr"/>
+      <c r="CS98" t="inlineStr"/>
+      <c r="CT98" t="inlineStr"/>
+      <c r="CU98" t="inlineStr"/>
+      <c r="CV98" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW98" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX98" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY98" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ98" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA98" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB98" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC98" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD98" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE98" t="n">
+        <v>312423424</v>
+      </c>
+      <c r="DF98" t="inlineStr"/>
+      <c r="DG98" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH98" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI98" t="n">
+        <v>0</v>
+      </c>
+      <c r="DJ98" t="n">
+        <v>174280130</v>
+      </c>
+      <c r="DK98" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL98" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM98" t="n">
+        <v>1234242354</v>
+      </c>
+      <c r="DN98" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO98" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP98" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ98" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR98" t="n">
+        <v>12121</v>
+      </c>
+      <c r="DS98" t="n">
+        <v>3144</v>
+      </c>
+      <c r="DT98" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU98" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV98" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW98" t="n">
+        <v>762</v>
+      </c>
+      <c r="DX98" t="inlineStr"/>
+      <c r="DY98" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ98" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA98" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB98" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC98" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED98" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE98" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF98" t="inlineStr"/>
+      <c r="EG98" t="inlineStr"/>
+      <c r="EH98" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI98" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ98" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK98" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL98" t="inlineStr"/>
+      <c r="EM98" t="inlineStr"/>
+      <c r="EN98" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO98" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP98" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ98" t="inlineStr">
+        <is>
+          <t>R$ 12.700,00</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>03/07/2026, 17:06:56</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/triata/Sistema.php</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>147</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>0121000</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>01210000016</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr"/>
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>22820</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="M99" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>robo.relatorio@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="O99" t="inlineStr">
+        <is>
+          <t>408</t>
+        </is>
+      </c>
+      <c r="P99" t="inlineStr">
+        <is>
+          <t>Robo Cadastro Cliente</t>
+        </is>
+      </c>
+      <c r="Q99" t="inlineStr">
+        <is>
+          <t>1783047600</t>
+        </is>
+      </c>
+      <c r="R99" t="inlineStr">
+        <is>
+          <t>1783109084</t>
+        </is>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>17:04</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>03/07/2026 17:04</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>01/07/2026 09:31</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>22820</t>
+        </is>
+      </c>
+      <c r="X99" t="inlineStr">
+        <is>
+          <t>01/07/2026 16:17</t>
+        </is>
+      </c>
+      <c r="Y99" t="inlineStr">
+        <is>
+          <t>02/07/2026 16:18</t>
+        </is>
+      </c>
+      <c r="Z99" t="inlineStr">
+        <is>
+          <t>131607</t>
+        </is>
+      </c>
+      <c r="AA99" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="AB99" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="AC99" t="inlineStr">
+        <is>
+          <t>427</t>
+        </is>
+      </c>
+      <c r="AD99" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AE99" t="inlineStr">
+        <is>
+          <t>0121</t>
+        </is>
+      </c>
+      <c r="AF99" t="inlineStr">
+        <is>
+          <t>Arantes - Contratação PJ</t>
+        </is>
+      </c>
+      <c r="AG99" t="inlineStr">
+        <is>
+          <t>https://workflow.folhatech.com.br/</t>
+        </is>
+      </c>
+      <c r="AH99" t="inlineStr"/>
+      <c r="AI99" t="inlineStr"/>
+      <c r="AJ99" t="inlineStr"/>
+      <c r="AK99" t="inlineStr"/>
+      <c r="AL99" t="inlineStr"/>
+      <c r="AM99" t="inlineStr">
+        <is>
+          <t>131607</t>
+        </is>
+      </c>
+      <c r="AN99" t="inlineStr">
+        <is>
+          <t>tiago izaias</t>
+        </is>
+      </c>
+      <c r="AO99" t="inlineStr">
+        <is>
+          <t>tiago.izaias@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="AP99" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AQ99" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AR99" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AS99" t="inlineStr">
+        <is>
+          <t>Aumento de quadro</t>
+        </is>
+      </c>
+      <c r="AT99" t="inlineStr">
+        <is>
+          <t>12700.00</t>
+        </is>
+      </c>
+      <c r="AU99" t="inlineStr"/>
+      <c r="AV99" t="inlineStr">
+        <is>
+          <t>TI</t>
+        </is>
+      </c>
+      <c r="AW99" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AX99" t="inlineStr">
+        <is>
+          <t>Folha Tech</t>
+        </is>
+      </c>
+      <c r="AY99" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="AZ99" t="inlineStr">
+        <is>
+          <t>Fernando Andrade (Folha Tech)</t>
+        </is>
+      </c>
+      <c r="BA99" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BB99" t="inlineStr">
+        <is>
+          <t>fernando.andrade@folhatech.com.br</t>
+        </is>
+      </c>
+      <c r="BC99" t="inlineStr"/>
+      <c r="BD99" t="inlineStr"/>
+      <c r="BE99" t="inlineStr"/>
+      <c r="BF99" t="inlineStr"/>
+      <c r="BG99" t="inlineStr"/>
+      <c r="BH99" t="inlineStr"/>
+      <c r="BI99" t="inlineStr"/>
+      <c r="BJ99" t="inlineStr"/>
+      <c r="BK99" t="inlineStr"/>
+      <c r="BL99" t="inlineStr"/>
+      <c r="BM99" t="inlineStr"/>
+      <c r="BN99" t="inlineStr"/>
+      <c r="BO99" t="inlineStr"/>
+      <c r="BP99" t="inlineStr"/>
+      <c r="BQ99" t="inlineStr"/>
+      <c r="BR99" t="inlineStr"/>
+      <c r="BS99" t="inlineStr"/>
+      <c r="BT99" t="inlineStr"/>
+      <c r="BU99" t="inlineStr"/>
+      <c r="BV99" t="inlineStr"/>
+      <c r="BW99" t="inlineStr"/>
+      <c r="BX99" t="inlineStr"/>
+      <c r="BY99" t="inlineStr"/>
+      <c r="BZ99" t="inlineStr"/>
+      <c r="CA99" t="inlineStr"/>
+      <c r="CB99" t="inlineStr"/>
+      <c r="CC99" t="inlineStr"/>
+      <c r="CD99" t="inlineStr"/>
+      <c r="CE99" t="inlineStr"/>
+      <c r="CF99" t="inlineStr"/>
+      <c r="CG99" t="inlineStr"/>
+      <c r="CH99" t="inlineStr"/>
+      <c r="CI99" t="inlineStr"/>
+      <c r="CJ99" t="inlineStr"/>
+      <c r="CK99" t="inlineStr"/>
+      <c r="CL99" t="inlineStr"/>
+      <c r="CM99" t="inlineStr"/>
+      <c r="CN99" t="inlineStr"/>
+      <c r="CO99" t="inlineStr"/>
+      <c r="CP99" t="inlineStr"/>
+      <c r="CQ99" t="inlineStr"/>
+      <c r="CR99" t="inlineStr"/>
+      <c r="CS99" t="inlineStr"/>
+      <c r="CT99" t="inlineStr"/>
+      <c r="CU99" t="inlineStr"/>
+      <c r="CV99" t="inlineStr">
+        <is>
+          <t>Mirella Daiane Stella Lima</t>
+        </is>
+      </c>
+      <c r="CW99" t="inlineStr">
+        <is>
+          <t>24/06/2004</t>
+        </is>
+      </c>
+      <c r="CX99" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CY99" t="inlineStr">
+        <is>
+          <t>Solteiro</t>
+        </is>
+      </c>
+      <c r="CZ99" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DA99" t="inlineStr">
+        <is>
+          <t>Betina Sara Carla</t>
+        </is>
+      </c>
+      <c r="DB99" t="inlineStr">
+        <is>
+          <t>Fernando Osvaldo Raul Lima</t>
+        </is>
+      </c>
+      <c r="DC99" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DD99" t="inlineStr">
+        <is>
+          <t>Pai</t>
+        </is>
+      </c>
+      <c r="DE99" t="inlineStr">
+        <is>
+          <t>312423424</t>
+        </is>
+      </c>
+      <c r="DF99" t="inlineStr"/>
+      <c r="DG99" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DH99" t="inlineStr">
+        <is>
+          <t>- Selecione algo -</t>
+        </is>
+      </c>
+      <c r="DI99" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DJ99" t="inlineStr">
+        <is>
+          <t>174280130</t>
+        </is>
+      </c>
+      <c r="DK99" t="inlineStr">
+        <is>
+          <t>579.445.157-26</t>
+        </is>
+      </c>
+      <c r="DL99" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.br</t>
+        </is>
+      </c>
+      <c r="DM99" t="inlineStr">
+        <is>
+          <t>1234242354</t>
+        </is>
+      </c>
+      <c r="DN99" t="inlineStr">
+        <is>
+          <t>98.923.964/0001-06</t>
+        </is>
+      </c>
+      <c r="DO99" t="inlineStr">
+        <is>
+          <t>Nubank</t>
+        </is>
+      </c>
+      <c r="DP99" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DQ99" t="inlineStr">
+        <is>
+          <t>Conta Corrente</t>
+        </is>
+      </c>
+      <c r="DR99" t="inlineStr">
+        <is>
+          <t>12121</t>
+        </is>
+      </c>
+      <c r="DS99" t="inlineStr">
+        <is>
+          <t>3144</t>
+        </is>
+      </c>
+      <c r="DT99" t="inlineStr">
+        <is>
+          <t>mirella_daiane_lima@a-qualitybrasil.com.</t>
+        </is>
+      </c>
+      <c r="DU99" t="inlineStr">
+        <is>
+          <t>tetwetete</t>
+        </is>
+      </c>
+      <c r="DV99" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28</t>
+        </is>
+      </c>
+      <c r="DW99" t="inlineStr">
+        <is>
+          <t>762</t>
+        </is>
+      </c>
+      <c r="DX99" t="inlineStr"/>
+      <c r="DY99" t="inlineStr">
+        <is>
+          <t>42880-971</t>
+        </is>
+      </c>
+      <c r="DZ99" t="inlineStr">
+        <is>
+          <t>Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EA99" t="inlineStr">
+        <is>
+          <t>Mata de São João</t>
+        </is>
+      </c>
+      <c r="EB99" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="EC99" t="inlineStr">
+        <is>
+          <t>Ensino superior completo</t>
+        </is>
+      </c>
+      <c r="ED99" t="inlineStr">
+        <is>
+          <t>adm</t>
+        </is>
+      </c>
+      <c r="EE99" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="EF99" t="inlineStr"/>
+      <c r="EG99" t="inlineStr"/>
+      <c r="EH99" t="inlineStr">
+        <is>
+          <t>_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 07 - Sistema / Equipamento TI&lt;br&gt;Pedro Santana - {{2026-07-01 16:17:12}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 06 - Proposta&lt;br&gt;Adrielly Santana - {{2026-07-01 16:16:28}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;segue &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 05.1 - Confecção Proposta&lt;br&gt;Robo Cadastro Cliente - {{2026-07-01 11:44:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;concluido pelo robo &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 05 - Validação jurídico&lt;br&gt;Leonardo Toledo - {{2026-07-01 09:36:50}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;ok &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 04 - Aprovação gestor&lt;br&gt;tiago izaias - {{2026-07-01 09:36:34}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 03 - Recrutamento&lt;br&gt;Luana Lidia - {{2026-07-01 09:36:14}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_1"&gt;{{TAREFA}}: 02 - Aprovação Financeiro&lt;br&gt;Jefferson Silva - {{2026-07-01 09:32:24}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_1"&gt;aaa &lt;/div&gt;_BR_TRIATA_&lt;div class="hist_autor hist_cor_2"&gt;{{TAREFA}}: 01 - Requisição&lt;br&gt;tiago izaias - {{2026-07-01 09:32:02}}&lt;/div&gt;&lt;div class="hist_texto hist_cor_2"&gt;aaa &lt;/div&gt;</t>
+        </is>
+      </c>
+      <c r="EI99" t="inlineStr">
+        <is>
+          <t>{{TAREFA}}: 08 - Confecção 30 dias (Contrato)&lt;br&gt;</t>
+        </is>
+      </c>
+      <c r="EJ99" t="inlineStr">
+        <is>
+          <t>08 - Confecção 30 dias (Contrato)</t>
+        </is>
+      </c>
+      <c r="EK99" t="inlineStr">
+        <is>
+          <t>Mirella Manicure</t>
+        </is>
+      </c>
+      <c r="EL99" t="inlineStr"/>
+      <c r="EM99" t="inlineStr"/>
+      <c r="EN99" t="inlineStr">
+        <is>
+          <t>03/07/2026</t>
+        </is>
+      </c>
+      <c r="EO99" t="inlineStr">
+        <is>
+          <t>Alameda dos Pescadores 202 Loja 28, 762  - Praia do Forte</t>
+        </is>
+      </c>
+      <c r="EP99" t="inlineStr">
+        <is>
+          <t>Mata de São João/SP</t>
+        </is>
+      </c>
+      <c r="EQ99" t="inlineStr">
         <is>
           <t>R$ 12.700,00</t>
         </is>

</xml_diff>